<commit_message>
Cải thiện giao diện nút
</commit_message>
<xml_diff>
--- a/04-Bieu-Mau/01-FRM-100/FRM-101_Master_Document_Register.xlsx
+++ b/04-Bieu-Mau/01-FRM-100/FRM-101_Master_Document_Register.xlsx
@@ -26,10 +26,750 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="245">
+  <si>
+    <t>  1. CONTROLLED LOOKUP LISTS</t>
+  </si>
+  <si>
+    <t>  1. REFERENCE INFORMATION</t>
+  </si>
+  <si>
+    <t>  2. ACTIVE LOG TABLE</t>
+  </si>
+  <si>
+    <t>  3. PERIODIC REVIEW / CLOSURE</t>
+  </si>
+  <si>
+    <t>  4. PERIODIC REVIEW SIGN-OFF</t>
+  </si>
+  <si>
+    <t>  REFERENCE / SOURCE CONTEXT</t>
+  </si>
+  <si>
+    <t>  SUPPORT TABLE</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>=ROW()-ROW($A$14)+1</t>
+  </si>
+  <si>
+    <t>ABSENT</t>
+  </si>
+  <si>
+    <t>ACCESS</t>
+  </si>
+  <si>
+    <t>ACCESS_ACTION_TYPE</t>
+  </si>
+  <si>
+    <t>ADJUST</t>
+  </si>
+  <si>
+    <t>ADMIN</t>
+  </si>
+  <si>
+    <t>ALL HANDS</t>
+  </si>
+  <si>
+    <t>ANNEX</t>
+  </si>
+  <si>
+    <t>APPROVED</t>
+  </si>
+  <si>
+    <t>APPROVER</t>
+  </si>
+  <si>
+    <t>ATTENDANCE_STATUS</t>
+  </si>
+  <si>
+    <t>AUDIENCE_CLASS</t>
+  </si>
+  <si>
+    <t>AUDIT_FINDING_SEVERITY</t>
+  </si>
+  <si>
+    <t>AUTHORITY_ROLE</t>
+  </si>
+  <si>
+    <t>AUTHORIZATION_STATUS</t>
+  </si>
+  <si>
+    <t>AUTHORIZED</t>
+  </si>
+  <si>
+    <t>Approved</t>
+  </si>
+  <si>
+    <t>Approved by</t>
+  </si>
+  <si>
+    <t>BACKUP_FLAG</t>
+  </si>
+  <si>
+    <t>Boundary / SoR</t>
+  </si>
+  <si>
+    <t>CHANGE</t>
+  </si>
+  <si>
+    <t>CHANGE_PRIORITY</t>
+  </si>
+  <si>
+    <t>CHANGE_TYPE</t>
+  </si>
+  <si>
+    <t>CLOSED</t>
+  </si>
+  <si>
+    <t>COMMERCIAL_REFERENCE</t>
+  </si>
+  <si>
+    <t>COMM_CHANNEL</t>
+  </si>
+  <si>
+    <t>COMPETENCY_LEVEL</t>
+  </si>
+  <si>
+    <t>COMPLIANCE</t>
+  </si>
+  <si>
+    <t>CONDITIONAL</t>
+  </si>
+  <si>
+    <t>CONFIGURATION</t>
+  </si>
+  <si>
+    <t>CONTAINED</t>
+  </si>
+  <si>
+    <t>CONTEXT_CLASS</t>
+  </si>
+  <si>
+    <t>CONTRACT</t>
+  </si>
+  <si>
+    <t>CONTRACT REVIEW</t>
+  </si>
+  <si>
+    <t>CONTRIBUTOR</t>
+  </si>
+  <si>
+    <t>CONTROL_METHOD</t>
+  </si>
+  <si>
+    <t>COST</t>
+  </si>
+  <si>
+    <t>CREATE</t>
+  </si>
+  <si>
+    <t>CRITICAL</t>
+  </si>
+  <si>
+    <t>CSR</t>
+  </si>
+  <si>
+    <t>CUSTOMER</t>
+  </si>
+  <si>
+    <t>DAILY</t>
+  </si>
+  <si>
+    <t>DECISION</t>
+  </si>
+  <si>
+    <t>DELIVERY</t>
+  </si>
+  <si>
+    <t>DEPT</t>
+  </si>
+  <si>
+    <t>DETECTION</t>
+  </si>
+  <si>
+    <t>DIMENSIONAL</t>
+  </si>
+  <si>
+    <t>DOCUMENT</t>
+  </si>
+  <si>
+    <t>DOC_STATUS</t>
+  </si>
+  <si>
+    <t>DOC_TYPE</t>
+  </si>
+  <si>
+    <t>DRAFT</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Department / Owner</t>
+  </si>
+  <si>
+    <t>Deployment Evidence Ref</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Doc Type</t>
+  </si>
+  <si>
+    <t>Document Code</t>
+  </si>
+  <si>
+    <t>Document Code / Title</t>
+  </si>
+  <si>
+    <t>Document Register Period</t>
+  </si>
+  <si>
+    <t>Document Title</t>
+  </si>
+  <si>
+    <t>EACH LOT</t>
+  </si>
+  <si>
+    <t>EFFECTIVE</t>
+  </si>
+  <si>
+    <t>EMAIL</t>
+  </si>
+  <si>
+    <t>ENG</t>
+  </si>
+  <si>
+    <t>ESCALATE</t>
+  </si>
+  <si>
+    <t>ESCALATED</t>
+  </si>
+  <si>
+    <t>ESCALATION</t>
+  </si>
+  <si>
+    <t>EXCUSED</t>
+  </si>
+  <si>
+    <t>EXPIRED</t>
+  </si>
+  <si>
+    <t>Eff. Date</t>
+  </si>
+  <si>
+    <t>Effective Date</t>
+  </si>
+  <si>
+    <t>Evidence ID</t>
+  </si>
+  <si>
+    <t>Evidence Ref</t>
+  </si>
+  <si>
+    <t>Excel Table — rolling document register (freeze / filter required)</t>
+  </si>
+  <si>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t>FINAL</t>
+  </si>
+  <si>
+    <t>FIRST ARTICLE</t>
+  </si>
+  <si>
+    <t>FIRST OFF</t>
+  </si>
+  <si>
+    <t>FIRST PIECE</t>
+  </si>
+  <si>
+    <t>FMEA_RANK</t>
+  </si>
+  <si>
+    <t>FORM</t>
+  </si>
+  <si>
+    <t>FRM-101</t>
+  </si>
+  <si>
+    <t>FUNCTION</t>
+  </si>
+  <si>
+    <t>FUNCTIONAL</t>
+  </si>
+  <si>
+    <t>Form Code</t>
+  </si>
+  <si>
+    <t>GATE</t>
+  </si>
+  <si>
+    <t>HESEM Engineering · ISO 9001 / AS9100 · Semiconductor Equipment Parts</t>
+  </si>
+  <si>
+    <t>HIGH</t>
+  </si>
+  <si>
+    <t>HOLD</t>
+  </si>
+  <si>
+    <t>HOURLY</t>
+  </si>
+  <si>
+    <t>HR</t>
+  </si>
+  <si>
+    <t>IMPACT_LEVEL</t>
+  </si>
+  <si>
+    <t>IMPACT_SCOPE</t>
+  </si>
+  <si>
+    <t>IN PROCESS</t>
+  </si>
+  <si>
+    <t>IN PROGRESS</t>
+  </si>
+  <si>
+    <t>IN-PROCESS</t>
+  </si>
+  <si>
+    <t>INTERNAL</t>
+  </si>
+  <si>
+    <t>IT</t>
+  </si>
+  <si>
+    <t>KPI-COST</t>
+  </si>
+  <si>
+    <t>KPI-DELIVERY</t>
+  </si>
+  <si>
+    <t>KPI-QUALITY</t>
+  </si>
+  <si>
+    <t>KPI-SAFETY</t>
+  </si>
+  <si>
+    <t>KPI-TRAINING</t>
+  </si>
+  <si>
+    <t>KPI_OWNER_SET</t>
+  </si>
+  <si>
+    <t>LATE</t>
+  </si>
+  <si>
+    <t>LESSON_CLASS</t>
+  </si>
+  <si>
+    <t>LOW</t>
+  </si>
+  <si>
+    <t>M365 / shared workbook remains the master list and evidence owner; workbook captures controlled review / log rows only and must not duplicate system-owned master data.</t>
+  </si>
+  <si>
+    <t>MAJOR</t>
+  </si>
+  <si>
+    <t>MANAGEMENT</t>
+  </si>
+  <si>
+    <t>MASTER DOCUMENT REGISTER</t>
+  </si>
+  <si>
+    <t>MASTER DOCUMENT REGISTER — CONTROLLED LOOKUP LISTS</t>
+  </si>
+  <si>
+    <t>MASTER DOCUMENT REGISTER — EVIDENCE REFERENCE REGISTER</t>
+  </si>
+  <si>
+    <t>MASTER DOCUMENT REGISTER — REVIEW QUESTIONS / PERIODIC REVIEW</t>
+  </si>
+  <si>
+    <t>MEDIUM</t>
+  </si>
+  <si>
+    <t>MEETING</t>
+  </si>
+  <si>
+    <t>MGT</t>
+  </si>
+  <si>
+    <t>MINOR</t>
+  </si>
+  <si>
+    <t>MONITORING</t>
+  </si>
+  <si>
+    <t>Migration Status</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>NONE</t>
+  </si>
+  <si>
+    <t>NOT AUTHORIZED</t>
+  </si>
+  <si>
+    <t>NOT TRAINED</t>
+  </si>
+  <si>
+    <t>NOTICE</t>
+  </si>
+  <si>
+    <t>NOTICE: Controlled dropdown source sheet. Do not edit values without formal document control because validations in the workbook depend on these lists.</t>
+  </si>
+  <si>
+    <t>NOTICE: Controlled lookup lists only. Change values only through formal document control because dropdown behavior and validation depend on this sheet.</t>
+  </si>
+  <si>
+    <t>NOTICE: Keep one row per controlled document. Maintain code, revision, status, effective date, storage path and superseded reference so documented information stays traceable and current.</t>
+  </si>
+  <si>
+    <t>NOTICE: Keep review questions and periodic review data aligned to the current controlled criteria set; do not embed unofficial rules in this support sheet.</t>
+  </si>
+  <si>
+    <t>NOTICE: Reference evidence by owner, date and source path only; do not duplicate system-owned master records in this support sheet.</t>
+  </si>
+  <si>
+    <t>Name / Signature / Date</t>
+  </si>
+  <si>
+    <t>No.</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>OBSERVED</t>
+  </si>
+  <si>
+    <t>OBSOLETE</t>
+  </si>
+  <si>
+    <t>ON HOLD</t>
+  </si>
+  <si>
+    <t>OPEN</t>
+  </si>
+  <si>
+    <t>OWNER</t>
+  </si>
+  <si>
+    <t>Obsolete Count</t>
+  </si>
+  <si>
+    <t>Open Issues</t>
+  </si>
+  <si>
+    <t>Overdue Count</t>
+  </si>
+  <si>
+    <t>Owner</t>
+  </si>
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
+    <t>PEOPLE</t>
+  </si>
+  <si>
+    <t>PESTLE</t>
+  </si>
+  <si>
+    <t>PLANNING</t>
+  </si>
+  <si>
+    <t>PO</t>
+  </si>
+  <si>
+    <t>POLICY</t>
+  </si>
+  <si>
+    <t>PORTAL</t>
+  </si>
+  <si>
+    <t>PRESENT</t>
+  </si>
+  <si>
+    <t>PREVENTION</t>
+  </si>
+  <si>
+    <t>PROCESS</t>
+  </si>
+  <si>
+    <t>PROD</t>
+  </si>
+  <si>
+    <t>PUR</t>
+  </si>
+  <si>
+    <t>Per authority matrix</t>
+  </si>
+  <si>
+    <t>Prepared By</t>
+  </si>
+  <si>
+    <t>Prepared Date</t>
+  </si>
+  <si>
+    <t>Process Owner</t>
+  </si>
+  <si>
+    <t>Purpose</t>
+  </si>
+  <si>
+    <t>QA</t>
+  </si>
+  <si>
+    <t>QMS</t>
+  </si>
+  <si>
+    <t>QUALITY</t>
+  </si>
+  <si>
+    <t>QUOTE</t>
+  </si>
+  <si>
+    <t>Quality Management System · Controlled Document</t>
+  </si>
+  <si>
+    <t>REACTION_CLASS</t>
+  </si>
+  <si>
+    <t>RECHECK</t>
+  </si>
+  <si>
+    <t>RECORD</t>
+  </si>
+  <si>
+    <t>RECOVERING</t>
+  </si>
+  <si>
+    <t>RECOVERY_STATUS</t>
+  </si>
+  <si>
+    <t>REGULATORY</t>
+  </si>
+  <si>
+    <t>REJECTED</t>
+  </si>
+  <si>
+    <t>REMOVE</t>
+  </si>
+  <si>
+    <t>REQUESTER</t>
+  </si>
+  <si>
+    <t>RESPONSE</t>
+  </si>
+  <si>
+    <t>RESTORED</t>
+  </si>
+  <si>
+    <t>RESULT</t>
+  </si>
+  <si>
+    <t>REVIEWER</t>
+  </si>
+  <si>
+    <t>RISK</t>
+  </si>
+  <si>
+    <t>RISK_CATEGORY</t>
+  </si>
+  <si>
+    <t>ROLE</t>
+  </si>
+  <si>
+    <t>ROLE_ACCESS_PROFILE</t>
+  </si>
+  <si>
+    <t>Record ID</t>
+  </si>
+  <si>
+    <t>Record Status</t>
+  </si>
+  <si>
+    <t>Record traceable evidence references only; do not duplicate system-owned master data.</t>
+  </si>
+  <si>
+    <t>Reference Path or Link</t>
+  </si>
+  <si>
+    <t>Register identity / revision only; do not recreate operational content from other packs.</t>
+  </si>
+  <si>
+    <t>Related Record</t>
+  </si>
+  <si>
+    <t>Remarks</t>
+  </si>
+  <si>
+    <t>Retention / Archive Ref</t>
+  </si>
+  <si>
+    <t>Review Date</t>
+  </si>
+  <si>
+    <t>Review Due</t>
+  </si>
+  <si>
+    <t>Review Period</t>
+  </si>
+  <si>
+    <t>Reviewed By</t>
+  </si>
+  <si>
+    <t>Reviewer</t>
+  </si>
+  <si>
+    <t>Revision</t>
+  </si>
+  <si>
+    <t>SAFETY</t>
+  </si>
+  <si>
+    <t>SALES</t>
+  </si>
+  <si>
+    <t>SAMPLE_FREQUENCY</t>
+  </si>
+  <si>
+    <t>SEGREGATE</t>
+  </si>
+  <si>
+    <t>SHIFT</t>
+  </si>
+  <si>
+    <t>SHIPPING</t>
+  </si>
+  <si>
+    <t>SO</t>
+  </si>
+  <si>
+    <t>SOP</t>
+  </si>
+  <si>
+    <t>SOP: SOP-101, SOP-102</t>
+  </si>
+  <si>
+    <t>STATUS</t>
+  </si>
+  <si>
+    <t>STOP</t>
+  </si>
+  <si>
+    <t>SUPERSEDED</t>
+  </si>
+  <si>
+    <t>SUPERVISED</t>
+  </si>
+  <si>
+    <t>SUSPENDED</t>
+  </si>
+  <si>
+    <t>SWOT</t>
+  </si>
+  <si>
+    <t>SYSTEM</t>
+  </si>
+  <si>
+    <t>Source Links</t>
+  </si>
+  <si>
+    <t>Source System</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Storage Path</t>
+  </si>
+  <si>
+    <t>Superseded Ref</t>
+  </si>
+  <si>
+    <t>TRAINER</t>
+  </si>
+  <si>
+    <t>TRAINING</t>
+  </si>
+  <si>
+    <t>V0</t>
+  </si>
+  <si>
+    <t>VIEWER</t>
+  </si>
+  <si>
+    <t>VISUAL</t>
+  </si>
+  <si>
+    <t>WEEKLY</t>
+  </si>
+  <si>
+    <t>WHS</t>
+  </si>
+  <si>
+    <t>WI</t>
+  </si>
+  <si>
+    <t>YES</t>
+  </si>
+  <si>
+    <t>YES_NO</t>
+  </si>
+  <si>
+    <t>YYYY-MM-DD</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -140,8 +880,13 @@
       <color rgb="001B3A6B"/>
       <sz val="14"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="007B4F00"/>
+      <sz val="7"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -198,8 +943,13 @@
         <fgColor rgb="000C2D48"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF8E1"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="147">
+  <borders count="150">
     <border>
       <left/>
       <right/>
@@ -1785,11 +2535,45 @@
       </top>
       <bottom/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00F9A825"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="00F9A825"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00F9A825"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00F9A825"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00F9A825"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00F9A825"/>
+      </right>
+      <top style="thin">
+        <color rgb="00F9A825"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00F9A825"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="409">
+  <cellXfs count="412">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -2878,6 +3662,15 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="132" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="147" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="148" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="149" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5711,67 +6504,67 @@
       <c r="BC37" s="32" t="n"/>
       <c r="BD37" s="368" t="n"/>
     </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="360" t="inlineStr">
+    <row r="38" ht="26" customHeight="1">
+      <c r="A38" s="409" t="inlineStr">
         <is>
           <t>NOTICE: Keep one row per controlled document. Maintain code, revision, status, effective date, storage path and superseded reference so documented information stays traceable and current.</t>
         </is>
       </c>
-      <c r="B38" s="22" t="n"/>
-      <c r="C38" s="22" t="n"/>
-      <c r="D38" s="22" t="n"/>
-      <c r="E38" s="22" t="n"/>
-      <c r="F38" s="22" t="n"/>
-      <c r="G38" s="22" t="n"/>
-      <c r="H38" s="22" t="n"/>
-      <c r="I38" s="22" t="n"/>
-      <c r="J38" s="22" t="n"/>
-      <c r="K38" s="22" t="n"/>
-      <c r="L38" s="22" t="n"/>
-      <c r="M38" s="22" t="n"/>
-      <c r="N38" s="22" t="n"/>
-      <c r="O38" s="22" t="n"/>
-      <c r="P38" s="22" t="n"/>
-      <c r="Q38" s="22" t="n"/>
-      <c r="R38" s="22" t="n"/>
-      <c r="S38" s="22" t="n"/>
-      <c r="T38" s="22" t="n"/>
-      <c r="U38" s="22" t="n"/>
-      <c r="V38" s="22" t="n"/>
-      <c r="W38" s="22" t="n"/>
-      <c r="X38" s="22" t="n"/>
-      <c r="Y38" s="22" t="n"/>
-      <c r="Z38" s="22" t="n"/>
-      <c r="AA38" s="22" t="n"/>
-      <c r="AB38" s="22" t="n"/>
-      <c r="AC38" s="22" t="n"/>
-      <c r="AD38" s="22" t="n"/>
-      <c r="AE38" s="22" t="n"/>
-      <c r="AF38" s="22" t="n"/>
-      <c r="AG38" s="22" t="n"/>
-      <c r="AH38" s="22" t="n"/>
-      <c r="AI38" s="22" t="n"/>
-      <c r="AJ38" s="22" t="n"/>
-      <c r="AK38" s="22" t="n"/>
-      <c r="AL38" s="22" t="n"/>
-      <c r="AM38" s="22" t="n"/>
-      <c r="AN38" s="22" t="n"/>
-      <c r="AO38" s="22" t="n"/>
-      <c r="AP38" s="22" t="n"/>
-      <c r="AQ38" s="22" t="n"/>
-      <c r="AR38" s="22" t="n"/>
-      <c r="AS38" s="22" t="n"/>
-      <c r="AT38" s="22" t="n"/>
-      <c r="AU38" s="22" t="n"/>
-      <c r="AV38" s="22" t="n"/>
-      <c r="AW38" s="22" t="n"/>
-      <c r="AX38" s="22" t="n"/>
-      <c r="AY38" s="22" t="n"/>
-      <c r="AZ38" s="22" t="n"/>
-      <c r="BA38" s="22" t="n"/>
-      <c r="BB38" s="22" t="n"/>
-      <c r="BC38" s="22" t="n"/>
-      <c r="BD38" s="23" t="n"/>
+      <c r="B38" s="410" t="n"/>
+      <c r="C38" s="410" t="n"/>
+      <c r="D38" s="410" t="n"/>
+      <c r="E38" s="410" t="n"/>
+      <c r="F38" s="410" t="n"/>
+      <c r="G38" s="410" t="n"/>
+      <c r="H38" s="410" t="n"/>
+      <c r="I38" s="410" t="n"/>
+      <c r="J38" s="410" t="n"/>
+      <c r="K38" s="410" t="n"/>
+      <c r="L38" s="410" t="n"/>
+      <c r="M38" s="410" t="n"/>
+      <c r="N38" s="410" t="n"/>
+      <c r="O38" s="410" t="n"/>
+      <c r="P38" s="410" t="n"/>
+      <c r="Q38" s="410" t="n"/>
+      <c r="R38" s="410" t="n"/>
+      <c r="S38" s="410" t="n"/>
+      <c r="T38" s="410" t="n"/>
+      <c r="U38" s="410" t="n"/>
+      <c r="V38" s="410" t="n"/>
+      <c r="W38" s="410" t="n"/>
+      <c r="X38" s="410" t="n"/>
+      <c r="Y38" s="410" t="n"/>
+      <c r="Z38" s="410" t="n"/>
+      <c r="AA38" s="410" t="n"/>
+      <c r="AB38" s="410" t="n"/>
+      <c r="AC38" s="410" t="n"/>
+      <c r="AD38" s="410" t="n"/>
+      <c r="AE38" s="410" t="n"/>
+      <c r="AF38" s="410" t="n"/>
+      <c r="AG38" s="410" t="n"/>
+      <c r="AH38" s="410" t="n"/>
+      <c r="AI38" s="410" t="n"/>
+      <c r="AJ38" s="410" t="n"/>
+      <c r="AK38" s="410" t="n"/>
+      <c r="AL38" s="410" t="n"/>
+      <c r="AM38" s="410" t="n"/>
+      <c r="AN38" s="410" t="n"/>
+      <c r="AO38" s="410" t="n"/>
+      <c r="AP38" s="410" t="n"/>
+      <c r="AQ38" s="410" t="n"/>
+      <c r="AR38" s="410" t="n"/>
+      <c r="AS38" s="410" t="n"/>
+      <c r="AT38" s="410" t="n"/>
+      <c r="AU38" s="410" t="n"/>
+      <c r="AV38" s="410" t="n"/>
+      <c r="AW38" s="410" t="n"/>
+      <c r="AX38" s="410" t="n"/>
+      <c r="AY38" s="410" t="n"/>
+      <c r="AZ38" s="410" t="n"/>
+      <c r="BA38" s="410" t="n"/>
+      <c r="BB38" s="410" t="n"/>
+      <c r="BC38" s="410" t="n"/>
+      <c r="BD38" s="411" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>

</xml_diff>

<commit_message>
Tối ưu hiển thị di động portal
</commit_message>
<xml_diff>
--- a/04-Bieu-Mau/01-FRM-100/FRM-101_Master_Document_Register.xlsx
+++ b/04-Bieu-Mau/01-FRM-100/FRM-101_Master_Document_Register.xlsx
@@ -949,7 +949,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="150">
+  <borders count="155">
     <border>
       <left/>
       <right/>
@@ -2568,6 +2568,64 @@
       <bottom style="thin">
         <color rgb="00F9A825"/>
       </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00F9A825"/>
+      </left>
+      <right style="thin">
+        <color rgb="00F9A825"/>
+      </right>
+      <top style="thin">
+        <color rgb="00F9A825"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00F9A825"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00F9A825"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00F9A825"/>
+      </right>
+      <top style="thin">
+        <color rgb="00F9A825"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00F9A825"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00F9A825"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00F9A825"/>
+      </right>
+      <top style="thin">
+        <color rgb="00F9A825"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00F9A825"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">

</xml_diff>

<commit_message>
Optimize portal mobile layout
</commit_message>
<xml_diff>
--- a/04-Bieu-Mau/01-FRM-100/FRM-101_Master_Document_Register.xlsx
+++ b/04-Bieu-Mau/01-FRM-100/FRM-101_Master_Document_Register.xlsx
@@ -24,746 +24,6 @@
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" calcOnSave="1" forceFullCalc="1"/>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="245">
-  <si>
-    <t>  1. CONTROLLED LOOKUP LISTS</t>
-  </si>
-  <si>
-    <t>  1. REFERENCE INFORMATION</t>
-  </si>
-  <si>
-    <t>  2. ACTIVE LOG TABLE</t>
-  </si>
-  <si>
-    <t>  3. PERIODIC REVIEW / CLOSURE</t>
-  </si>
-  <si>
-    <t>  4. PERIODIC REVIEW SIGN-OFF</t>
-  </si>
-  <si>
-    <t>  REFERENCE / SOURCE CONTEXT</t>
-  </si>
-  <si>
-    <t>  SUPPORT TABLE</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>=ROW()-ROW($A$14)+1</t>
-  </si>
-  <si>
-    <t>ABSENT</t>
-  </si>
-  <si>
-    <t>ACCESS</t>
-  </si>
-  <si>
-    <t>ACCESS_ACTION_TYPE</t>
-  </si>
-  <si>
-    <t>ADJUST</t>
-  </si>
-  <si>
-    <t>ADMIN</t>
-  </si>
-  <si>
-    <t>ALL HANDS</t>
-  </si>
-  <si>
-    <t>ANNEX</t>
-  </si>
-  <si>
-    <t>APPROVED</t>
-  </si>
-  <si>
-    <t>APPROVER</t>
-  </si>
-  <si>
-    <t>ATTENDANCE_STATUS</t>
-  </si>
-  <si>
-    <t>AUDIENCE_CLASS</t>
-  </si>
-  <si>
-    <t>AUDIT_FINDING_SEVERITY</t>
-  </si>
-  <si>
-    <t>AUTHORITY_ROLE</t>
-  </si>
-  <si>
-    <t>AUTHORIZATION_STATUS</t>
-  </si>
-  <si>
-    <t>AUTHORIZED</t>
-  </si>
-  <si>
-    <t>Approved</t>
-  </si>
-  <si>
-    <t>Approved by</t>
-  </si>
-  <si>
-    <t>BACKUP_FLAG</t>
-  </si>
-  <si>
-    <t>Boundary / SoR</t>
-  </si>
-  <si>
-    <t>CHANGE</t>
-  </si>
-  <si>
-    <t>CHANGE_PRIORITY</t>
-  </si>
-  <si>
-    <t>CHANGE_TYPE</t>
-  </si>
-  <si>
-    <t>CLOSED</t>
-  </si>
-  <si>
-    <t>COMMERCIAL_REFERENCE</t>
-  </si>
-  <si>
-    <t>COMM_CHANNEL</t>
-  </si>
-  <si>
-    <t>COMPETENCY_LEVEL</t>
-  </si>
-  <si>
-    <t>COMPLIANCE</t>
-  </si>
-  <si>
-    <t>CONDITIONAL</t>
-  </si>
-  <si>
-    <t>CONFIGURATION</t>
-  </si>
-  <si>
-    <t>CONTAINED</t>
-  </si>
-  <si>
-    <t>CONTEXT_CLASS</t>
-  </si>
-  <si>
-    <t>CONTRACT</t>
-  </si>
-  <si>
-    <t>CONTRACT REVIEW</t>
-  </si>
-  <si>
-    <t>CONTRIBUTOR</t>
-  </si>
-  <si>
-    <t>CONTROL_METHOD</t>
-  </si>
-  <si>
-    <t>COST</t>
-  </si>
-  <si>
-    <t>CREATE</t>
-  </si>
-  <si>
-    <t>CRITICAL</t>
-  </si>
-  <si>
-    <t>CSR</t>
-  </si>
-  <si>
-    <t>CUSTOMER</t>
-  </si>
-  <si>
-    <t>DAILY</t>
-  </si>
-  <si>
-    <t>DECISION</t>
-  </si>
-  <si>
-    <t>DELIVERY</t>
-  </si>
-  <si>
-    <t>DEPT</t>
-  </si>
-  <si>
-    <t>DETECTION</t>
-  </si>
-  <si>
-    <t>DIMENSIONAL</t>
-  </si>
-  <si>
-    <t>DOCUMENT</t>
-  </si>
-  <si>
-    <t>DOC_STATUS</t>
-  </si>
-  <si>
-    <t>DOC_TYPE</t>
-  </si>
-  <si>
-    <t>DRAFT</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Department / Owner</t>
-  </si>
-  <si>
-    <t>Deployment Evidence Ref</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Doc Type</t>
-  </si>
-  <si>
-    <t>Document Code</t>
-  </si>
-  <si>
-    <t>Document Code / Title</t>
-  </si>
-  <si>
-    <t>Document Register Period</t>
-  </si>
-  <si>
-    <t>Document Title</t>
-  </si>
-  <si>
-    <t>EACH LOT</t>
-  </si>
-  <si>
-    <t>EFFECTIVE</t>
-  </si>
-  <si>
-    <t>EMAIL</t>
-  </si>
-  <si>
-    <t>ENG</t>
-  </si>
-  <si>
-    <t>ESCALATE</t>
-  </si>
-  <si>
-    <t>ESCALATED</t>
-  </si>
-  <si>
-    <t>ESCALATION</t>
-  </si>
-  <si>
-    <t>EXCUSED</t>
-  </si>
-  <si>
-    <t>EXPIRED</t>
-  </si>
-  <si>
-    <t>Eff. Date</t>
-  </si>
-  <si>
-    <t>Effective Date</t>
-  </si>
-  <si>
-    <t>Evidence ID</t>
-  </si>
-  <si>
-    <t>Evidence Ref</t>
-  </si>
-  <si>
-    <t>Excel Table — rolling document register (freeze / filter required)</t>
-  </si>
-  <si>
-    <t>FAIL</t>
-  </si>
-  <si>
-    <t>FINAL</t>
-  </si>
-  <si>
-    <t>FIRST ARTICLE</t>
-  </si>
-  <si>
-    <t>FIRST OFF</t>
-  </si>
-  <si>
-    <t>FIRST PIECE</t>
-  </si>
-  <si>
-    <t>FMEA_RANK</t>
-  </si>
-  <si>
-    <t>FORM</t>
-  </si>
-  <si>
-    <t>FRM-101</t>
-  </si>
-  <si>
-    <t>FUNCTION</t>
-  </si>
-  <si>
-    <t>FUNCTIONAL</t>
-  </si>
-  <si>
-    <t>Form Code</t>
-  </si>
-  <si>
-    <t>GATE</t>
-  </si>
-  <si>
-    <t>HESEM Engineering · ISO 9001 / AS9100 · Semiconductor Equipment Parts</t>
-  </si>
-  <si>
-    <t>HIGH</t>
-  </si>
-  <si>
-    <t>HOLD</t>
-  </si>
-  <si>
-    <t>HOURLY</t>
-  </si>
-  <si>
-    <t>HR</t>
-  </si>
-  <si>
-    <t>IMPACT_LEVEL</t>
-  </si>
-  <si>
-    <t>IMPACT_SCOPE</t>
-  </si>
-  <si>
-    <t>IN PROCESS</t>
-  </si>
-  <si>
-    <t>IN PROGRESS</t>
-  </si>
-  <si>
-    <t>IN-PROCESS</t>
-  </si>
-  <si>
-    <t>INTERNAL</t>
-  </si>
-  <si>
-    <t>IT</t>
-  </si>
-  <si>
-    <t>KPI-COST</t>
-  </si>
-  <si>
-    <t>KPI-DELIVERY</t>
-  </si>
-  <si>
-    <t>KPI-QUALITY</t>
-  </si>
-  <si>
-    <t>KPI-SAFETY</t>
-  </si>
-  <si>
-    <t>KPI-TRAINING</t>
-  </si>
-  <si>
-    <t>KPI_OWNER_SET</t>
-  </si>
-  <si>
-    <t>LATE</t>
-  </si>
-  <si>
-    <t>LESSON_CLASS</t>
-  </si>
-  <si>
-    <t>LOW</t>
-  </si>
-  <si>
-    <t>M365 / shared workbook remains the master list and evidence owner; workbook captures controlled review / log rows only and must not duplicate system-owned master data.</t>
-  </si>
-  <si>
-    <t>MAJOR</t>
-  </si>
-  <si>
-    <t>MANAGEMENT</t>
-  </si>
-  <si>
-    <t>MASTER DOCUMENT REGISTER</t>
-  </si>
-  <si>
-    <t>MASTER DOCUMENT REGISTER — CONTROLLED LOOKUP LISTS</t>
-  </si>
-  <si>
-    <t>MASTER DOCUMENT REGISTER — EVIDENCE REFERENCE REGISTER</t>
-  </si>
-  <si>
-    <t>MASTER DOCUMENT REGISTER — REVIEW QUESTIONS / PERIODIC REVIEW</t>
-  </si>
-  <si>
-    <t>MEDIUM</t>
-  </si>
-  <si>
-    <t>MEETING</t>
-  </si>
-  <si>
-    <t>MGT</t>
-  </si>
-  <si>
-    <t>MINOR</t>
-  </si>
-  <si>
-    <t>MONITORING</t>
-  </si>
-  <si>
-    <t>Migration Status</t>
-  </si>
-  <si>
-    <t>NA</t>
-  </si>
-  <si>
-    <t>NO</t>
-  </si>
-  <si>
-    <t>NONE</t>
-  </si>
-  <si>
-    <t>NOT AUTHORIZED</t>
-  </si>
-  <si>
-    <t>NOT TRAINED</t>
-  </si>
-  <si>
-    <t>NOTICE</t>
-  </si>
-  <si>
-    <t>NOTICE: Controlled dropdown source sheet. Do not edit values without formal document control because validations in the workbook depend on these lists.</t>
-  </si>
-  <si>
-    <t>NOTICE: Controlled lookup lists only. Change values only through formal document control because dropdown behavior and validation depend on this sheet.</t>
-  </si>
-  <si>
-    <t>NOTICE: Keep one row per controlled document. Maintain code, revision, status, effective date, storage path and superseded reference so documented information stays traceable and current.</t>
-  </si>
-  <si>
-    <t>NOTICE: Keep review questions and periodic review data aligned to the current controlled criteria set; do not embed unofficial rules in this support sheet.</t>
-  </si>
-  <si>
-    <t>NOTICE: Reference evidence by owner, date and source path only; do not duplicate system-owned master records in this support sheet.</t>
-  </si>
-  <si>
-    <t>Name / Signature / Date</t>
-  </si>
-  <si>
-    <t>No.</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>OBSERVED</t>
-  </si>
-  <si>
-    <t>OBSOLETE</t>
-  </si>
-  <si>
-    <t>ON HOLD</t>
-  </si>
-  <si>
-    <t>OPEN</t>
-  </si>
-  <si>
-    <t>OWNER</t>
-  </si>
-  <si>
-    <t>Obsolete Count</t>
-  </si>
-  <si>
-    <t>Open Issues</t>
-  </si>
-  <si>
-    <t>Overdue Count</t>
-  </si>
-  <si>
-    <t>Owner</t>
-  </si>
-  <si>
-    <t>PASS</t>
-  </si>
-  <si>
-    <t>PEOPLE</t>
-  </si>
-  <si>
-    <t>PESTLE</t>
-  </si>
-  <si>
-    <t>PLANNING</t>
-  </si>
-  <si>
-    <t>PO</t>
-  </si>
-  <si>
-    <t>POLICY</t>
-  </si>
-  <si>
-    <t>PORTAL</t>
-  </si>
-  <si>
-    <t>PRESENT</t>
-  </si>
-  <si>
-    <t>PREVENTION</t>
-  </si>
-  <si>
-    <t>PROCESS</t>
-  </si>
-  <si>
-    <t>PROD</t>
-  </si>
-  <si>
-    <t>PUR</t>
-  </si>
-  <si>
-    <t>Per authority matrix</t>
-  </si>
-  <si>
-    <t>Prepared By</t>
-  </si>
-  <si>
-    <t>Prepared Date</t>
-  </si>
-  <si>
-    <t>Process Owner</t>
-  </si>
-  <si>
-    <t>Purpose</t>
-  </si>
-  <si>
-    <t>QA</t>
-  </si>
-  <si>
-    <t>QMS</t>
-  </si>
-  <si>
-    <t>QUALITY</t>
-  </si>
-  <si>
-    <t>QUOTE</t>
-  </si>
-  <si>
-    <t>Quality Management System · Controlled Document</t>
-  </si>
-  <si>
-    <t>REACTION_CLASS</t>
-  </si>
-  <si>
-    <t>RECHECK</t>
-  </si>
-  <si>
-    <t>RECORD</t>
-  </si>
-  <si>
-    <t>RECOVERING</t>
-  </si>
-  <si>
-    <t>RECOVERY_STATUS</t>
-  </si>
-  <si>
-    <t>REGULATORY</t>
-  </si>
-  <si>
-    <t>REJECTED</t>
-  </si>
-  <si>
-    <t>REMOVE</t>
-  </si>
-  <si>
-    <t>REQUESTER</t>
-  </si>
-  <si>
-    <t>RESPONSE</t>
-  </si>
-  <si>
-    <t>RESTORED</t>
-  </si>
-  <si>
-    <t>RESULT</t>
-  </si>
-  <si>
-    <t>REVIEWER</t>
-  </si>
-  <si>
-    <t>RISK</t>
-  </si>
-  <si>
-    <t>RISK_CATEGORY</t>
-  </si>
-  <si>
-    <t>ROLE</t>
-  </si>
-  <si>
-    <t>ROLE_ACCESS_PROFILE</t>
-  </si>
-  <si>
-    <t>Record ID</t>
-  </si>
-  <si>
-    <t>Record Status</t>
-  </si>
-  <si>
-    <t>Record traceable evidence references only; do not duplicate system-owned master data.</t>
-  </si>
-  <si>
-    <t>Reference Path or Link</t>
-  </si>
-  <si>
-    <t>Register identity / revision only; do not recreate operational content from other packs.</t>
-  </si>
-  <si>
-    <t>Related Record</t>
-  </si>
-  <si>
-    <t>Remarks</t>
-  </si>
-  <si>
-    <t>Retention / Archive Ref</t>
-  </si>
-  <si>
-    <t>Review Date</t>
-  </si>
-  <si>
-    <t>Review Due</t>
-  </si>
-  <si>
-    <t>Review Period</t>
-  </si>
-  <si>
-    <t>Reviewed By</t>
-  </si>
-  <si>
-    <t>Reviewer</t>
-  </si>
-  <si>
-    <t>Revision</t>
-  </si>
-  <si>
-    <t>SAFETY</t>
-  </si>
-  <si>
-    <t>SALES</t>
-  </si>
-  <si>
-    <t>SAMPLE_FREQUENCY</t>
-  </si>
-  <si>
-    <t>SEGREGATE</t>
-  </si>
-  <si>
-    <t>SHIFT</t>
-  </si>
-  <si>
-    <t>SHIPPING</t>
-  </si>
-  <si>
-    <t>SO</t>
-  </si>
-  <si>
-    <t>SOP</t>
-  </si>
-  <si>
-    <t>SOP: SOP-101, SOP-102</t>
-  </si>
-  <si>
-    <t>STATUS</t>
-  </si>
-  <si>
-    <t>STOP</t>
-  </si>
-  <si>
-    <t>SUPERSEDED</t>
-  </si>
-  <si>
-    <t>SUPERVISED</t>
-  </si>
-  <si>
-    <t>SUSPENDED</t>
-  </si>
-  <si>
-    <t>SWOT</t>
-  </si>
-  <si>
-    <t>SYSTEM</t>
-  </si>
-  <si>
-    <t>Source Links</t>
-  </si>
-  <si>
-    <t>Source System</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Storage Path</t>
-  </si>
-  <si>
-    <t>Superseded Ref</t>
-  </si>
-  <si>
-    <t>TRAINER</t>
-  </si>
-  <si>
-    <t>TRAINING</t>
-  </si>
-  <si>
-    <t>V0</t>
-  </si>
-  <si>
-    <t>VIEWER</t>
-  </si>
-  <si>
-    <t>VISUAL</t>
-  </si>
-  <si>
-    <t>WEEKLY</t>
-  </si>
-  <si>
-    <t>WHS</t>
-  </si>
-  <si>
-    <t>WI</t>
-  </si>
-  <si>
-    <t>YES</t>
-  </si>
-  <si>
-    <t>YES_NO</t>
-  </si>
-  <si>
-    <t>YYYY-MM-DD</t>
-  </si>
-</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8035,67 +7295,67 @@
       <c r="BC18" s="371" t="n"/>
       <c r="BD18" s="375" t="n"/>
     </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="360" t="inlineStr">
+    <row r="19" ht="26" customHeight="1">
+      <c r="A19" s="409" t="inlineStr">
         <is>
           <t>NOTICE: Keep review questions and periodic review data aligned to the current controlled criteria set; do not embed unofficial rules in this support sheet.</t>
         </is>
       </c>
-      <c r="B19" s="22" t="n"/>
-      <c r="C19" s="22" t="n"/>
-      <c r="D19" s="22" t="n"/>
-      <c r="E19" s="22" t="n"/>
-      <c r="F19" s="22" t="n"/>
-      <c r="G19" s="22" t="n"/>
-      <c r="H19" s="22" t="n"/>
-      <c r="I19" s="22" t="n"/>
-      <c r="J19" s="22" t="n"/>
-      <c r="K19" s="22" t="n"/>
-      <c r="L19" s="22" t="n"/>
-      <c r="M19" s="22" t="n"/>
-      <c r="N19" s="22" t="n"/>
-      <c r="O19" s="22" t="n"/>
-      <c r="P19" s="22" t="n"/>
-      <c r="Q19" s="22" t="n"/>
-      <c r="R19" s="22" t="n"/>
-      <c r="S19" s="22" t="n"/>
-      <c r="T19" s="22" t="n"/>
-      <c r="U19" s="22" t="n"/>
-      <c r="V19" s="22" t="n"/>
-      <c r="W19" s="22" t="n"/>
-      <c r="X19" s="22" t="n"/>
-      <c r="Y19" s="22" t="n"/>
-      <c r="Z19" s="22" t="n"/>
-      <c r="AA19" s="22" t="n"/>
-      <c r="AB19" s="22" t="n"/>
-      <c r="AC19" s="22" t="n"/>
-      <c r="AD19" s="22" t="n"/>
-      <c r="AE19" s="22" t="n"/>
-      <c r="AF19" s="22" t="n"/>
-      <c r="AG19" s="22" t="n"/>
-      <c r="AH19" s="22" t="n"/>
-      <c r="AI19" s="22" t="n"/>
-      <c r="AJ19" s="22" t="n"/>
-      <c r="AK19" s="22" t="n"/>
-      <c r="AL19" s="22" t="n"/>
-      <c r="AM19" s="22" t="n"/>
-      <c r="AN19" s="22" t="n"/>
-      <c r="AO19" s="22" t="n"/>
-      <c r="AP19" s="22" t="n"/>
-      <c r="AQ19" s="22" t="n"/>
-      <c r="AR19" s="22" t="n"/>
-      <c r="AS19" s="22" t="n"/>
-      <c r="AT19" s="22" t="n"/>
-      <c r="AU19" s="22" t="n"/>
-      <c r="AV19" s="22" t="n"/>
-      <c r="AW19" s="22" t="n"/>
-      <c r="AX19" s="22" t="n"/>
-      <c r="AY19" s="22" t="n"/>
-      <c r="AZ19" s="22" t="n"/>
-      <c r="BA19" s="22" t="n"/>
-      <c r="BB19" s="22" t="n"/>
-      <c r="BC19" s="22" t="n"/>
-      <c r="BD19" s="23" t="n"/>
+      <c r="B19" s="410" t="n"/>
+      <c r="C19" s="410" t="n"/>
+      <c r="D19" s="410" t="n"/>
+      <c r="E19" s="410" t="n"/>
+      <c r="F19" s="410" t="n"/>
+      <c r="G19" s="410" t="n"/>
+      <c r="H19" s="410" t="n"/>
+      <c r="I19" s="410" t="n"/>
+      <c r="J19" s="410" t="n"/>
+      <c r="K19" s="410" t="n"/>
+      <c r="L19" s="410" t="n"/>
+      <c r="M19" s="410" t="n"/>
+      <c r="N19" s="410" t="n"/>
+      <c r="O19" s="410" t="n"/>
+      <c r="P19" s="410" t="n"/>
+      <c r="Q19" s="410" t="n"/>
+      <c r="R19" s="410" t="n"/>
+      <c r="S19" s="410" t="n"/>
+      <c r="T19" s="410" t="n"/>
+      <c r="U19" s="410" t="n"/>
+      <c r="V19" s="410" t="n"/>
+      <c r="W19" s="410" t="n"/>
+      <c r="X19" s="410" t="n"/>
+      <c r="Y19" s="410" t="n"/>
+      <c r="Z19" s="410" t="n"/>
+      <c r="AA19" s="410" t="n"/>
+      <c r="AB19" s="410" t="n"/>
+      <c r="AC19" s="410" t="n"/>
+      <c r="AD19" s="410" t="n"/>
+      <c r="AE19" s="410" t="n"/>
+      <c r="AF19" s="410" t="n"/>
+      <c r="AG19" s="410" t="n"/>
+      <c r="AH19" s="410" t="n"/>
+      <c r="AI19" s="410" t="n"/>
+      <c r="AJ19" s="410" t="n"/>
+      <c r="AK19" s="410" t="n"/>
+      <c r="AL19" s="410" t="n"/>
+      <c r="AM19" s="410" t="n"/>
+      <c r="AN19" s="410" t="n"/>
+      <c r="AO19" s="410" t="n"/>
+      <c r="AP19" s="410" t="n"/>
+      <c r="AQ19" s="410" t="n"/>
+      <c r="AR19" s="410" t="n"/>
+      <c r="AS19" s="410" t="n"/>
+      <c r="AT19" s="410" t="n"/>
+      <c r="AU19" s="410" t="n"/>
+      <c r="AV19" s="410" t="n"/>
+      <c r="AW19" s="410" t="n"/>
+      <c r="AX19" s="410" t="n"/>
+      <c r="AY19" s="410" t="n"/>
+      <c r="AZ19" s="410" t="n"/>
+      <c r="BA19" s="410" t="n"/>
+      <c r="BB19" s="410" t="n"/>
+      <c r="BC19" s="410" t="n"/>
+      <c r="BD19" s="411" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
@@ -9253,67 +8513,67 @@
       <c r="BC17" s="371" t="n"/>
       <c r="BD17" s="375" t="n"/>
     </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="360" t="inlineStr">
+    <row r="18" ht="26" customHeight="1">
+      <c r="A18" s="409" t="inlineStr">
         <is>
           <t>NOTICE: Reference evidence by owner, date and source path only; do not duplicate system-owned master records in this support sheet.</t>
         </is>
       </c>
-      <c r="B18" s="22" t="n"/>
-      <c r="C18" s="22" t="n"/>
-      <c r="D18" s="22" t="n"/>
-      <c r="E18" s="22" t="n"/>
-      <c r="F18" s="22" t="n"/>
-      <c r="G18" s="22" t="n"/>
-      <c r="H18" s="22" t="n"/>
-      <c r="I18" s="22" t="n"/>
-      <c r="J18" s="22" t="n"/>
-      <c r="K18" s="22" t="n"/>
-      <c r="L18" s="22" t="n"/>
-      <c r="M18" s="22" t="n"/>
-      <c r="N18" s="22" t="n"/>
-      <c r="O18" s="22" t="n"/>
-      <c r="P18" s="22" t="n"/>
-      <c r="Q18" s="22" t="n"/>
-      <c r="R18" s="22" t="n"/>
-      <c r="S18" s="22" t="n"/>
-      <c r="T18" s="22" t="n"/>
-      <c r="U18" s="22" t="n"/>
-      <c r="V18" s="22" t="n"/>
-      <c r="W18" s="22" t="n"/>
-      <c r="X18" s="22" t="n"/>
-      <c r="Y18" s="22" t="n"/>
-      <c r="Z18" s="22" t="n"/>
-      <c r="AA18" s="22" t="n"/>
-      <c r="AB18" s="22" t="n"/>
-      <c r="AC18" s="22" t="n"/>
-      <c r="AD18" s="22" t="n"/>
-      <c r="AE18" s="22" t="n"/>
-      <c r="AF18" s="22" t="n"/>
-      <c r="AG18" s="22" t="n"/>
-      <c r="AH18" s="22" t="n"/>
-      <c r="AI18" s="22" t="n"/>
-      <c r="AJ18" s="22" t="n"/>
-      <c r="AK18" s="22" t="n"/>
-      <c r="AL18" s="22" t="n"/>
-      <c r="AM18" s="22" t="n"/>
-      <c r="AN18" s="22" t="n"/>
-      <c r="AO18" s="22" t="n"/>
-      <c r="AP18" s="22" t="n"/>
-      <c r="AQ18" s="22" t="n"/>
-      <c r="AR18" s="22" t="n"/>
-      <c r="AS18" s="22" t="n"/>
-      <c r="AT18" s="22" t="n"/>
-      <c r="AU18" s="22" t="n"/>
-      <c r="AV18" s="22" t="n"/>
-      <c r="AW18" s="22" t="n"/>
-      <c r="AX18" s="22" t="n"/>
-      <c r="AY18" s="22" t="n"/>
-      <c r="AZ18" s="22" t="n"/>
-      <c r="BA18" s="22" t="n"/>
-      <c r="BB18" s="22" t="n"/>
-      <c r="BC18" s="22" t="n"/>
-      <c r="BD18" s="23" t="n"/>
+      <c r="B18" s="410" t="n"/>
+      <c r="C18" s="410" t="n"/>
+      <c r="D18" s="410" t="n"/>
+      <c r="E18" s="410" t="n"/>
+      <c r="F18" s="410" t="n"/>
+      <c r="G18" s="410" t="n"/>
+      <c r="H18" s="410" t="n"/>
+      <c r="I18" s="410" t="n"/>
+      <c r="J18" s="410" t="n"/>
+      <c r="K18" s="410" t="n"/>
+      <c r="L18" s="410" t="n"/>
+      <c r="M18" s="410" t="n"/>
+      <c r="N18" s="410" t="n"/>
+      <c r="O18" s="410" t="n"/>
+      <c r="P18" s="410" t="n"/>
+      <c r="Q18" s="410" t="n"/>
+      <c r="R18" s="410" t="n"/>
+      <c r="S18" s="410" t="n"/>
+      <c r="T18" s="410" t="n"/>
+      <c r="U18" s="410" t="n"/>
+      <c r="V18" s="410" t="n"/>
+      <c r="W18" s="410" t="n"/>
+      <c r="X18" s="410" t="n"/>
+      <c r="Y18" s="410" t="n"/>
+      <c r="Z18" s="410" t="n"/>
+      <c r="AA18" s="410" t="n"/>
+      <c r="AB18" s="410" t="n"/>
+      <c r="AC18" s="410" t="n"/>
+      <c r="AD18" s="410" t="n"/>
+      <c r="AE18" s="410" t="n"/>
+      <c r="AF18" s="410" t="n"/>
+      <c r="AG18" s="410" t="n"/>
+      <c r="AH18" s="410" t="n"/>
+      <c r="AI18" s="410" t="n"/>
+      <c r="AJ18" s="410" t="n"/>
+      <c r="AK18" s="410" t="n"/>
+      <c r="AL18" s="410" t="n"/>
+      <c r="AM18" s="410" t="n"/>
+      <c r="AN18" s="410" t="n"/>
+      <c r="AO18" s="410" t="n"/>
+      <c r="AP18" s="410" t="n"/>
+      <c r="AQ18" s="410" t="n"/>
+      <c r="AR18" s="410" t="n"/>
+      <c r="AS18" s="410" t="n"/>
+      <c r="AT18" s="410" t="n"/>
+      <c r="AU18" s="410" t="n"/>
+      <c r="AV18" s="410" t="n"/>
+      <c r="AW18" s="410" t="n"/>
+      <c r="AX18" s="410" t="n"/>
+      <c r="AY18" s="410" t="n"/>
+      <c r="AZ18" s="410" t="n"/>
+      <c r="BA18" s="410" t="n"/>
+      <c r="BB18" s="410" t="n"/>
+      <c r="BC18" s="410" t="n"/>
+      <c r="BD18" s="411" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
@@ -9771,67 +9031,67 @@
       <c r="BC7" s="22" t="n"/>
       <c r="BD7" s="23" t="n"/>
     </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="42" t="inlineStr">
+    <row r="8" ht="26" customHeight="1">
+      <c r="A8" s="409" t="inlineStr">
         <is>
           <t>NOTICE: Controlled dropdown source sheet. Do not edit values without formal document control because validations in the workbook depend on these lists.</t>
         </is>
       </c>
-      <c r="B8" s="22" t="n"/>
-      <c r="C8" s="22" t="n"/>
-      <c r="D8" s="22" t="n"/>
-      <c r="E8" s="22" t="n"/>
-      <c r="F8" s="22" t="n"/>
-      <c r="G8" s="22" t="n"/>
-      <c r="H8" s="22" t="n"/>
-      <c r="I8" s="22" t="n"/>
-      <c r="J8" s="22" t="n"/>
-      <c r="K8" s="22" t="n"/>
-      <c r="L8" s="22" t="n"/>
-      <c r="M8" s="22" t="n"/>
-      <c r="N8" s="22" t="n"/>
-      <c r="O8" s="22" t="n"/>
-      <c r="P8" s="22" t="n"/>
-      <c r="Q8" s="22" t="n"/>
-      <c r="R8" s="22" t="n"/>
-      <c r="S8" s="22" t="n"/>
-      <c r="T8" s="22" t="n"/>
-      <c r="U8" s="22" t="n"/>
-      <c r="V8" s="22" t="n"/>
-      <c r="W8" s="22" t="n"/>
-      <c r="X8" s="22" t="n"/>
-      <c r="Y8" s="22" t="n"/>
-      <c r="Z8" s="22" t="n"/>
-      <c r="AA8" s="22" t="n"/>
-      <c r="AB8" s="22" t="n"/>
-      <c r="AC8" s="22" t="n"/>
-      <c r="AD8" s="22" t="n"/>
-      <c r="AE8" s="22" t="n"/>
-      <c r="AF8" s="22" t="n"/>
-      <c r="AG8" s="22" t="n"/>
-      <c r="AH8" s="22" t="n"/>
-      <c r="AI8" s="22" t="n"/>
-      <c r="AJ8" s="22" t="n"/>
-      <c r="AK8" s="22" t="n"/>
-      <c r="AL8" s="22" t="n"/>
-      <c r="AM8" s="22" t="n"/>
-      <c r="AN8" s="22" t="n"/>
-      <c r="AO8" s="22" t="n"/>
-      <c r="AP8" s="22" t="n"/>
-      <c r="AQ8" s="22" t="n"/>
-      <c r="AR8" s="22" t="n"/>
-      <c r="AS8" s="22" t="n"/>
-      <c r="AT8" s="22" t="n"/>
-      <c r="AU8" s="22" t="n"/>
-      <c r="AV8" s="22" t="n"/>
-      <c r="AW8" s="22" t="n"/>
-      <c r="AX8" s="22" t="n"/>
-      <c r="AY8" s="22" t="n"/>
-      <c r="AZ8" s="22" t="n"/>
-      <c r="BA8" s="22" t="n"/>
-      <c r="BB8" s="22" t="n"/>
-      <c r="BC8" s="22" t="n"/>
-      <c r="BD8" s="23" t="n"/>
+      <c r="B8" s="410" t="n"/>
+      <c r="C8" s="410" t="n"/>
+      <c r="D8" s="410" t="n"/>
+      <c r="E8" s="410" t="n"/>
+      <c r="F8" s="410" t="n"/>
+      <c r="G8" s="410" t="n"/>
+      <c r="H8" s="410" t="n"/>
+      <c r="I8" s="410" t="n"/>
+      <c r="J8" s="410" t="n"/>
+      <c r="K8" s="410" t="n"/>
+      <c r="L8" s="410" t="n"/>
+      <c r="M8" s="410" t="n"/>
+      <c r="N8" s="410" t="n"/>
+      <c r="O8" s="410" t="n"/>
+      <c r="P8" s="410" t="n"/>
+      <c r="Q8" s="410" t="n"/>
+      <c r="R8" s="410" t="n"/>
+      <c r="S8" s="410" t="n"/>
+      <c r="T8" s="410" t="n"/>
+      <c r="U8" s="410" t="n"/>
+      <c r="V8" s="410" t="n"/>
+      <c r="W8" s="410" t="n"/>
+      <c r="X8" s="410" t="n"/>
+      <c r="Y8" s="410" t="n"/>
+      <c r="Z8" s="410" t="n"/>
+      <c r="AA8" s="410" t="n"/>
+      <c r="AB8" s="410" t="n"/>
+      <c r="AC8" s="410" t="n"/>
+      <c r="AD8" s="410" t="n"/>
+      <c r="AE8" s="410" t="n"/>
+      <c r="AF8" s="410" t="n"/>
+      <c r="AG8" s="410" t="n"/>
+      <c r="AH8" s="410" t="n"/>
+      <c r="AI8" s="410" t="n"/>
+      <c r="AJ8" s="410" t="n"/>
+      <c r="AK8" s="410" t="n"/>
+      <c r="AL8" s="410" t="n"/>
+      <c r="AM8" s="410" t="n"/>
+      <c r="AN8" s="410" t="n"/>
+      <c r="AO8" s="410" t="n"/>
+      <c r="AP8" s="410" t="n"/>
+      <c r="AQ8" s="410" t="n"/>
+      <c r="AR8" s="410" t="n"/>
+      <c r="AS8" s="410" t="n"/>
+      <c r="AT8" s="410" t="n"/>
+      <c r="AU8" s="410" t="n"/>
+      <c r="AV8" s="410" t="n"/>
+      <c r="AW8" s="410" t="n"/>
+      <c r="AX8" s="410" t="n"/>
+      <c r="AY8" s="410" t="n"/>
+      <c r="AZ8" s="410" t="n"/>
+      <c r="BA8" s="410" t="n"/>
+      <c r="BB8" s="410" t="n"/>
+      <c r="BC8" s="410" t="n"/>
+      <c r="BD8" s="411" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="300" t="inlineStr">
@@ -11279,67 +10539,67 @@
       <c r="BC19" s="344" t="n"/>
       <c r="BD19" s="345" t="n"/>
     </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="42" t="inlineStr">
+    <row r="20" ht="26" customHeight="1">
+      <c r="A20" s="409" t="inlineStr">
         <is>
           <t>NOTICE: Controlled lookup lists only. Change values only through formal document control because dropdown behavior and validation depend on this sheet.</t>
         </is>
       </c>
-      <c r="B20" s="22" t="n"/>
-      <c r="C20" s="22" t="n"/>
-      <c r="D20" s="22" t="n"/>
-      <c r="E20" s="22" t="n"/>
-      <c r="F20" s="22" t="n"/>
-      <c r="G20" s="22" t="n"/>
-      <c r="H20" s="22" t="n"/>
-      <c r="I20" s="22" t="n"/>
-      <c r="J20" s="22" t="n"/>
-      <c r="K20" s="22" t="n"/>
-      <c r="L20" s="22" t="n"/>
-      <c r="M20" s="22" t="n"/>
-      <c r="N20" s="22" t="n"/>
-      <c r="O20" s="22" t="n"/>
-      <c r="P20" s="22" t="n"/>
-      <c r="Q20" s="22" t="n"/>
-      <c r="R20" s="22" t="n"/>
-      <c r="S20" s="22" t="n"/>
-      <c r="T20" s="22" t="n"/>
-      <c r="U20" s="22" t="n"/>
-      <c r="V20" s="22" t="n"/>
-      <c r="W20" s="22" t="n"/>
-      <c r="X20" s="22" t="n"/>
-      <c r="Y20" s="22" t="n"/>
-      <c r="Z20" s="22" t="n"/>
-      <c r="AA20" s="22" t="n"/>
-      <c r="AB20" s="22" t="n"/>
-      <c r="AC20" s="22" t="n"/>
-      <c r="AD20" s="22" t="n"/>
-      <c r="AE20" s="22" t="n"/>
-      <c r="AF20" s="22" t="n"/>
-      <c r="AG20" s="22" t="n"/>
-      <c r="AH20" s="22" t="n"/>
-      <c r="AI20" s="22" t="n"/>
-      <c r="AJ20" s="22" t="n"/>
-      <c r="AK20" s="22" t="n"/>
-      <c r="AL20" s="22" t="n"/>
-      <c r="AM20" s="22" t="n"/>
-      <c r="AN20" s="22" t="n"/>
-      <c r="AO20" s="22" t="n"/>
-      <c r="AP20" s="22" t="n"/>
-      <c r="AQ20" s="22" t="n"/>
-      <c r="AR20" s="22" t="n"/>
-      <c r="AS20" s="22" t="n"/>
-      <c r="AT20" s="22" t="n"/>
-      <c r="AU20" s="22" t="n"/>
-      <c r="AV20" s="22" t="n"/>
-      <c r="AW20" s="22" t="n"/>
-      <c r="AX20" s="22" t="n"/>
-      <c r="AY20" s="22" t="n"/>
-      <c r="AZ20" s="22" t="n"/>
-      <c r="BA20" s="22" t="n"/>
-      <c r="BB20" s="22" t="n"/>
-      <c r="BC20" s="22" t="n"/>
-      <c r="BD20" s="23" t="n"/>
+      <c r="B20" s="410" t="n"/>
+      <c r="C20" s="410" t="n"/>
+      <c r="D20" s="410" t="n"/>
+      <c r="E20" s="410" t="n"/>
+      <c r="F20" s="410" t="n"/>
+      <c r="G20" s="410" t="n"/>
+      <c r="H20" s="410" t="n"/>
+      <c r="I20" s="410" t="n"/>
+      <c r="J20" s="410" t="n"/>
+      <c r="K20" s="410" t="n"/>
+      <c r="L20" s="410" t="n"/>
+      <c r="M20" s="410" t="n"/>
+      <c r="N20" s="410" t="n"/>
+      <c r="O20" s="410" t="n"/>
+      <c r="P20" s="410" t="n"/>
+      <c r="Q20" s="410" t="n"/>
+      <c r="R20" s="410" t="n"/>
+      <c r="S20" s="410" t="n"/>
+      <c r="T20" s="410" t="n"/>
+      <c r="U20" s="410" t="n"/>
+      <c r="V20" s="410" t="n"/>
+      <c r="W20" s="410" t="n"/>
+      <c r="X20" s="410" t="n"/>
+      <c r="Y20" s="410" t="n"/>
+      <c r="Z20" s="410" t="n"/>
+      <c r="AA20" s="410" t="n"/>
+      <c r="AB20" s="410" t="n"/>
+      <c r="AC20" s="410" t="n"/>
+      <c r="AD20" s="410" t="n"/>
+      <c r="AE20" s="410" t="n"/>
+      <c r="AF20" s="410" t="n"/>
+      <c r="AG20" s="410" t="n"/>
+      <c r="AH20" s="410" t="n"/>
+      <c r="AI20" s="410" t="n"/>
+      <c r="AJ20" s="410" t="n"/>
+      <c r="AK20" s="410" t="n"/>
+      <c r="AL20" s="410" t="n"/>
+      <c r="AM20" s="410" t="n"/>
+      <c r="AN20" s="410" t="n"/>
+      <c r="AO20" s="410" t="n"/>
+      <c r="AP20" s="410" t="n"/>
+      <c r="AQ20" s="410" t="n"/>
+      <c r="AR20" s="410" t="n"/>
+      <c r="AS20" s="410" t="n"/>
+      <c r="AT20" s="410" t="n"/>
+      <c r="AU20" s="410" t="n"/>
+      <c r="AV20" s="410" t="n"/>
+      <c r="AW20" s="410" t="n"/>
+      <c r="AX20" s="410" t="n"/>
+      <c r="AY20" s="410" t="n"/>
+      <c r="AZ20" s="410" t="n"/>
+      <c r="BA20" s="410" t="n"/>
+      <c r="BB20" s="410" t="n"/>
+      <c r="BC20" s="410" t="n"/>
+      <c r="BD20" s="411" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="18">

</xml_diff>

<commit_message>
Cập nhật portal zoom và layout
</commit_message>
<xml_diff>
--- a/04-Bieu-Mau/01-FRM-100/FRM-101_Master_Document_Register.xlsx
+++ b/04-Bieu-Mau/01-FRM-100/FRM-101_Master_Document_Register.xlsx
@@ -209,7 +209,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="155">
+  <borders count="157">
     <border>
       <left/>
       <right/>
@@ -1887,11 +1887,35 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="000078D4"/>
+      </left>
+      <right style="thin">
+        <color rgb="000078D4"/>
+      </right>
+      <top style="thin">
+        <color rgb="000078D4"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="000078D4"/>
+      </left>
+      <right style="thin">
+        <color rgb="000078D4"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="000078D4"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="412">
+  <cellXfs count="450">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -2989,6 +3013,98 @@
     </xf>
     <xf numFmtId="0" fontId="20" fillId="12" borderId="149" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="119" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="120" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="121" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="135" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="135" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="135" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="135" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="123" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="136" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="136" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="136" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="128" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="34" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="128" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="137" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="128" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="133" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="134" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="128" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="128" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="137" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="128" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="155" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="155" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3071,11 +3187,11 @@
   <oneCellAnchor>
     <from>
       <col>0</col>
-      <colOff>298782</colOff>
-      <row>0</row>
-      <rowOff>275446</rowOff>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
     </from>
-    <ext cx="1394316" cy="402206"/>
+    <ext cx="1552575" cy="438150"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -3089,9 +3205,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3104,11 +3217,11 @@
   <oneCellAnchor>
     <from>
       <col>0</col>
-      <colOff>298782</colOff>
-      <row>0</row>
-      <rowOff>275446</rowOff>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
     </from>
-    <ext cx="1394316" cy="402206"/>
+    <ext cx="1552575" cy="438150"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -3122,9 +3235,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3137,11 +3247,11 @@
   <oneCellAnchor>
     <from>
       <col>0</col>
-      <colOff>298782</colOff>
-      <row>0</row>
-      <rowOff>275446</rowOff>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
     </from>
-    <ext cx="1394316" cy="402206"/>
+    <ext cx="1552575" cy="438150"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -3155,9 +3265,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3170,11 +3277,11 @@
   <oneCellAnchor>
     <from>
       <col>0</col>
-      <colOff>298782</colOff>
-      <row>0</row>
-      <rowOff>275446</rowOff>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
     </from>
-    <ext cx="1394316" cy="402206"/>
+    <ext cx="1552575" cy="438150"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -3188,9 +3295,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3548,7 +3652,7 @@
     <col width="2.33" customWidth="1" min="56" max="56"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1">
+    <row r="1" hidden="1">
       <c r="A1" s="346" t="n"/>
       <c r="B1" s="2" t="n"/>
       <c r="C1" s="2" t="n"/>
@@ -3560,7 +3664,7 @@
       <c r="I1" s="2" t="n"/>
       <c r="J1" s="2" t="n"/>
       <c r="K1" s="3" t="n"/>
-      <c r="L1" s="252" t="inlineStr">
+      <c r="L1" s="448" t="inlineStr">
         <is>
           <t>MASTER DOCUMENT REGISTER</t>
         </is>
@@ -3594,7 +3698,7 @@
       <c r="AM1" s="2" t="n"/>
       <c r="AN1" s="2" t="n"/>
       <c r="AO1" s="2" t="n"/>
-      <c r="AP1" s="2" t="n"/>
+      <c r="AP1" s="3" t="n"/>
       <c r="AQ1" s="347" t="inlineStr">
         <is>
           <t>Form Code</t>
@@ -3619,279 +3723,392 @@
       <c r="BD1" s="3" t="n"/>
     </row>
     <row r="2" ht="15" customHeight="1">
-      <c r="A2" s="10" t="n"/>
-      <c r="K2" s="11" t="n"/>
-      <c r="L2" s="10" t="n"/>
-      <c r="AQ2" s="350" t="inlineStr">
+      <c r="A2" s="412" t="n"/>
+      <c r="B2" s="413" t="n"/>
+      <c r="C2" s="413" t="n"/>
+      <c r="D2" s="413" t="n"/>
+      <c r="E2" s="413" t="n"/>
+      <c r="F2" s="413" t="n"/>
+      <c r="G2" s="413" t="n"/>
+      <c r="H2" s="413" t="n"/>
+      <c r="I2" s="413" t="n"/>
+      <c r="J2" s="413" t="n"/>
+      <c r="K2" s="414" t="n"/>
+      <c r="L2" s="413" t="n"/>
+      <c r="M2" s="413" t="n"/>
+      <c r="N2" s="413" t="n"/>
+      <c r="O2" s="413" t="n"/>
+      <c r="P2" s="413" t="n"/>
+      <c r="Q2" s="413" t="n"/>
+      <c r="R2" s="413" t="n"/>
+      <c r="S2" s="413" t="n"/>
+      <c r="T2" s="413" t="n"/>
+      <c r="U2" s="413" t="n"/>
+      <c r="V2" s="413" t="n"/>
+      <c r="W2" s="413" t="n"/>
+      <c r="X2" s="413" t="n"/>
+      <c r="Y2" s="413" t="n"/>
+      <c r="Z2" s="413" t="n"/>
+      <c r="AA2" s="413" t="n"/>
+      <c r="AB2" s="413" t="n"/>
+      <c r="AC2" s="413" t="n"/>
+      <c r="AD2" s="413" t="n"/>
+      <c r="AE2" s="413" t="n"/>
+      <c r="AF2" s="413" t="n"/>
+      <c r="AG2" s="413" t="n"/>
+      <c r="AH2" s="413" t="n"/>
+      <c r="AI2" s="413" t="n"/>
+      <c r="AJ2" s="413" t="n"/>
+      <c r="AK2" s="413" t="n"/>
+      <c r="AL2" s="413" t="n"/>
+      <c r="AM2" s="413" t="n"/>
+      <c r="AN2" s="413" t="n"/>
+      <c r="AO2" s="413" t="n"/>
+      <c r="AP2" s="414" t="n"/>
+      <c r="AQ2" s="415" t="inlineStr">
         <is>
           <t>Revision</t>
         </is>
       </c>
-      <c r="AR2" s="351" t="n"/>
-      <c r="AS2" s="351" t="n"/>
-      <c r="AT2" s="351" t="n"/>
-      <c r="AU2" s="351" t="n"/>
-      <c r="AV2" s="352" t="n"/>
-      <c r="AW2" s="353" t="inlineStr">
+      <c r="AR2" s="416" t="n"/>
+      <c r="AS2" s="416" t="n"/>
+      <c r="AT2" s="416" t="n"/>
+      <c r="AU2" s="416" t="n"/>
+      <c r="AV2" s="417" t="n"/>
+      <c r="AW2" s="418" t="inlineStr">
         <is>
           <t>V0</t>
         </is>
       </c>
-      <c r="AX2" s="351" t="n"/>
-      <c r="AY2" s="351" t="n"/>
-      <c r="AZ2" s="351" t="n"/>
-      <c r="BA2" s="351" t="n"/>
-      <c r="BB2" s="351" t="n"/>
-      <c r="BC2" s="351" t="n"/>
-      <c r="BD2" s="354" t="n"/>
+      <c r="AX2" s="419" t="n"/>
+      <c r="AY2" s="419" t="n"/>
+      <c r="AZ2" s="419" t="n"/>
+      <c r="BA2" s="419" t="n"/>
+      <c r="BB2" s="419" t="n"/>
+      <c r="BC2" s="419" t="n"/>
+      <c r="BD2" s="420" t="n"/>
     </row>
     <row r="3" ht="15" customHeight="1">
-      <c r="A3" s="10" t="n"/>
-      <c r="K3" s="11" t="n"/>
-      <c r="L3" s="10" t="n"/>
-      <c r="AQ3" s="350" t="inlineStr">
+      <c r="A3" s="421" t="n"/>
+      <c r="B3" s="54" t="n"/>
+      <c r="C3" s="54" t="n"/>
+      <c r="D3" s="54" t="n"/>
+      <c r="E3" s="54" t="n"/>
+      <c r="F3" s="54" t="n"/>
+      <c r="G3" s="54" t="n"/>
+      <c r="H3" s="54" t="n"/>
+      <c r="I3" s="54" t="n"/>
+      <c r="J3" s="54" t="n"/>
+      <c r="K3" s="422" t="n"/>
+      <c r="L3" s="54" t="n"/>
+      <c r="M3" s="54" t="n"/>
+      <c r="N3" s="54" t="n"/>
+      <c r="O3" s="54" t="n"/>
+      <c r="P3" s="54" t="n"/>
+      <c r="Q3" s="54" t="n"/>
+      <c r="R3" s="54" t="n"/>
+      <c r="S3" s="54" t="n"/>
+      <c r="T3" s="54" t="n"/>
+      <c r="U3" s="54" t="n"/>
+      <c r="V3" s="54" t="n"/>
+      <c r="W3" s="54" t="n"/>
+      <c r="X3" s="54" t="n"/>
+      <c r="Y3" s="54" t="n"/>
+      <c r="Z3" s="54" t="n"/>
+      <c r="AA3" s="54" t="n"/>
+      <c r="AB3" s="54" t="n"/>
+      <c r="AC3" s="54" t="n"/>
+      <c r="AD3" s="54" t="n"/>
+      <c r="AE3" s="54" t="n"/>
+      <c r="AF3" s="54" t="n"/>
+      <c r="AG3" s="54" t="n"/>
+      <c r="AH3" s="54" t="n"/>
+      <c r="AI3" s="54" t="n"/>
+      <c r="AJ3" s="54" t="n"/>
+      <c r="AK3" s="54" t="n"/>
+      <c r="AL3" s="54" t="n"/>
+      <c r="AM3" s="54" t="n"/>
+      <c r="AN3" s="54" t="n"/>
+      <c r="AO3" s="54" t="n"/>
+      <c r="AP3" s="422" t="n"/>
+      <c r="AQ3" s="423" t="inlineStr">
         <is>
           <t>Eff. Date</t>
         </is>
       </c>
-      <c r="AR3" s="351" t="n"/>
-      <c r="AS3" s="351" t="n"/>
-      <c r="AT3" s="351" t="n"/>
-      <c r="AU3" s="351" t="n"/>
-      <c r="AV3" s="352" t="n"/>
-      <c r="AW3" s="353" t="inlineStr">
+      <c r="AR3" s="424" t="n"/>
+      <c r="AS3" s="424" t="n"/>
+      <c r="AT3" s="424" t="n"/>
+      <c r="AU3" s="424" t="n"/>
+      <c r="AV3" s="425" t="n"/>
+      <c r="AW3" s="318" t="inlineStr">
         <is>
           <t>YYYY-MM-DD</t>
         </is>
       </c>
-      <c r="AX3" s="351" t="n"/>
-      <c r="AY3" s="351" t="n"/>
-      <c r="AZ3" s="351" t="n"/>
-      <c r="BA3" s="351" t="n"/>
-      <c r="BB3" s="351" t="n"/>
-      <c r="BC3" s="351" t="n"/>
-      <c r="BD3" s="354" t="n"/>
+      <c r="AX3" s="426" t="n"/>
+      <c r="AY3" s="426" t="n"/>
+      <c r="AZ3" s="426" t="n"/>
+      <c r="BA3" s="426" t="n"/>
+      <c r="BB3" s="426" t="n"/>
+      <c r="BC3" s="426" t="n"/>
+      <c r="BD3" s="427" t="n"/>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="10" t="n"/>
-      <c r="K4" s="11" t="n"/>
-      <c r="L4" s="264" t="inlineStr">
+      <c r="A4" s="421" t="n"/>
+      <c r="B4" s="54" t="n"/>
+      <c r="C4" s="54" t="n"/>
+      <c r="D4" s="54" t="n"/>
+      <c r="E4" s="54" t="n"/>
+      <c r="F4" s="54" t="n"/>
+      <c r="G4" s="54" t="n"/>
+      <c r="H4" s="54" t="n"/>
+      <c r="I4" s="54" t="n"/>
+      <c r="J4" s="54" t="n"/>
+      <c r="K4" s="422" t="n"/>
+      <c r="L4" s="428" t="inlineStr">
         <is>
           <t>Quality Management System · Controlled Document</t>
         </is>
       </c>
-      <c r="AQ4" s="350" t="inlineStr">
+      <c r="M4" s="54" t="n"/>
+      <c r="N4" s="54" t="n"/>
+      <c r="O4" s="54" t="n"/>
+      <c r="P4" s="54" t="n"/>
+      <c r="Q4" s="54" t="n"/>
+      <c r="R4" s="54" t="n"/>
+      <c r="S4" s="54" t="n"/>
+      <c r="T4" s="54" t="n"/>
+      <c r="U4" s="54" t="n"/>
+      <c r="V4" s="54" t="n"/>
+      <c r="W4" s="54" t="n"/>
+      <c r="X4" s="54" t="n"/>
+      <c r="Y4" s="54" t="n"/>
+      <c r="Z4" s="54" t="n"/>
+      <c r="AA4" s="54" t="n"/>
+      <c r="AB4" s="54" t="n"/>
+      <c r="AC4" s="54" t="n"/>
+      <c r="AD4" s="54" t="n"/>
+      <c r="AE4" s="54" t="n"/>
+      <c r="AF4" s="54" t="n"/>
+      <c r="AG4" s="54" t="n"/>
+      <c r="AH4" s="54" t="n"/>
+      <c r="AI4" s="54" t="n"/>
+      <c r="AJ4" s="54" t="n"/>
+      <c r="AK4" s="54" t="n"/>
+      <c r="AL4" s="54" t="n"/>
+      <c r="AM4" s="54" t="n"/>
+      <c r="AN4" s="54" t="n"/>
+      <c r="AO4" s="54" t="n"/>
+      <c r="AP4" s="422" t="n"/>
+      <c r="AQ4" s="423" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="AR4" s="351" t="n"/>
-      <c r="AS4" s="351" t="n"/>
-      <c r="AT4" s="351" t="n"/>
-      <c r="AU4" s="351" t="n"/>
-      <c r="AV4" s="352" t="n"/>
-      <c r="AW4" s="353" t="inlineStr">
+      <c r="AR4" s="424" t="n"/>
+      <c r="AS4" s="424" t="n"/>
+      <c r="AT4" s="424" t="n"/>
+      <c r="AU4" s="424" t="n"/>
+      <c r="AV4" s="425" t="n"/>
+      <c r="AW4" s="318" t="inlineStr">
         <is>
           <t>QMS</t>
         </is>
       </c>
-      <c r="AX4" s="351" t="n"/>
-      <c r="AY4" s="351" t="n"/>
-      <c r="AZ4" s="351" t="n"/>
-      <c r="BA4" s="351" t="n"/>
-      <c r="BB4" s="351" t="n"/>
-      <c r="BC4" s="351" t="n"/>
-      <c r="BD4" s="354" t="n"/>
+      <c r="AX4" s="426" t="n"/>
+      <c r="AY4" s="426" t="n"/>
+      <c r="AZ4" s="426" t="n"/>
+      <c r="BA4" s="426" t="n"/>
+      <c r="BB4" s="426" t="n"/>
+      <c r="BC4" s="426" t="n"/>
+      <c r="BD4" s="427" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="16" t="n"/>
-      <c r="B5" s="17" t="n"/>
-      <c r="C5" s="17" t="n"/>
-      <c r="D5" s="17" t="n"/>
-      <c r="E5" s="17" t="n"/>
-      <c r="F5" s="17" t="n"/>
-      <c r="G5" s="17" t="n"/>
-      <c r="H5" s="17" t="n"/>
-      <c r="I5" s="17" t="n"/>
-      <c r="J5" s="17" t="n"/>
-      <c r="K5" s="18" t="n"/>
-      <c r="L5" s="50" t="inlineStr">
+      <c r="A5" s="421" t="n"/>
+      <c r="B5" s="54" t="n"/>
+      <c r="C5" s="54" t="n"/>
+      <c r="D5" s="54" t="n"/>
+      <c r="E5" s="54" t="n"/>
+      <c r="F5" s="54" t="n"/>
+      <c r="G5" s="54" t="n"/>
+      <c r="H5" s="54" t="n"/>
+      <c r="I5" s="54" t="n"/>
+      <c r="J5" s="54" t="n"/>
+      <c r="K5" s="422" t="n"/>
+      <c r="L5" s="429" t="inlineStr">
         <is>
           <t>HESEM Engineering · ISO 9001 / AS9100 · Semiconductor Equipment Parts</t>
         </is>
       </c>
-      <c r="M5" s="17" t="n"/>
-      <c r="N5" s="17" t="n"/>
-      <c r="O5" s="17" t="n"/>
-      <c r="P5" s="17" t="n"/>
-      <c r="Q5" s="17" t="n"/>
-      <c r="R5" s="17" t="n"/>
-      <c r="S5" s="17" t="n"/>
-      <c r="T5" s="17" t="n"/>
-      <c r="U5" s="17" t="n"/>
-      <c r="V5" s="17" t="n"/>
-      <c r="W5" s="17" t="n"/>
-      <c r="X5" s="17" t="n"/>
-      <c r="Y5" s="17" t="n"/>
-      <c r="Z5" s="17" t="n"/>
-      <c r="AA5" s="17" t="n"/>
-      <c r="AB5" s="17" t="n"/>
-      <c r="AC5" s="17" t="n"/>
-      <c r="AD5" s="17" t="n"/>
-      <c r="AE5" s="17" t="n"/>
-      <c r="AF5" s="17" t="n"/>
-      <c r="AG5" s="17" t="n"/>
-      <c r="AH5" s="17" t="n"/>
-      <c r="AI5" s="17" t="n"/>
-      <c r="AJ5" s="17" t="n"/>
-      <c r="AK5" s="17" t="n"/>
-      <c r="AL5" s="17" t="n"/>
-      <c r="AM5" s="17" t="n"/>
-      <c r="AN5" s="17" t="n"/>
-      <c r="AO5" s="17" t="n"/>
-      <c r="AP5" s="17" t="n"/>
-      <c r="AQ5" s="355" t="inlineStr">
+      <c r="M5" s="54" t="n"/>
+      <c r="N5" s="54" t="n"/>
+      <c r="O5" s="54" t="n"/>
+      <c r="P5" s="54" t="n"/>
+      <c r="Q5" s="54" t="n"/>
+      <c r="R5" s="54" t="n"/>
+      <c r="S5" s="54" t="n"/>
+      <c r="T5" s="54" t="n"/>
+      <c r="U5" s="54" t="n"/>
+      <c r="V5" s="54" t="n"/>
+      <c r="W5" s="54" t="n"/>
+      <c r="X5" s="54" t="n"/>
+      <c r="Y5" s="54" t="n"/>
+      <c r="Z5" s="54" t="n"/>
+      <c r="AA5" s="54" t="n"/>
+      <c r="AB5" s="54" t="n"/>
+      <c r="AC5" s="54" t="n"/>
+      <c r="AD5" s="54" t="n"/>
+      <c r="AE5" s="54" t="n"/>
+      <c r="AF5" s="54" t="n"/>
+      <c r="AG5" s="54" t="n"/>
+      <c r="AH5" s="54" t="n"/>
+      <c r="AI5" s="54" t="n"/>
+      <c r="AJ5" s="54" t="n"/>
+      <c r="AK5" s="54" t="n"/>
+      <c r="AL5" s="54" t="n"/>
+      <c r="AM5" s="54" t="n"/>
+      <c r="AN5" s="54" t="n"/>
+      <c r="AO5" s="54" t="n"/>
+      <c r="AP5" s="422" t="n"/>
+      <c r="AQ5" s="423" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="AR5" s="356" t="n"/>
-      <c r="AS5" s="356" t="n"/>
-      <c r="AT5" s="356" t="n"/>
-      <c r="AU5" s="356" t="n"/>
-      <c r="AV5" s="357" t="n"/>
-      <c r="AW5" s="358" t="inlineStr">
+      <c r="AR5" s="424" t="n"/>
+      <c r="AS5" s="424" t="n"/>
+      <c r="AT5" s="424" t="n"/>
+      <c r="AU5" s="424" t="n"/>
+      <c r="AV5" s="425" t="n"/>
+      <c r="AW5" s="318" t="inlineStr">
         <is>
           <t>Per authority matrix</t>
         </is>
       </c>
-      <c r="AX5" s="356" t="n"/>
-      <c r="AY5" s="356" t="n"/>
-      <c r="AZ5" s="356" t="n"/>
-      <c r="BA5" s="356" t="n"/>
-      <c r="BB5" s="356" t="n"/>
-      <c r="BC5" s="356" t="n"/>
-      <c r="BD5" s="359" t="n"/>
+      <c r="AX5" s="426" t="n"/>
+      <c r="AY5" s="426" t="n"/>
+      <c r="AZ5" s="426" t="n"/>
+      <c r="BA5" s="426" t="n"/>
+      <c r="BB5" s="426" t="n"/>
+      <c r="BC5" s="426" t="n"/>
+      <c r="BD5" s="427" t="n"/>
     </row>
-    <row r="6" ht="1.5" customHeight="1">
-      <c r="A6" s="273" t="n"/>
-      <c r="B6" s="273" t="n"/>
-      <c r="C6" s="273" t="n"/>
-      <c r="D6" s="273" t="n"/>
-      <c r="E6" s="273" t="n"/>
-      <c r="F6" s="273" t="n"/>
-      <c r="G6" s="273" t="n"/>
-      <c r="H6" s="273" t="n"/>
-      <c r="I6" s="273" t="n"/>
-      <c r="J6" s="273" t="n"/>
-      <c r="K6" s="273" t="n"/>
-      <c r="L6" s="273" t="n"/>
-      <c r="M6" s="273" t="n"/>
-      <c r="N6" s="273" t="n"/>
-      <c r="O6" s="273" t="n"/>
-      <c r="P6" s="273" t="n"/>
-      <c r="Q6" s="273" t="n"/>
-      <c r="R6" s="273" t="n"/>
-      <c r="S6" s="273" t="n"/>
-      <c r="T6" s="273" t="n"/>
-      <c r="U6" s="273" t="n"/>
-      <c r="V6" s="273" t="n"/>
-      <c r="W6" s="273" t="n"/>
-      <c r="X6" s="273" t="n"/>
-      <c r="Y6" s="273" t="n"/>
-      <c r="Z6" s="273" t="n"/>
-      <c r="AA6" s="273" t="n"/>
-      <c r="AB6" s="273" t="n"/>
-      <c r="AC6" s="273" t="n"/>
-      <c r="AD6" s="273" t="n"/>
-      <c r="AE6" s="273" t="n"/>
-      <c r="AF6" s="273" t="n"/>
-      <c r="AG6" s="273" t="n"/>
-      <c r="AH6" s="273" t="n"/>
-      <c r="AI6" s="273" t="n"/>
-      <c r="AJ6" s="273" t="n"/>
-      <c r="AK6" s="273" t="n"/>
-      <c r="AL6" s="273" t="n"/>
-      <c r="AM6" s="273" t="n"/>
-      <c r="AN6" s="273" t="n"/>
-      <c r="AO6" s="273" t="n"/>
-      <c r="AP6" s="273" t="n"/>
-      <c r="AQ6" s="273" t="n"/>
-      <c r="AR6" s="273" t="n"/>
-      <c r="AS6" s="273" t="n"/>
-      <c r="AT6" s="273" t="n"/>
-      <c r="AU6" s="273" t="n"/>
-      <c r="AV6" s="273" t="n"/>
-      <c r="AW6" s="273" t="n"/>
-      <c r="AX6" s="273" t="n"/>
-      <c r="AY6" s="273" t="n"/>
-      <c r="AZ6" s="273" t="n"/>
-      <c r="BA6" s="273" t="n"/>
-      <c r="BB6" s="273" t="n"/>
-      <c r="BC6" s="273" t="n"/>
-      <c r="BD6" s="273" t="n"/>
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" s="430" t="n"/>
+      <c r="B6" s="431" t="n"/>
+      <c r="C6" s="431" t="n"/>
+      <c r="D6" s="431" t="n"/>
+      <c r="E6" s="431" t="n"/>
+      <c r="F6" s="431" t="n"/>
+      <c r="G6" s="431" t="n"/>
+      <c r="H6" s="431" t="n"/>
+      <c r="I6" s="431" t="n"/>
+      <c r="J6" s="431" t="n"/>
+      <c r="K6" s="432" t="n"/>
+      <c r="L6" s="431" t="n"/>
+      <c r="M6" s="431" t="n"/>
+      <c r="N6" s="431" t="n"/>
+      <c r="O6" s="431" t="n"/>
+      <c r="P6" s="431" t="n"/>
+      <c r="Q6" s="431" t="n"/>
+      <c r="R6" s="431" t="n"/>
+      <c r="S6" s="431" t="n"/>
+      <c r="T6" s="431" t="n"/>
+      <c r="U6" s="431" t="n"/>
+      <c r="V6" s="431" t="n"/>
+      <c r="W6" s="431" t="n"/>
+      <c r="X6" s="431" t="n"/>
+      <c r="Y6" s="431" t="n"/>
+      <c r="Z6" s="431" t="n"/>
+      <c r="AA6" s="431" t="n"/>
+      <c r="AB6" s="431" t="n"/>
+      <c r="AC6" s="431" t="n"/>
+      <c r="AD6" s="431" t="n"/>
+      <c r="AE6" s="431" t="n"/>
+      <c r="AF6" s="431" t="n"/>
+      <c r="AG6" s="431" t="n"/>
+      <c r="AH6" s="431" t="n"/>
+      <c r="AI6" s="431" t="n"/>
+      <c r="AJ6" s="431" t="n"/>
+      <c r="AK6" s="431" t="n"/>
+      <c r="AL6" s="431" t="n"/>
+      <c r="AM6" s="431" t="n"/>
+      <c r="AN6" s="431" t="n"/>
+      <c r="AO6" s="431" t="n"/>
+      <c r="AP6" s="432" t="n"/>
+      <c r="AQ6" s="433" t="n"/>
+      <c r="AR6" s="433" t="n"/>
+      <c r="AS6" s="433" t="n"/>
+      <c r="AT6" s="433" t="n"/>
+      <c r="AU6" s="433" t="n"/>
+      <c r="AV6" s="434" t="n"/>
+      <c r="AW6" s="435" t="n"/>
+      <c r="AX6" s="435" t="n"/>
+      <c r="AY6" s="435" t="n"/>
+      <c r="AZ6" s="435" t="n"/>
+      <c r="BA6" s="435" t="n"/>
+      <c r="BB6" s="435" t="n"/>
+      <c r="BC6" s="435" t="n"/>
+      <c r="BD6" s="436" t="n"/>
     </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="360" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  1. REFERENCE INFORMATION</t>
-        </is>
-      </c>
-      <c r="B7" s="22" t="n"/>
-      <c r="C7" s="22" t="n"/>
-      <c r="D7" s="22" t="n"/>
-      <c r="E7" s="22" t="n"/>
-      <c r="F7" s="22" t="n"/>
-      <c r="G7" s="22" t="n"/>
-      <c r="H7" s="22" t="n"/>
-      <c r="I7" s="22" t="n"/>
-      <c r="J7" s="22" t="n"/>
-      <c r="K7" s="22" t="n"/>
-      <c r="L7" s="22" t="n"/>
-      <c r="M7" s="22" t="n"/>
-      <c r="N7" s="22" t="n"/>
-      <c r="O7" s="22" t="n"/>
-      <c r="P7" s="22" t="n"/>
-      <c r="Q7" s="22" t="n"/>
-      <c r="R7" s="22" t="n"/>
-      <c r="S7" s="22" t="n"/>
-      <c r="T7" s="22" t="n"/>
-      <c r="U7" s="22" t="n"/>
-      <c r="V7" s="22" t="n"/>
-      <c r="W7" s="22" t="n"/>
-      <c r="X7" s="22" t="n"/>
-      <c r="Y7" s="22" t="n"/>
-      <c r="Z7" s="22" t="n"/>
-      <c r="AA7" s="22" t="n"/>
-      <c r="AB7" s="22" t="n"/>
-      <c r="AC7" s="22" t="n"/>
-      <c r="AD7" s="22" t="n"/>
-      <c r="AE7" s="22" t="n"/>
-      <c r="AF7" s="22" t="n"/>
-      <c r="AG7" s="22" t="n"/>
-      <c r="AH7" s="22" t="n"/>
-      <c r="AI7" s="22" t="n"/>
-      <c r="AJ7" s="22" t="n"/>
-      <c r="AK7" s="22" t="n"/>
-      <c r="AL7" s="22" t="n"/>
-      <c r="AM7" s="22" t="n"/>
-      <c r="AN7" s="22" t="n"/>
-      <c r="AO7" s="22" t="n"/>
-      <c r="AP7" s="22" t="n"/>
-      <c r="AQ7" s="22" t="n"/>
-      <c r="AR7" s="22" t="n"/>
-      <c r="AS7" s="22" t="n"/>
-      <c r="AT7" s="22" t="n"/>
-      <c r="AU7" s="22" t="n"/>
-      <c r="AV7" s="22" t="n"/>
-      <c r="AW7" s="22" t="n"/>
-      <c r="AX7" s="22" t="n"/>
-      <c r="AY7" s="22" t="n"/>
-      <c r="AZ7" s="22" t="n"/>
-      <c r="BA7" s="22" t="n"/>
-      <c r="BB7" s="22" t="n"/>
-      <c r="BC7" s="22" t="n"/>
-      <c r="BD7" s="23" t="n"/>
+    <row r="7" ht="4" customHeight="1">
+      <c r="A7" s="437" t="n"/>
+      <c r="B7" s="438" t="n"/>
+      <c r="C7" s="438" t="n"/>
+      <c r="D7" s="438" t="n"/>
+      <c r="E7" s="438" t="n"/>
+      <c r="F7" s="438" t="n"/>
+      <c r="G7" s="438" t="n"/>
+      <c r="H7" s="438" t="n"/>
+      <c r="I7" s="438" t="n"/>
+      <c r="J7" s="438" t="n"/>
+      <c r="K7" s="438" t="n"/>
+      <c r="L7" s="438" t="n"/>
+      <c r="M7" s="438" t="n"/>
+      <c r="N7" s="438" t="n"/>
+      <c r="O7" s="438" t="n"/>
+      <c r="P7" s="438" t="n"/>
+      <c r="Q7" s="438" t="n"/>
+      <c r="R7" s="438" t="n"/>
+      <c r="S7" s="438" t="n"/>
+      <c r="T7" s="438" t="n"/>
+      <c r="U7" s="438" t="n"/>
+      <c r="V7" s="438" t="n"/>
+      <c r="W7" s="438" t="n"/>
+      <c r="X7" s="438" t="n"/>
+      <c r="Y7" s="438" t="n"/>
+      <c r="Z7" s="438" t="n"/>
+      <c r="AA7" s="438" t="n"/>
+      <c r="AB7" s="438" t="n"/>
+      <c r="AC7" s="438" t="n"/>
+      <c r="AD7" s="438" t="n"/>
+      <c r="AE7" s="438" t="n"/>
+      <c r="AF7" s="438" t="n"/>
+      <c r="AG7" s="438" t="n"/>
+      <c r="AH7" s="438" t="n"/>
+      <c r="AI7" s="438" t="n"/>
+      <c r="AJ7" s="438" t="n"/>
+      <c r="AK7" s="438" t="n"/>
+      <c r="AL7" s="438" t="n"/>
+      <c r="AM7" s="438" t="n"/>
+      <c r="AN7" s="438" t="n"/>
+      <c r="AO7" s="438" t="n"/>
+      <c r="AP7" s="438" t="n"/>
+      <c r="AQ7" s="438" t="n"/>
+      <c r="AR7" s="438" t="n"/>
+      <c r="AS7" s="438" t="n"/>
+      <c r="AT7" s="438" t="n"/>
+      <c r="AU7" s="438" t="n"/>
+      <c r="AV7" s="438" t="n"/>
+      <c r="AW7" s="438" t="n"/>
+      <c r="AX7" s="438" t="n"/>
+      <c r="AY7" s="438" t="n"/>
+      <c r="AZ7" s="438" t="n"/>
+      <c r="BA7" s="438" t="n"/>
+      <c r="BB7" s="438" t="n"/>
+      <c r="BC7" s="438" t="n"/>
+      <c r="BD7" s="438" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="361" t="inlineStr">
@@ -5823,66 +6040,66 @@
       <c r="BD37" s="368" t="n"/>
     </row>
     <row r="38" ht="26" customHeight="1">
-      <c r="A38" s="409" t="inlineStr">
+      <c r="A38" s="336" t="inlineStr">
         <is>
           <t>NOTICE: Keep one row per controlled document. Maintain code, revision, status, effective date, storage path and superseded reference so documented information stays traceable and current.</t>
         </is>
       </c>
-      <c r="B38" s="410" t="n"/>
-      <c r="C38" s="410" t="n"/>
-      <c r="D38" s="410" t="n"/>
-      <c r="E38" s="410" t="n"/>
-      <c r="F38" s="410" t="n"/>
-      <c r="G38" s="410" t="n"/>
-      <c r="H38" s="410" t="n"/>
-      <c r="I38" s="410" t="n"/>
-      <c r="J38" s="410" t="n"/>
-      <c r="K38" s="410" t="n"/>
-      <c r="L38" s="410" t="n"/>
-      <c r="M38" s="410" t="n"/>
-      <c r="N38" s="410" t="n"/>
-      <c r="O38" s="410" t="n"/>
-      <c r="P38" s="410" t="n"/>
-      <c r="Q38" s="410" t="n"/>
-      <c r="R38" s="410" t="n"/>
-      <c r="S38" s="410" t="n"/>
-      <c r="T38" s="410" t="n"/>
-      <c r="U38" s="410" t="n"/>
-      <c r="V38" s="410" t="n"/>
-      <c r="W38" s="410" t="n"/>
-      <c r="X38" s="410" t="n"/>
-      <c r="Y38" s="410" t="n"/>
-      <c r="Z38" s="410" t="n"/>
-      <c r="AA38" s="410" t="n"/>
-      <c r="AB38" s="410" t="n"/>
-      <c r="AC38" s="410" t="n"/>
-      <c r="AD38" s="410" t="n"/>
-      <c r="AE38" s="410" t="n"/>
-      <c r="AF38" s="410" t="n"/>
-      <c r="AG38" s="410" t="n"/>
-      <c r="AH38" s="410" t="n"/>
-      <c r="AI38" s="410" t="n"/>
-      <c r="AJ38" s="410" t="n"/>
-      <c r="AK38" s="410" t="n"/>
-      <c r="AL38" s="410" t="n"/>
-      <c r="AM38" s="410" t="n"/>
-      <c r="AN38" s="410" t="n"/>
-      <c r="AO38" s="410" t="n"/>
-      <c r="AP38" s="410" t="n"/>
-      <c r="AQ38" s="410" t="n"/>
-      <c r="AR38" s="410" t="n"/>
-      <c r="AS38" s="410" t="n"/>
-      <c r="AT38" s="410" t="n"/>
-      <c r="AU38" s="410" t="n"/>
-      <c r="AV38" s="410" t="n"/>
-      <c r="AW38" s="410" t="n"/>
-      <c r="AX38" s="410" t="n"/>
-      <c r="AY38" s="410" t="n"/>
-      <c r="AZ38" s="410" t="n"/>
-      <c r="BA38" s="410" t="n"/>
-      <c r="BB38" s="410" t="n"/>
-      <c r="BC38" s="410" t="n"/>
-      <c r="BD38" s="411" t="n"/>
+      <c r="B38" s="439" t="n"/>
+      <c r="C38" s="439" t="n"/>
+      <c r="D38" s="439" t="n"/>
+      <c r="E38" s="439" t="n"/>
+      <c r="F38" s="439" t="n"/>
+      <c r="G38" s="439" t="n"/>
+      <c r="H38" s="439" t="n"/>
+      <c r="I38" s="439" t="n"/>
+      <c r="J38" s="439" t="n"/>
+      <c r="K38" s="439" t="n"/>
+      <c r="L38" s="439" t="n"/>
+      <c r="M38" s="439" t="n"/>
+      <c r="N38" s="439" t="n"/>
+      <c r="O38" s="439" t="n"/>
+      <c r="P38" s="439" t="n"/>
+      <c r="Q38" s="439" t="n"/>
+      <c r="R38" s="439" t="n"/>
+      <c r="S38" s="439" t="n"/>
+      <c r="T38" s="439" t="n"/>
+      <c r="U38" s="439" t="n"/>
+      <c r="V38" s="439" t="n"/>
+      <c r="W38" s="439" t="n"/>
+      <c r="X38" s="439" t="n"/>
+      <c r="Y38" s="439" t="n"/>
+      <c r="Z38" s="439" t="n"/>
+      <c r="AA38" s="439" t="n"/>
+      <c r="AB38" s="439" t="n"/>
+      <c r="AC38" s="439" t="n"/>
+      <c r="AD38" s="439" t="n"/>
+      <c r="AE38" s="439" t="n"/>
+      <c r="AF38" s="439" t="n"/>
+      <c r="AG38" s="439" t="n"/>
+      <c r="AH38" s="439" t="n"/>
+      <c r="AI38" s="439" t="n"/>
+      <c r="AJ38" s="439" t="n"/>
+      <c r="AK38" s="439" t="n"/>
+      <c r="AL38" s="439" t="n"/>
+      <c r="AM38" s="439" t="n"/>
+      <c r="AN38" s="439" t="n"/>
+      <c r="AO38" s="439" t="n"/>
+      <c r="AP38" s="439" t="n"/>
+      <c r="AQ38" s="439" t="n"/>
+      <c r="AR38" s="439" t="n"/>
+      <c r="AS38" s="439" t="n"/>
+      <c r="AT38" s="439" t="n"/>
+      <c r="AU38" s="439" t="n"/>
+      <c r="AV38" s="439" t="n"/>
+      <c r="AW38" s="439" t="n"/>
+      <c r="AX38" s="439" t="n"/>
+      <c r="AY38" s="439" t="n"/>
+      <c r="AZ38" s="439" t="n"/>
+      <c r="BA38" s="439" t="n"/>
+      <c r="BB38" s="439" t="n"/>
+      <c r="BC38" s="439" t="n"/>
+      <c r="BD38" s="440" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
@@ -6252,7 +6469,7 @@
     <col width="2.33" customWidth="1" min="56" max="56"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1">
+    <row r="1" hidden="1">
       <c r="A1" s="346" t="n"/>
       <c r="B1" s="2" t="n"/>
       <c r="C1" s="2" t="n"/>
@@ -6264,7 +6481,7 @@
       <c r="I1" s="2" t="n"/>
       <c r="J1" s="2" t="n"/>
       <c r="K1" s="3" t="n"/>
-      <c r="L1" s="252" t="inlineStr">
+      <c r="L1" s="448" t="inlineStr">
         <is>
           <t>MASTER DOCUMENT REGISTER — REVIEW QUESTIONS / PERIODIC REVIEW</t>
         </is>
@@ -6298,7 +6515,7 @@
       <c r="AM1" s="2" t="n"/>
       <c r="AN1" s="2" t="n"/>
       <c r="AO1" s="2" t="n"/>
-      <c r="AP1" s="2" t="n"/>
+      <c r="AP1" s="3" t="n"/>
       <c r="AQ1" s="347" t="inlineStr">
         <is>
           <t>Form Code</t>
@@ -6323,279 +6540,392 @@
       <c r="BD1" s="3" t="n"/>
     </row>
     <row r="2" ht="15" customHeight="1">
-      <c r="A2" s="10" t="n"/>
-      <c r="K2" s="11" t="n"/>
-      <c r="L2" s="10" t="n"/>
-      <c r="AQ2" s="350" t="inlineStr">
+      <c r="A2" s="412" t="n"/>
+      <c r="B2" s="413" t="n"/>
+      <c r="C2" s="413" t="n"/>
+      <c r="D2" s="413" t="n"/>
+      <c r="E2" s="413" t="n"/>
+      <c r="F2" s="413" t="n"/>
+      <c r="G2" s="413" t="n"/>
+      <c r="H2" s="413" t="n"/>
+      <c r="I2" s="413" t="n"/>
+      <c r="J2" s="413" t="n"/>
+      <c r="K2" s="414" t="n"/>
+      <c r="L2" s="413" t="n"/>
+      <c r="M2" s="413" t="n"/>
+      <c r="N2" s="413" t="n"/>
+      <c r="O2" s="413" t="n"/>
+      <c r="P2" s="413" t="n"/>
+      <c r="Q2" s="413" t="n"/>
+      <c r="R2" s="413" t="n"/>
+      <c r="S2" s="413" t="n"/>
+      <c r="T2" s="413" t="n"/>
+      <c r="U2" s="413" t="n"/>
+      <c r="V2" s="413" t="n"/>
+      <c r="W2" s="413" t="n"/>
+      <c r="X2" s="413" t="n"/>
+      <c r="Y2" s="413" t="n"/>
+      <c r="Z2" s="413" t="n"/>
+      <c r="AA2" s="413" t="n"/>
+      <c r="AB2" s="413" t="n"/>
+      <c r="AC2" s="413" t="n"/>
+      <c r="AD2" s="413" t="n"/>
+      <c r="AE2" s="413" t="n"/>
+      <c r="AF2" s="413" t="n"/>
+      <c r="AG2" s="413" t="n"/>
+      <c r="AH2" s="413" t="n"/>
+      <c r="AI2" s="413" t="n"/>
+      <c r="AJ2" s="413" t="n"/>
+      <c r="AK2" s="413" t="n"/>
+      <c r="AL2" s="413" t="n"/>
+      <c r="AM2" s="413" t="n"/>
+      <c r="AN2" s="413" t="n"/>
+      <c r="AO2" s="413" t="n"/>
+      <c r="AP2" s="414" t="n"/>
+      <c r="AQ2" s="415" t="inlineStr">
         <is>
           <t>Revision</t>
         </is>
       </c>
-      <c r="AR2" s="351" t="n"/>
-      <c r="AS2" s="351" t="n"/>
-      <c r="AT2" s="351" t="n"/>
-      <c r="AU2" s="351" t="n"/>
-      <c r="AV2" s="352" t="n"/>
-      <c r="AW2" s="353" t="inlineStr">
+      <c r="AR2" s="416" t="n"/>
+      <c r="AS2" s="416" t="n"/>
+      <c r="AT2" s="416" t="n"/>
+      <c r="AU2" s="416" t="n"/>
+      <c r="AV2" s="417" t="n"/>
+      <c r="AW2" s="418" t="inlineStr">
         <is>
           <t>V0</t>
         </is>
       </c>
-      <c r="AX2" s="351" t="n"/>
-      <c r="AY2" s="351" t="n"/>
-      <c r="AZ2" s="351" t="n"/>
-      <c r="BA2" s="351" t="n"/>
-      <c r="BB2" s="351" t="n"/>
-      <c r="BC2" s="351" t="n"/>
-      <c r="BD2" s="354" t="n"/>
+      <c r="AX2" s="419" t="n"/>
+      <c r="AY2" s="419" t="n"/>
+      <c r="AZ2" s="419" t="n"/>
+      <c r="BA2" s="419" t="n"/>
+      <c r="BB2" s="419" t="n"/>
+      <c r="BC2" s="419" t="n"/>
+      <c r="BD2" s="420" t="n"/>
     </row>
     <row r="3" ht="15" customHeight="1">
-      <c r="A3" s="10" t="n"/>
-      <c r="K3" s="11" t="n"/>
-      <c r="L3" s="10" t="n"/>
-      <c r="AQ3" s="350" t="inlineStr">
+      <c r="A3" s="421" t="n"/>
+      <c r="B3" s="54" t="n"/>
+      <c r="C3" s="54" t="n"/>
+      <c r="D3" s="54" t="n"/>
+      <c r="E3" s="54" t="n"/>
+      <c r="F3" s="54" t="n"/>
+      <c r="G3" s="54" t="n"/>
+      <c r="H3" s="54" t="n"/>
+      <c r="I3" s="54" t="n"/>
+      <c r="J3" s="54" t="n"/>
+      <c r="K3" s="422" t="n"/>
+      <c r="L3" s="54" t="n"/>
+      <c r="M3" s="54" t="n"/>
+      <c r="N3" s="54" t="n"/>
+      <c r="O3" s="54" t="n"/>
+      <c r="P3" s="54" t="n"/>
+      <c r="Q3" s="54" t="n"/>
+      <c r="R3" s="54" t="n"/>
+      <c r="S3" s="54" t="n"/>
+      <c r="T3" s="54" t="n"/>
+      <c r="U3" s="54" t="n"/>
+      <c r="V3" s="54" t="n"/>
+      <c r="W3" s="54" t="n"/>
+      <c r="X3" s="54" t="n"/>
+      <c r="Y3" s="54" t="n"/>
+      <c r="Z3" s="54" t="n"/>
+      <c r="AA3" s="54" t="n"/>
+      <c r="AB3" s="54" t="n"/>
+      <c r="AC3" s="54" t="n"/>
+      <c r="AD3" s="54" t="n"/>
+      <c r="AE3" s="54" t="n"/>
+      <c r="AF3" s="54" t="n"/>
+      <c r="AG3" s="54" t="n"/>
+      <c r="AH3" s="54" t="n"/>
+      <c r="AI3" s="54" t="n"/>
+      <c r="AJ3" s="54" t="n"/>
+      <c r="AK3" s="54" t="n"/>
+      <c r="AL3" s="54" t="n"/>
+      <c r="AM3" s="54" t="n"/>
+      <c r="AN3" s="54" t="n"/>
+      <c r="AO3" s="54" t="n"/>
+      <c r="AP3" s="422" t="n"/>
+      <c r="AQ3" s="423" t="inlineStr">
         <is>
           <t>Eff. Date</t>
         </is>
       </c>
-      <c r="AR3" s="351" t="n"/>
-      <c r="AS3" s="351" t="n"/>
-      <c r="AT3" s="351" t="n"/>
-      <c r="AU3" s="351" t="n"/>
-      <c r="AV3" s="352" t="n"/>
-      <c r="AW3" s="353" t="inlineStr">
+      <c r="AR3" s="424" t="n"/>
+      <c r="AS3" s="424" t="n"/>
+      <c r="AT3" s="424" t="n"/>
+      <c r="AU3" s="424" t="n"/>
+      <c r="AV3" s="425" t="n"/>
+      <c r="AW3" s="318" t="inlineStr">
         <is>
           <t>YYYY-MM-DD</t>
         </is>
       </c>
-      <c r="AX3" s="351" t="n"/>
-      <c r="AY3" s="351" t="n"/>
-      <c r="AZ3" s="351" t="n"/>
-      <c r="BA3" s="351" t="n"/>
-      <c r="BB3" s="351" t="n"/>
-      <c r="BC3" s="351" t="n"/>
-      <c r="BD3" s="354" t="n"/>
+      <c r="AX3" s="426" t="n"/>
+      <c r="AY3" s="426" t="n"/>
+      <c r="AZ3" s="426" t="n"/>
+      <c r="BA3" s="426" t="n"/>
+      <c r="BB3" s="426" t="n"/>
+      <c r="BC3" s="426" t="n"/>
+      <c r="BD3" s="427" t="n"/>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="10" t="n"/>
-      <c r="K4" s="11" t="n"/>
-      <c r="L4" s="264" t="inlineStr">
+      <c r="A4" s="421" t="n"/>
+      <c r="B4" s="54" t="n"/>
+      <c r="C4" s="54" t="n"/>
+      <c r="D4" s="54" t="n"/>
+      <c r="E4" s="54" t="n"/>
+      <c r="F4" s="54" t="n"/>
+      <c r="G4" s="54" t="n"/>
+      <c r="H4" s="54" t="n"/>
+      <c r="I4" s="54" t="n"/>
+      <c r="J4" s="54" t="n"/>
+      <c r="K4" s="422" t="n"/>
+      <c r="L4" s="428" t="inlineStr">
         <is>
           <t>Quality Management System · Controlled Document</t>
         </is>
       </c>
-      <c r="AQ4" s="350" t="inlineStr">
+      <c r="M4" s="54" t="n"/>
+      <c r="N4" s="54" t="n"/>
+      <c r="O4" s="54" t="n"/>
+      <c r="P4" s="54" t="n"/>
+      <c r="Q4" s="54" t="n"/>
+      <c r="R4" s="54" t="n"/>
+      <c r="S4" s="54" t="n"/>
+      <c r="T4" s="54" t="n"/>
+      <c r="U4" s="54" t="n"/>
+      <c r="V4" s="54" t="n"/>
+      <c r="W4" s="54" t="n"/>
+      <c r="X4" s="54" t="n"/>
+      <c r="Y4" s="54" t="n"/>
+      <c r="Z4" s="54" t="n"/>
+      <c r="AA4" s="54" t="n"/>
+      <c r="AB4" s="54" t="n"/>
+      <c r="AC4" s="54" t="n"/>
+      <c r="AD4" s="54" t="n"/>
+      <c r="AE4" s="54" t="n"/>
+      <c r="AF4" s="54" t="n"/>
+      <c r="AG4" s="54" t="n"/>
+      <c r="AH4" s="54" t="n"/>
+      <c r="AI4" s="54" t="n"/>
+      <c r="AJ4" s="54" t="n"/>
+      <c r="AK4" s="54" t="n"/>
+      <c r="AL4" s="54" t="n"/>
+      <c r="AM4" s="54" t="n"/>
+      <c r="AN4" s="54" t="n"/>
+      <c r="AO4" s="54" t="n"/>
+      <c r="AP4" s="422" t="n"/>
+      <c r="AQ4" s="423" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="AR4" s="351" t="n"/>
-      <c r="AS4" s="351" t="n"/>
-      <c r="AT4" s="351" t="n"/>
-      <c r="AU4" s="351" t="n"/>
-      <c r="AV4" s="352" t="n"/>
-      <c r="AW4" s="353" t="inlineStr">
+      <c r="AR4" s="424" t="n"/>
+      <c r="AS4" s="424" t="n"/>
+      <c r="AT4" s="424" t="n"/>
+      <c r="AU4" s="424" t="n"/>
+      <c r="AV4" s="425" t="n"/>
+      <c r="AW4" s="318" t="inlineStr">
         <is>
           <t>QMS</t>
         </is>
       </c>
-      <c r="AX4" s="351" t="n"/>
-      <c r="AY4" s="351" t="n"/>
-      <c r="AZ4" s="351" t="n"/>
-      <c r="BA4" s="351" t="n"/>
-      <c r="BB4" s="351" t="n"/>
-      <c r="BC4" s="351" t="n"/>
-      <c r="BD4" s="354" t="n"/>
+      <c r="AX4" s="426" t="n"/>
+      <c r="AY4" s="426" t="n"/>
+      <c r="AZ4" s="426" t="n"/>
+      <c r="BA4" s="426" t="n"/>
+      <c r="BB4" s="426" t="n"/>
+      <c r="BC4" s="426" t="n"/>
+      <c r="BD4" s="427" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="16" t="n"/>
-      <c r="B5" s="17" t="n"/>
-      <c r="C5" s="17" t="n"/>
-      <c r="D5" s="17" t="n"/>
-      <c r="E5" s="17" t="n"/>
-      <c r="F5" s="17" t="n"/>
-      <c r="G5" s="17" t="n"/>
-      <c r="H5" s="17" t="n"/>
-      <c r="I5" s="17" t="n"/>
-      <c r="J5" s="17" t="n"/>
-      <c r="K5" s="18" t="n"/>
-      <c r="L5" s="50" t="inlineStr">
+      <c r="A5" s="421" t="n"/>
+      <c r="B5" s="54" t="n"/>
+      <c r="C5" s="54" t="n"/>
+      <c r="D5" s="54" t="n"/>
+      <c r="E5" s="54" t="n"/>
+      <c r="F5" s="54" t="n"/>
+      <c r="G5" s="54" t="n"/>
+      <c r="H5" s="54" t="n"/>
+      <c r="I5" s="54" t="n"/>
+      <c r="J5" s="54" t="n"/>
+      <c r="K5" s="422" t="n"/>
+      <c r="L5" s="429" t="inlineStr">
         <is>
           <t>HESEM Engineering · ISO 9001 / AS9100 · Semiconductor Equipment Parts</t>
         </is>
       </c>
-      <c r="M5" s="17" t="n"/>
-      <c r="N5" s="17" t="n"/>
-      <c r="O5" s="17" t="n"/>
-      <c r="P5" s="17" t="n"/>
-      <c r="Q5" s="17" t="n"/>
-      <c r="R5" s="17" t="n"/>
-      <c r="S5" s="17" t="n"/>
-      <c r="T5" s="17" t="n"/>
-      <c r="U5" s="17" t="n"/>
-      <c r="V5" s="17" t="n"/>
-      <c r="W5" s="17" t="n"/>
-      <c r="X5" s="17" t="n"/>
-      <c r="Y5" s="17" t="n"/>
-      <c r="Z5" s="17" t="n"/>
-      <c r="AA5" s="17" t="n"/>
-      <c r="AB5" s="17" t="n"/>
-      <c r="AC5" s="17" t="n"/>
-      <c r="AD5" s="17" t="n"/>
-      <c r="AE5" s="17" t="n"/>
-      <c r="AF5" s="17" t="n"/>
-      <c r="AG5" s="17" t="n"/>
-      <c r="AH5" s="17" t="n"/>
-      <c r="AI5" s="17" t="n"/>
-      <c r="AJ5" s="17" t="n"/>
-      <c r="AK5" s="17" t="n"/>
-      <c r="AL5" s="17" t="n"/>
-      <c r="AM5" s="17" t="n"/>
-      <c r="AN5" s="17" t="n"/>
-      <c r="AO5" s="17" t="n"/>
-      <c r="AP5" s="17" t="n"/>
-      <c r="AQ5" s="355" t="inlineStr">
+      <c r="M5" s="54" t="n"/>
+      <c r="N5" s="54" t="n"/>
+      <c r="O5" s="54" t="n"/>
+      <c r="P5" s="54" t="n"/>
+      <c r="Q5" s="54" t="n"/>
+      <c r="R5" s="54" t="n"/>
+      <c r="S5" s="54" t="n"/>
+      <c r="T5" s="54" t="n"/>
+      <c r="U5" s="54" t="n"/>
+      <c r="V5" s="54" t="n"/>
+      <c r="W5" s="54" t="n"/>
+      <c r="X5" s="54" t="n"/>
+      <c r="Y5" s="54" t="n"/>
+      <c r="Z5" s="54" t="n"/>
+      <c r="AA5" s="54" t="n"/>
+      <c r="AB5" s="54" t="n"/>
+      <c r="AC5" s="54" t="n"/>
+      <c r="AD5" s="54" t="n"/>
+      <c r="AE5" s="54" t="n"/>
+      <c r="AF5" s="54" t="n"/>
+      <c r="AG5" s="54" t="n"/>
+      <c r="AH5" s="54" t="n"/>
+      <c r="AI5" s="54" t="n"/>
+      <c r="AJ5" s="54" t="n"/>
+      <c r="AK5" s="54" t="n"/>
+      <c r="AL5" s="54" t="n"/>
+      <c r="AM5" s="54" t="n"/>
+      <c r="AN5" s="54" t="n"/>
+      <c r="AO5" s="54" t="n"/>
+      <c r="AP5" s="422" t="n"/>
+      <c r="AQ5" s="423" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="AR5" s="356" t="n"/>
-      <c r="AS5" s="356" t="n"/>
-      <c r="AT5" s="356" t="n"/>
-      <c r="AU5" s="356" t="n"/>
-      <c r="AV5" s="357" t="n"/>
-      <c r="AW5" s="358" t="inlineStr">
+      <c r="AR5" s="424" t="n"/>
+      <c r="AS5" s="424" t="n"/>
+      <c r="AT5" s="424" t="n"/>
+      <c r="AU5" s="424" t="n"/>
+      <c r="AV5" s="425" t="n"/>
+      <c r="AW5" s="318" t="inlineStr">
         <is>
           <t>Per authority matrix</t>
         </is>
       </c>
-      <c r="AX5" s="356" t="n"/>
-      <c r="AY5" s="356" t="n"/>
-      <c r="AZ5" s="356" t="n"/>
-      <c r="BA5" s="356" t="n"/>
-      <c r="BB5" s="356" t="n"/>
-      <c r="BC5" s="356" t="n"/>
-      <c r="BD5" s="359" t="n"/>
+      <c r="AX5" s="426" t="n"/>
+      <c r="AY5" s="426" t="n"/>
+      <c r="AZ5" s="426" t="n"/>
+      <c r="BA5" s="426" t="n"/>
+      <c r="BB5" s="426" t="n"/>
+      <c r="BC5" s="426" t="n"/>
+      <c r="BD5" s="427" t="n"/>
     </row>
-    <row r="6" ht="1.5" customHeight="1">
-      <c r="A6" s="273" t="n"/>
-      <c r="B6" s="273" t="n"/>
-      <c r="C6" s="273" t="n"/>
-      <c r="D6" s="273" t="n"/>
-      <c r="E6" s="273" t="n"/>
-      <c r="F6" s="273" t="n"/>
-      <c r="G6" s="273" t="n"/>
-      <c r="H6" s="273" t="n"/>
-      <c r="I6" s="273" t="n"/>
-      <c r="J6" s="273" t="n"/>
-      <c r="K6" s="273" t="n"/>
-      <c r="L6" s="273" t="n"/>
-      <c r="M6" s="273" t="n"/>
-      <c r="N6" s="273" t="n"/>
-      <c r="O6" s="273" t="n"/>
-      <c r="P6" s="273" t="n"/>
-      <c r="Q6" s="273" t="n"/>
-      <c r="R6" s="273" t="n"/>
-      <c r="S6" s="273" t="n"/>
-      <c r="T6" s="273" t="n"/>
-      <c r="U6" s="273" t="n"/>
-      <c r="V6" s="273" t="n"/>
-      <c r="W6" s="273" t="n"/>
-      <c r="X6" s="273" t="n"/>
-      <c r="Y6" s="273" t="n"/>
-      <c r="Z6" s="273" t="n"/>
-      <c r="AA6" s="273" t="n"/>
-      <c r="AB6" s="273" t="n"/>
-      <c r="AC6" s="273" t="n"/>
-      <c r="AD6" s="273" t="n"/>
-      <c r="AE6" s="273" t="n"/>
-      <c r="AF6" s="273" t="n"/>
-      <c r="AG6" s="273" t="n"/>
-      <c r="AH6" s="273" t="n"/>
-      <c r="AI6" s="273" t="n"/>
-      <c r="AJ6" s="273" t="n"/>
-      <c r="AK6" s="273" t="n"/>
-      <c r="AL6" s="273" t="n"/>
-      <c r="AM6" s="273" t="n"/>
-      <c r="AN6" s="273" t="n"/>
-      <c r="AO6" s="273" t="n"/>
-      <c r="AP6" s="273" t="n"/>
-      <c r="AQ6" s="273" t="n"/>
-      <c r="AR6" s="273" t="n"/>
-      <c r="AS6" s="273" t="n"/>
-      <c r="AT6" s="273" t="n"/>
-      <c r="AU6" s="273" t="n"/>
-      <c r="AV6" s="273" t="n"/>
-      <c r="AW6" s="273" t="n"/>
-      <c r="AX6" s="273" t="n"/>
-      <c r="AY6" s="273" t="n"/>
-      <c r="AZ6" s="273" t="n"/>
-      <c r="BA6" s="273" t="n"/>
-      <c r="BB6" s="273" t="n"/>
-      <c r="BC6" s="273" t="n"/>
-      <c r="BD6" s="273" t="n"/>
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" s="430" t="n"/>
+      <c r="B6" s="431" t="n"/>
+      <c r="C6" s="431" t="n"/>
+      <c r="D6" s="431" t="n"/>
+      <c r="E6" s="431" t="n"/>
+      <c r="F6" s="431" t="n"/>
+      <c r="G6" s="431" t="n"/>
+      <c r="H6" s="431" t="n"/>
+      <c r="I6" s="431" t="n"/>
+      <c r="J6" s="431" t="n"/>
+      <c r="K6" s="432" t="n"/>
+      <c r="L6" s="431" t="n"/>
+      <c r="M6" s="431" t="n"/>
+      <c r="N6" s="431" t="n"/>
+      <c r="O6" s="431" t="n"/>
+      <c r="P6" s="431" t="n"/>
+      <c r="Q6" s="431" t="n"/>
+      <c r="R6" s="431" t="n"/>
+      <c r="S6" s="431" t="n"/>
+      <c r="T6" s="431" t="n"/>
+      <c r="U6" s="431" t="n"/>
+      <c r="V6" s="431" t="n"/>
+      <c r="W6" s="431" t="n"/>
+      <c r="X6" s="431" t="n"/>
+      <c r="Y6" s="431" t="n"/>
+      <c r="Z6" s="431" t="n"/>
+      <c r="AA6" s="431" t="n"/>
+      <c r="AB6" s="431" t="n"/>
+      <c r="AC6" s="431" t="n"/>
+      <c r="AD6" s="431" t="n"/>
+      <c r="AE6" s="431" t="n"/>
+      <c r="AF6" s="431" t="n"/>
+      <c r="AG6" s="431" t="n"/>
+      <c r="AH6" s="431" t="n"/>
+      <c r="AI6" s="431" t="n"/>
+      <c r="AJ6" s="431" t="n"/>
+      <c r="AK6" s="431" t="n"/>
+      <c r="AL6" s="431" t="n"/>
+      <c r="AM6" s="431" t="n"/>
+      <c r="AN6" s="431" t="n"/>
+      <c r="AO6" s="431" t="n"/>
+      <c r="AP6" s="432" t="n"/>
+      <c r="AQ6" s="433" t="n"/>
+      <c r="AR6" s="433" t="n"/>
+      <c r="AS6" s="433" t="n"/>
+      <c r="AT6" s="433" t="n"/>
+      <c r="AU6" s="433" t="n"/>
+      <c r="AV6" s="434" t="n"/>
+      <c r="AW6" s="435" t="n"/>
+      <c r="AX6" s="435" t="n"/>
+      <c r="AY6" s="435" t="n"/>
+      <c r="AZ6" s="435" t="n"/>
+      <c r="BA6" s="435" t="n"/>
+      <c r="BB6" s="435" t="n"/>
+      <c r="BC6" s="435" t="n"/>
+      <c r="BD6" s="436" t="n"/>
     </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="360" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  REFERENCE / SOURCE CONTEXT</t>
-        </is>
-      </c>
-      <c r="B7" s="22" t="n"/>
-      <c r="C7" s="22" t="n"/>
-      <c r="D7" s="22" t="n"/>
-      <c r="E7" s="22" t="n"/>
-      <c r="F7" s="22" t="n"/>
-      <c r="G7" s="22" t="n"/>
-      <c r="H7" s="22" t="n"/>
-      <c r="I7" s="22" t="n"/>
-      <c r="J7" s="22" t="n"/>
-      <c r="K7" s="22" t="n"/>
-      <c r="L7" s="22" t="n"/>
-      <c r="M7" s="22" t="n"/>
-      <c r="N7" s="22" t="n"/>
-      <c r="O7" s="22" t="n"/>
-      <c r="P7" s="22" t="n"/>
-      <c r="Q7" s="22" t="n"/>
-      <c r="R7" s="22" t="n"/>
-      <c r="S7" s="22" t="n"/>
-      <c r="T7" s="22" t="n"/>
-      <c r="U7" s="22" t="n"/>
-      <c r="V7" s="22" t="n"/>
-      <c r="W7" s="22" t="n"/>
-      <c r="X7" s="22" t="n"/>
-      <c r="Y7" s="22" t="n"/>
-      <c r="Z7" s="22" t="n"/>
-      <c r="AA7" s="22" t="n"/>
-      <c r="AB7" s="22" t="n"/>
-      <c r="AC7" s="22" t="n"/>
-      <c r="AD7" s="22" t="n"/>
-      <c r="AE7" s="22" t="n"/>
-      <c r="AF7" s="22" t="n"/>
-      <c r="AG7" s="22" t="n"/>
-      <c r="AH7" s="22" t="n"/>
-      <c r="AI7" s="22" t="n"/>
-      <c r="AJ7" s="22" t="n"/>
-      <c r="AK7" s="22" t="n"/>
-      <c r="AL7" s="22" t="n"/>
-      <c r="AM7" s="22" t="n"/>
-      <c r="AN7" s="22" t="n"/>
-      <c r="AO7" s="22" t="n"/>
-      <c r="AP7" s="22" t="n"/>
-      <c r="AQ7" s="22" t="n"/>
-      <c r="AR7" s="22" t="n"/>
-      <c r="AS7" s="22" t="n"/>
-      <c r="AT7" s="22" t="n"/>
-      <c r="AU7" s="22" t="n"/>
-      <c r="AV7" s="22" t="n"/>
-      <c r="AW7" s="22" t="n"/>
-      <c r="AX7" s="22" t="n"/>
-      <c r="AY7" s="22" t="n"/>
-      <c r="AZ7" s="22" t="n"/>
-      <c r="BA7" s="22" t="n"/>
-      <c r="BB7" s="22" t="n"/>
-      <c r="BC7" s="22" t="n"/>
-      <c r="BD7" s="23" t="n"/>
+    <row r="7" ht="4" customHeight="1">
+      <c r="A7" s="437" t="n"/>
+      <c r="B7" s="438" t="n"/>
+      <c r="C7" s="438" t="n"/>
+      <c r="D7" s="438" t="n"/>
+      <c r="E7" s="438" t="n"/>
+      <c r="F7" s="438" t="n"/>
+      <c r="G7" s="438" t="n"/>
+      <c r="H7" s="438" t="n"/>
+      <c r="I7" s="438" t="n"/>
+      <c r="J7" s="438" t="n"/>
+      <c r="K7" s="438" t="n"/>
+      <c r="L7" s="438" t="n"/>
+      <c r="M7" s="438" t="n"/>
+      <c r="N7" s="438" t="n"/>
+      <c r="O7" s="438" t="n"/>
+      <c r="P7" s="438" t="n"/>
+      <c r="Q7" s="438" t="n"/>
+      <c r="R7" s="438" t="n"/>
+      <c r="S7" s="438" t="n"/>
+      <c r="T7" s="438" t="n"/>
+      <c r="U7" s="438" t="n"/>
+      <c r="V7" s="438" t="n"/>
+      <c r="W7" s="438" t="n"/>
+      <c r="X7" s="438" t="n"/>
+      <c r="Y7" s="438" t="n"/>
+      <c r="Z7" s="438" t="n"/>
+      <c r="AA7" s="438" t="n"/>
+      <c r="AB7" s="438" t="n"/>
+      <c r="AC7" s="438" t="n"/>
+      <c r="AD7" s="438" t="n"/>
+      <c r="AE7" s="438" t="n"/>
+      <c r="AF7" s="438" t="n"/>
+      <c r="AG7" s="438" t="n"/>
+      <c r="AH7" s="438" t="n"/>
+      <c r="AI7" s="438" t="n"/>
+      <c r="AJ7" s="438" t="n"/>
+      <c r="AK7" s="438" t="n"/>
+      <c r="AL7" s="438" t="n"/>
+      <c r="AM7" s="438" t="n"/>
+      <c r="AN7" s="438" t="n"/>
+      <c r="AO7" s="438" t="n"/>
+      <c r="AP7" s="438" t="n"/>
+      <c r="AQ7" s="438" t="n"/>
+      <c r="AR7" s="438" t="n"/>
+      <c r="AS7" s="438" t="n"/>
+      <c r="AT7" s="438" t="n"/>
+      <c r="AU7" s="438" t="n"/>
+      <c r="AV7" s="438" t="n"/>
+      <c r="AW7" s="438" t="n"/>
+      <c r="AX7" s="438" t="n"/>
+      <c r="AY7" s="438" t="n"/>
+      <c r="AZ7" s="438" t="n"/>
+      <c r="BA7" s="438" t="n"/>
+      <c r="BB7" s="438" t="n"/>
+      <c r="BC7" s="438" t="n"/>
+      <c r="BD7" s="438" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="361" t="inlineStr">
@@ -7296,66 +7626,66 @@
       <c r="BD18" s="375" t="n"/>
     </row>
     <row r="19" ht="26" customHeight="1">
-      <c r="A19" s="409" t="inlineStr">
+      <c r="A19" s="336" t="inlineStr">
         <is>
           <t>NOTICE: Keep review questions and periodic review data aligned to the current controlled criteria set; do not embed unofficial rules in this support sheet.</t>
         </is>
       </c>
-      <c r="B19" s="410" t="n"/>
-      <c r="C19" s="410" t="n"/>
-      <c r="D19" s="410" t="n"/>
-      <c r="E19" s="410" t="n"/>
-      <c r="F19" s="410" t="n"/>
-      <c r="G19" s="410" t="n"/>
-      <c r="H19" s="410" t="n"/>
-      <c r="I19" s="410" t="n"/>
-      <c r="J19" s="410" t="n"/>
-      <c r="K19" s="410" t="n"/>
-      <c r="L19" s="410" t="n"/>
-      <c r="M19" s="410" t="n"/>
-      <c r="N19" s="410" t="n"/>
-      <c r="O19" s="410" t="n"/>
-      <c r="P19" s="410" t="n"/>
-      <c r="Q19" s="410" t="n"/>
-      <c r="R19" s="410" t="n"/>
-      <c r="S19" s="410" t="n"/>
-      <c r="T19" s="410" t="n"/>
-      <c r="U19" s="410" t="n"/>
-      <c r="V19" s="410" t="n"/>
-      <c r="W19" s="410" t="n"/>
-      <c r="X19" s="410" t="n"/>
-      <c r="Y19" s="410" t="n"/>
-      <c r="Z19" s="410" t="n"/>
-      <c r="AA19" s="410" t="n"/>
-      <c r="AB19" s="410" t="n"/>
-      <c r="AC19" s="410" t="n"/>
-      <c r="AD19" s="410" t="n"/>
-      <c r="AE19" s="410" t="n"/>
-      <c r="AF19" s="410" t="n"/>
-      <c r="AG19" s="410" t="n"/>
-      <c r="AH19" s="410" t="n"/>
-      <c r="AI19" s="410" t="n"/>
-      <c r="AJ19" s="410" t="n"/>
-      <c r="AK19" s="410" t="n"/>
-      <c r="AL19" s="410" t="n"/>
-      <c r="AM19" s="410" t="n"/>
-      <c r="AN19" s="410" t="n"/>
-      <c r="AO19" s="410" t="n"/>
-      <c r="AP19" s="410" t="n"/>
-      <c r="AQ19" s="410" t="n"/>
-      <c r="AR19" s="410" t="n"/>
-      <c r="AS19" s="410" t="n"/>
-      <c r="AT19" s="410" t="n"/>
-      <c r="AU19" s="410" t="n"/>
-      <c r="AV19" s="410" t="n"/>
-      <c r="AW19" s="410" t="n"/>
-      <c r="AX19" s="410" t="n"/>
-      <c r="AY19" s="410" t="n"/>
-      <c r="AZ19" s="410" t="n"/>
-      <c r="BA19" s="410" t="n"/>
-      <c r="BB19" s="410" t="n"/>
-      <c r="BC19" s="410" t="n"/>
-      <c r="BD19" s="411" t="n"/>
+      <c r="B19" s="439" t="n"/>
+      <c r="C19" s="439" t="n"/>
+      <c r="D19" s="439" t="n"/>
+      <c r="E19" s="439" t="n"/>
+      <c r="F19" s="439" t="n"/>
+      <c r="G19" s="439" t="n"/>
+      <c r="H19" s="439" t="n"/>
+      <c r="I19" s="439" t="n"/>
+      <c r="J19" s="439" t="n"/>
+      <c r="K19" s="439" t="n"/>
+      <c r="L19" s="439" t="n"/>
+      <c r="M19" s="439" t="n"/>
+      <c r="N19" s="439" t="n"/>
+      <c r="O19" s="439" t="n"/>
+      <c r="P19" s="439" t="n"/>
+      <c r="Q19" s="439" t="n"/>
+      <c r="R19" s="439" t="n"/>
+      <c r="S19" s="439" t="n"/>
+      <c r="T19" s="439" t="n"/>
+      <c r="U19" s="439" t="n"/>
+      <c r="V19" s="439" t="n"/>
+      <c r="W19" s="439" t="n"/>
+      <c r="X19" s="439" t="n"/>
+      <c r="Y19" s="439" t="n"/>
+      <c r="Z19" s="439" t="n"/>
+      <c r="AA19" s="439" t="n"/>
+      <c r="AB19" s="439" t="n"/>
+      <c r="AC19" s="439" t="n"/>
+      <c r="AD19" s="439" t="n"/>
+      <c r="AE19" s="439" t="n"/>
+      <c r="AF19" s="439" t="n"/>
+      <c r="AG19" s="439" t="n"/>
+      <c r="AH19" s="439" t="n"/>
+      <c r="AI19" s="439" t="n"/>
+      <c r="AJ19" s="439" t="n"/>
+      <c r="AK19" s="439" t="n"/>
+      <c r="AL19" s="439" t="n"/>
+      <c r="AM19" s="439" t="n"/>
+      <c r="AN19" s="439" t="n"/>
+      <c r="AO19" s="439" t="n"/>
+      <c r="AP19" s="439" t="n"/>
+      <c r="AQ19" s="439" t="n"/>
+      <c r="AR19" s="439" t="n"/>
+      <c r="AS19" s="439" t="n"/>
+      <c r="AT19" s="439" t="n"/>
+      <c r="AU19" s="439" t="n"/>
+      <c r="AV19" s="439" t="n"/>
+      <c r="AW19" s="439" t="n"/>
+      <c r="AX19" s="439" t="n"/>
+      <c r="AY19" s="439" t="n"/>
+      <c r="AZ19" s="439" t="n"/>
+      <c r="BA19" s="439" t="n"/>
+      <c r="BB19" s="439" t="n"/>
+      <c r="BC19" s="439" t="n"/>
+      <c r="BD19" s="440" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
@@ -7536,7 +7866,7 @@
     <col width="2.33" customWidth="1" min="56" max="56"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1">
+    <row r="1" hidden="1">
       <c r="A1" s="346" t="n"/>
       <c r="B1" s="2" t="n"/>
       <c r="C1" s="2" t="n"/>
@@ -7548,7 +7878,7 @@
       <c r="I1" s="2" t="n"/>
       <c r="J1" s="2" t="n"/>
       <c r="K1" s="3" t="n"/>
-      <c r="L1" s="252" t="inlineStr">
+      <c r="L1" s="448" t="inlineStr">
         <is>
           <t>MASTER DOCUMENT REGISTER — EVIDENCE REFERENCE REGISTER</t>
         </is>
@@ -7582,7 +7912,7 @@
       <c r="AM1" s="2" t="n"/>
       <c r="AN1" s="2" t="n"/>
       <c r="AO1" s="2" t="n"/>
-      <c r="AP1" s="2" t="n"/>
+      <c r="AP1" s="3" t="n"/>
       <c r="AQ1" s="347" t="inlineStr">
         <is>
           <t>Form Code</t>
@@ -7607,279 +7937,392 @@
       <c r="BD1" s="3" t="n"/>
     </row>
     <row r="2" ht="15" customHeight="1">
-      <c r="A2" s="10" t="n"/>
-      <c r="K2" s="11" t="n"/>
-      <c r="L2" s="10" t="n"/>
-      <c r="AQ2" s="350" t="inlineStr">
+      <c r="A2" s="412" t="n"/>
+      <c r="B2" s="413" t="n"/>
+      <c r="C2" s="413" t="n"/>
+      <c r="D2" s="413" t="n"/>
+      <c r="E2" s="413" t="n"/>
+      <c r="F2" s="413" t="n"/>
+      <c r="G2" s="413" t="n"/>
+      <c r="H2" s="413" t="n"/>
+      <c r="I2" s="413" t="n"/>
+      <c r="J2" s="413" t="n"/>
+      <c r="K2" s="414" t="n"/>
+      <c r="L2" s="413" t="n"/>
+      <c r="M2" s="413" t="n"/>
+      <c r="N2" s="413" t="n"/>
+      <c r="O2" s="413" t="n"/>
+      <c r="P2" s="413" t="n"/>
+      <c r="Q2" s="413" t="n"/>
+      <c r="R2" s="413" t="n"/>
+      <c r="S2" s="413" t="n"/>
+      <c r="T2" s="413" t="n"/>
+      <c r="U2" s="413" t="n"/>
+      <c r="V2" s="413" t="n"/>
+      <c r="W2" s="413" t="n"/>
+      <c r="X2" s="413" t="n"/>
+      <c r="Y2" s="413" t="n"/>
+      <c r="Z2" s="413" t="n"/>
+      <c r="AA2" s="413" t="n"/>
+      <c r="AB2" s="413" t="n"/>
+      <c r="AC2" s="413" t="n"/>
+      <c r="AD2" s="413" t="n"/>
+      <c r="AE2" s="413" t="n"/>
+      <c r="AF2" s="413" t="n"/>
+      <c r="AG2" s="413" t="n"/>
+      <c r="AH2" s="413" t="n"/>
+      <c r="AI2" s="413" t="n"/>
+      <c r="AJ2" s="413" t="n"/>
+      <c r="AK2" s="413" t="n"/>
+      <c r="AL2" s="413" t="n"/>
+      <c r="AM2" s="413" t="n"/>
+      <c r="AN2" s="413" t="n"/>
+      <c r="AO2" s="413" t="n"/>
+      <c r="AP2" s="414" t="n"/>
+      <c r="AQ2" s="415" t="inlineStr">
         <is>
           <t>Revision</t>
         </is>
       </c>
-      <c r="AR2" s="351" t="n"/>
-      <c r="AS2" s="351" t="n"/>
-      <c r="AT2" s="351" t="n"/>
-      <c r="AU2" s="351" t="n"/>
-      <c r="AV2" s="352" t="n"/>
-      <c r="AW2" s="353" t="inlineStr">
+      <c r="AR2" s="416" t="n"/>
+      <c r="AS2" s="416" t="n"/>
+      <c r="AT2" s="416" t="n"/>
+      <c r="AU2" s="416" t="n"/>
+      <c r="AV2" s="417" t="n"/>
+      <c r="AW2" s="418" t="inlineStr">
         <is>
           <t>V0</t>
         </is>
       </c>
-      <c r="AX2" s="351" t="n"/>
-      <c r="AY2" s="351" t="n"/>
-      <c r="AZ2" s="351" t="n"/>
-      <c r="BA2" s="351" t="n"/>
-      <c r="BB2" s="351" t="n"/>
-      <c r="BC2" s="351" t="n"/>
-      <c r="BD2" s="354" t="n"/>
+      <c r="AX2" s="419" t="n"/>
+      <c r="AY2" s="419" t="n"/>
+      <c r="AZ2" s="419" t="n"/>
+      <c r="BA2" s="419" t="n"/>
+      <c r="BB2" s="419" t="n"/>
+      <c r="BC2" s="419" t="n"/>
+      <c r="BD2" s="420" t="n"/>
     </row>
     <row r="3" ht="15" customHeight="1">
-      <c r="A3" s="10" t="n"/>
-      <c r="K3" s="11" t="n"/>
-      <c r="L3" s="10" t="n"/>
-      <c r="AQ3" s="350" t="inlineStr">
+      <c r="A3" s="421" t="n"/>
+      <c r="B3" s="54" t="n"/>
+      <c r="C3" s="54" t="n"/>
+      <c r="D3" s="54" t="n"/>
+      <c r="E3" s="54" t="n"/>
+      <c r="F3" s="54" t="n"/>
+      <c r="G3" s="54" t="n"/>
+      <c r="H3" s="54" t="n"/>
+      <c r="I3" s="54" t="n"/>
+      <c r="J3" s="54" t="n"/>
+      <c r="K3" s="422" t="n"/>
+      <c r="L3" s="54" t="n"/>
+      <c r="M3" s="54" t="n"/>
+      <c r="N3" s="54" t="n"/>
+      <c r="O3" s="54" t="n"/>
+      <c r="P3" s="54" t="n"/>
+      <c r="Q3" s="54" t="n"/>
+      <c r="R3" s="54" t="n"/>
+      <c r="S3" s="54" t="n"/>
+      <c r="T3" s="54" t="n"/>
+      <c r="U3" s="54" t="n"/>
+      <c r="V3" s="54" t="n"/>
+      <c r="W3" s="54" t="n"/>
+      <c r="X3" s="54" t="n"/>
+      <c r="Y3" s="54" t="n"/>
+      <c r="Z3" s="54" t="n"/>
+      <c r="AA3" s="54" t="n"/>
+      <c r="AB3" s="54" t="n"/>
+      <c r="AC3" s="54" t="n"/>
+      <c r="AD3" s="54" t="n"/>
+      <c r="AE3" s="54" t="n"/>
+      <c r="AF3" s="54" t="n"/>
+      <c r="AG3" s="54" t="n"/>
+      <c r="AH3" s="54" t="n"/>
+      <c r="AI3" s="54" t="n"/>
+      <c r="AJ3" s="54" t="n"/>
+      <c r="AK3" s="54" t="n"/>
+      <c r="AL3" s="54" t="n"/>
+      <c r="AM3" s="54" t="n"/>
+      <c r="AN3" s="54" t="n"/>
+      <c r="AO3" s="54" t="n"/>
+      <c r="AP3" s="422" t="n"/>
+      <c r="AQ3" s="423" t="inlineStr">
         <is>
           <t>Eff. Date</t>
         </is>
       </c>
-      <c r="AR3" s="351" t="n"/>
-      <c r="AS3" s="351" t="n"/>
-      <c r="AT3" s="351" t="n"/>
-      <c r="AU3" s="351" t="n"/>
-      <c r="AV3" s="352" t="n"/>
-      <c r="AW3" s="353" t="inlineStr">
+      <c r="AR3" s="424" t="n"/>
+      <c r="AS3" s="424" t="n"/>
+      <c r="AT3" s="424" t="n"/>
+      <c r="AU3" s="424" t="n"/>
+      <c r="AV3" s="425" t="n"/>
+      <c r="AW3" s="318" t="inlineStr">
         <is>
           <t>YYYY-MM-DD</t>
         </is>
       </c>
-      <c r="AX3" s="351" t="n"/>
-      <c r="AY3" s="351" t="n"/>
-      <c r="AZ3" s="351" t="n"/>
-      <c r="BA3" s="351" t="n"/>
-      <c r="BB3" s="351" t="n"/>
-      <c r="BC3" s="351" t="n"/>
-      <c r="BD3" s="354" t="n"/>
+      <c r="AX3" s="426" t="n"/>
+      <c r="AY3" s="426" t="n"/>
+      <c r="AZ3" s="426" t="n"/>
+      <c r="BA3" s="426" t="n"/>
+      <c r="BB3" s="426" t="n"/>
+      <c r="BC3" s="426" t="n"/>
+      <c r="BD3" s="427" t="n"/>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="10" t="n"/>
-      <c r="K4" s="11" t="n"/>
-      <c r="L4" s="264" t="inlineStr">
+      <c r="A4" s="421" t="n"/>
+      <c r="B4" s="54" t="n"/>
+      <c r="C4" s="54" t="n"/>
+      <c r="D4" s="54" t="n"/>
+      <c r="E4" s="54" t="n"/>
+      <c r="F4" s="54" t="n"/>
+      <c r="G4" s="54" t="n"/>
+      <c r="H4" s="54" t="n"/>
+      <c r="I4" s="54" t="n"/>
+      <c r="J4" s="54" t="n"/>
+      <c r="K4" s="422" t="n"/>
+      <c r="L4" s="428" t="inlineStr">
         <is>
           <t>Quality Management System · Controlled Document</t>
         </is>
       </c>
-      <c r="AQ4" s="350" t="inlineStr">
+      <c r="M4" s="54" t="n"/>
+      <c r="N4" s="54" t="n"/>
+      <c r="O4" s="54" t="n"/>
+      <c r="P4" s="54" t="n"/>
+      <c r="Q4" s="54" t="n"/>
+      <c r="R4" s="54" t="n"/>
+      <c r="S4" s="54" t="n"/>
+      <c r="T4" s="54" t="n"/>
+      <c r="U4" s="54" t="n"/>
+      <c r="V4" s="54" t="n"/>
+      <c r="W4" s="54" t="n"/>
+      <c r="X4" s="54" t="n"/>
+      <c r="Y4" s="54" t="n"/>
+      <c r="Z4" s="54" t="n"/>
+      <c r="AA4" s="54" t="n"/>
+      <c r="AB4" s="54" t="n"/>
+      <c r="AC4" s="54" t="n"/>
+      <c r="AD4" s="54" t="n"/>
+      <c r="AE4" s="54" t="n"/>
+      <c r="AF4" s="54" t="n"/>
+      <c r="AG4" s="54" t="n"/>
+      <c r="AH4" s="54" t="n"/>
+      <c r="AI4" s="54" t="n"/>
+      <c r="AJ4" s="54" t="n"/>
+      <c r="AK4" s="54" t="n"/>
+      <c r="AL4" s="54" t="n"/>
+      <c r="AM4" s="54" t="n"/>
+      <c r="AN4" s="54" t="n"/>
+      <c r="AO4" s="54" t="n"/>
+      <c r="AP4" s="422" t="n"/>
+      <c r="AQ4" s="423" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="AR4" s="351" t="n"/>
-      <c r="AS4" s="351" t="n"/>
-      <c r="AT4" s="351" t="n"/>
-      <c r="AU4" s="351" t="n"/>
-      <c r="AV4" s="352" t="n"/>
-      <c r="AW4" s="353" t="inlineStr">
+      <c r="AR4" s="424" t="n"/>
+      <c r="AS4" s="424" t="n"/>
+      <c r="AT4" s="424" t="n"/>
+      <c r="AU4" s="424" t="n"/>
+      <c r="AV4" s="425" t="n"/>
+      <c r="AW4" s="318" t="inlineStr">
         <is>
           <t>QMS</t>
         </is>
       </c>
-      <c r="AX4" s="351" t="n"/>
-      <c r="AY4" s="351" t="n"/>
-      <c r="AZ4" s="351" t="n"/>
-      <c r="BA4" s="351" t="n"/>
-      <c r="BB4" s="351" t="n"/>
-      <c r="BC4" s="351" t="n"/>
-      <c r="BD4" s="354" t="n"/>
+      <c r="AX4" s="426" t="n"/>
+      <c r="AY4" s="426" t="n"/>
+      <c r="AZ4" s="426" t="n"/>
+      <c r="BA4" s="426" t="n"/>
+      <c r="BB4" s="426" t="n"/>
+      <c r="BC4" s="426" t="n"/>
+      <c r="BD4" s="427" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="16" t="n"/>
-      <c r="B5" s="17" t="n"/>
-      <c r="C5" s="17" t="n"/>
-      <c r="D5" s="17" t="n"/>
-      <c r="E5" s="17" t="n"/>
-      <c r="F5" s="17" t="n"/>
-      <c r="G5" s="17" t="n"/>
-      <c r="H5" s="17" t="n"/>
-      <c r="I5" s="17" t="n"/>
-      <c r="J5" s="17" t="n"/>
-      <c r="K5" s="18" t="n"/>
-      <c r="L5" s="50" t="inlineStr">
+      <c r="A5" s="421" t="n"/>
+      <c r="B5" s="54" t="n"/>
+      <c r="C5" s="54" t="n"/>
+      <c r="D5" s="54" t="n"/>
+      <c r="E5" s="54" t="n"/>
+      <c r="F5" s="54" t="n"/>
+      <c r="G5" s="54" t="n"/>
+      <c r="H5" s="54" t="n"/>
+      <c r="I5" s="54" t="n"/>
+      <c r="J5" s="54" t="n"/>
+      <c r="K5" s="422" t="n"/>
+      <c r="L5" s="429" t="inlineStr">
         <is>
           <t>HESEM Engineering · ISO 9001 / AS9100 · Semiconductor Equipment Parts</t>
         </is>
       </c>
-      <c r="M5" s="17" t="n"/>
-      <c r="N5" s="17" t="n"/>
-      <c r="O5" s="17" t="n"/>
-      <c r="P5" s="17" t="n"/>
-      <c r="Q5" s="17" t="n"/>
-      <c r="R5" s="17" t="n"/>
-      <c r="S5" s="17" t="n"/>
-      <c r="T5" s="17" t="n"/>
-      <c r="U5" s="17" t="n"/>
-      <c r="V5" s="17" t="n"/>
-      <c r="W5" s="17" t="n"/>
-      <c r="X5" s="17" t="n"/>
-      <c r="Y5" s="17" t="n"/>
-      <c r="Z5" s="17" t="n"/>
-      <c r="AA5" s="17" t="n"/>
-      <c r="AB5" s="17" t="n"/>
-      <c r="AC5" s="17" t="n"/>
-      <c r="AD5" s="17" t="n"/>
-      <c r="AE5" s="17" t="n"/>
-      <c r="AF5" s="17" t="n"/>
-      <c r="AG5" s="17" t="n"/>
-      <c r="AH5" s="17" t="n"/>
-      <c r="AI5" s="17" t="n"/>
-      <c r="AJ5" s="17" t="n"/>
-      <c r="AK5" s="17" t="n"/>
-      <c r="AL5" s="17" t="n"/>
-      <c r="AM5" s="17" t="n"/>
-      <c r="AN5" s="17" t="n"/>
-      <c r="AO5" s="17" t="n"/>
-      <c r="AP5" s="17" t="n"/>
-      <c r="AQ5" s="355" t="inlineStr">
+      <c r="M5" s="54" t="n"/>
+      <c r="N5" s="54" t="n"/>
+      <c r="O5" s="54" t="n"/>
+      <c r="P5" s="54" t="n"/>
+      <c r="Q5" s="54" t="n"/>
+      <c r="R5" s="54" t="n"/>
+      <c r="S5" s="54" t="n"/>
+      <c r="T5" s="54" t="n"/>
+      <c r="U5" s="54" t="n"/>
+      <c r="V5" s="54" t="n"/>
+      <c r="W5" s="54" t="n"/>
+      <c r="X5" s="54" t="n"/>
+      <c r="Y5" s="54" t="n"/>
+      <c r="Z5" s="54" t="n"/>
+      <c r="AA5" s="54" t="n"/>
+      <c r="AB5" s="54" t="n"/>
+      <c r="AC5" s="54" t="n"/>
+      <c r="AD5" s="54" t="n"/>
+      <c r="AE5" s="54" t="n"/>
+      <c r="AF5" s="54" t="n"/>
+      <c r="AG5" s="54" t="n"/>
+      <c r="AH5" s="54" t="n"/>
+      <c r="AI5" s="54" t="n"/>
+      <c r="AJ5" s="54" t="n"/>
+      <c r="AK5" s="54" t="n"/>
+      <c r="AL5" s="54" t="n"/>
+      <c r="AM5" s="54" t="n"/>
+      <c r="AN5" s="54" t="n"/>
+      <c r="AO5" s="54" t="n"/>
+      <c r="AP5" s="422" t="n"/>
+      <c r="AQ5" s="423" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="AR5" s="356" t="n"/>
-      <c r="AS5" s="356" t="n"/>
-      <c r="AT5" s="356" t="n"/>
-      <c r="AU5" s="356" t="n"/>
-      <c r="AV5" s="357" t="n"/>
-      <c r="AW5" s="358" t="inlineStr">
+      <c r="AR5" s="424" t="n"/>
+      <c r="AS5" s="424" t="n"/>
+      <c r="AT5" s="424" t="n"/>
+      <c r="AU5" s="424" t="n"/>
+      <c r="AV5" s="425" t="n"/>
+      <c r="AW5" s="318" t="inlineStr">
         <is>
           <t>Per authority matrix</t>
         </is>
       </c>
-      <c r="AX5" s="356" t="n"/>
-      <c r="AY5" s="356" t="n"/>
-      <c r="AZ5" s="356" t="n"/>
-      <c r="BA5" s="356" t="n"/>
-      <c r="BB5" s="356" t="n"/>
-      <c r="BC5" s="356" t="n"/>
-      <c r="BD5" s="359" t="n"/>
+      <c r="AX5" s="426" t="n"/>
+      <c r="AY5" s="426" t="n"/>
+      <c r="AZ5" s="426" t="n"/>
+      <c r="BA5" s="426" t="n"/>
+      <c r="BB5" s="426" t="n"/>
+      <c r="BC5" s="426" t="n"/>
+      <c r="BD5" s="427" t="n"/>
     </row>
-    <row r="6" ht="1.5" customHeight="1">
-      <c r="A6" s="273" t="n"/>
-      <c r="B6" s="273" t="n"/>
-      <c r="C6" s="273" t="n"/>
-      <c r="D6" s="273" t="n"/>
-      <c r="E6" s="273" t="n"/>
-      <c r="F6" s="273" t="n"/>
-      <c r="G6" s="273" t="n"/>
-      <c r="H6" s="273" t="n"/>
-      <c r="I6" s="273" t="n"/>
-      <c r="J6" s="273" t="n"/>
-      <c r="K6" s="273" t="n"/>
-      <c r="L6" s="273" t="n"/>
-      <c r="M6" s="273" t="n"/>
-      <c r="N6" s="273" t="n"/>
-      <c r="O6" s="273" t="n"/>
-      <c r="P6" s="273" t="n"/>
-      <c r="Q6" s="273" t="n"/>
-      <c r="R6" s="273" t="n"/>
-      <c r="S6" s="273" t="n"/>
-      <c r="T6" s="273" t="n"/>
-      <c r="U6" s="273" t="n"/>
-      <c r="V6" s="273" t="n"/>
-      <c r="W6" s="273" t="n"/>
-      <c r="X6" s="273" t="n"/>
-      <c r="Y6" s="273" t="n"/>
-      <c r="Z6" s="273" t="n"/>
-      <c r="AA6" s="273" t="n"/>
-      <c r="AB6" s="273" t="n"/>
-      <c r="AC6" s="273" t="n"/>
-      <c r="AD6" s="273" t="n"/>
-      <c r="AE6" s="273" t="n"/>
-      <c r="AF6" s="273" t="n"/>
-      <c r="AG6" s="273" t="n"/>
-      <c r="AH6" s="273" t="n"/>
-      <c r="AI6" s="273" t="n"/>
-      <c r="AJ6" s="273" t="n"/>
-      <c r="AK6" s="273" t="n"/>
-      <c r="AL6" s="273" t="n"/>
-      <c r="AM6" s="273" t="n"/>
-      <c r="AN6" s="273" t="n"/>
-      <c r="AO6" s="273" t="n"/>
-      <c r="AP6" s="273" t="n"/>
-      <c r="AQ6" s="273" t="n"/>
-      <c r="AR6" s="273" t="n"/>
-      <c r="AS6" s="273" t="n"/>
-      <c r="AT6" s="273" t="n"/>
-      <c r="AU6" s="273" t="n"/>
-      <c r="AV6" s="273" t="n"/>
-      <c r="AW6" s="273" t="n"/>
-      <c r="AX6" s="273" t="n"/>
-      <c r="AY6" s="273" t="n"/>
-      <c r="AZ6" s="273" t="n"/>
-      <c r="BA6" s="273" t="n"/>
-      <c r="BB6" s="273" t="n"/>
-      <c r="BC6" s="273" t="n"/>
-      <c r="BD6" s="273" t="n"/>
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" s="430" t="n"/>
+      <c r="B6" s="431" t="n"/>
+      <c r="C6" s="431" t="n"/>
+      <c r="D6" s="431" t="n"/>
+      <c r="E6" s="431" t="n"/>
+      <c r="F6" s="431" t="n"/>
+      <c r="G6" s="431" t="n"/>
+      <c r="H6" s="431" t="n"/>
+      <c r="I6" s="431" t="n"/>
+      <c r="J6" s="431" t="n"/>
+      <c r="K6" s="432" t="n"/>
+      <c r="L6" s="431" t="n"/>
+      <c r="M6" s="431" t="n"/>
+      <c r="N6" s="431" t="n"/>
+      <c r="O6" s="431" t="n"/>
+      <c r="P6" s="431" t="n"/>
+      <c r="Q6" s="431" t="n"/>
+      <c r="R6" s="431" t="n"/>
+      <c r="S6" s="431" t="n"/>
+      <c r="T6" s="431" t="n"/>
+      <c r="U6" s="431" t="n"/>
+      <c r="V6" s="431" t="n"/>
+      <c r="W6" s="431" t="n"/>
+      <c r="X6" s="431" t="n"/>
+      <c r="Y6" s="431" t="n"/>
+      <c r="Z6" s="431" t="n"/>
+      <c r="AA6" s="431" t="n"/>
+      <c r="AB6" s="431" t="n"/>
+      <c r="AC6" s="431" t="n"/>
+      <c r="AD6" s="431" t="n"/>
+      <c r="AE6" s="431" t="n"/>
+      <c r="AF6" s="431" t="n"/>
+      <c r="AG6" s="431" t="n"/>
+      <c r="AH6" s="431" t="n"/>
+      <c r="AI6" s="431" t="n"/>
+      <c r="AJ6" s="431" t="n"/>
+      <c r="AK6" s="431" t="n"/>
+      <c r="AL6" s="431" t="n"/>
+      <c r="AM6" s="431" t="n"/>
+      <c r="AN6" s="431" t="n"/>
+      <c r="AO6" s="431" t="n"/>
+      <c r="AP6" s="432" t="n"/>
+      <c r="AQ6" s="433" t="n"/>
+      <c r="AR6" s="433" t="n"/>
+      <c r="AS6" s="433" t="n"/>
+      <c r="AT6" s="433" t="n"/>
+      <c r="AU6" s="433" t="n"/>
+      <c r="AV6" s="434" t="n"/>
+      <c r="AW6" s="435" t="n"/>
+      <c r="AX6" s="435" t="n"/>
+      <c r="AY6" s="435" t="n"/>
+      <c r="AZ6" s="435" t="n"/>
+      <c r="BA6" s="435" t="n"/>
+      <c r="BB6" s="435" t="n"/>
+      <c r="BC6" s="435" t="n"/>
+      <c r="BD6" s="436" t="n"/>
     </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="360" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  REFERENCE / SOURCE CONTEXT</t>
-        </is>
-      </c>
-      <c r="B7" s="22" t="n"/>
-      <c r="C7" s="22" t="n"/>
-      <c r="D7" s="22" t="n"/>
-      <c r="E7" s="22" t="n"/>
-      <c r="F7" s="22" t="n"/>
-      <c r="G7" s="22" t="n"/>
-      <c r="H7" s="22" t="n"/>
-      <c r="I7" s="22" t="n"/>
-      <c r="J7" s="22" t="n"/>
-      <c r="K7" s="22" t="n"/>
-      <c r="L7" s="22" t="n"/>
-      <c r="M7" s="22" t="n"/>
-      <c r="N7" s="22" t="n"/>
-      <c r="O7" s="22" t="n"/>
-      <c r="P7" s="22" t="n"/>
-      <c r="Q7" s="22" t="n"/>
-      <c r="R7" s="22" t="n"/>
-      <c r="S7" s="22" t="n"/>
-      <c r="T7" s="22" t="n"/>
-      <c r="U7" s="22" t="n"/>
-      <c r="V7" s="22" t="n"/>
-      <c r="W7" s="22" t="n"/>
-      <c r="X7" s="22" t="n"/>
-      <c r="Y7" s="22" t="n"/>
-      <c r="Z7" s="22" t="n"/>
-      <c r="AA7" s="22" t="n"/>
-      <c r="AB7" s="22" t="n"/>
-      <c r="AC7" s="22" t="n"/>
-      <c r="AD7" s="22" t="n"/>
-      <c r="AE7" s="22" t="n"/>
-      <c r="AF7" s="22" t="n"/>
-      <c r="AG7" s="22" t="n"/>
-      <c r="AH7" s="22" t="n"/>
-      <c r="AI7" s="22" t="n"/>
-      <c r="AJ7" s="22" t="n"/>
-      <c r="AK7" s="22" t="n"/>
-      <c r="AL7" s="22" t="n"/>
-      <c r="AM7" s="22" t="n"/>
-      <c r="AN7" s="22" t="n"/>
-      <c r="AO7" s="22" t="n"/>
-      <c r="AP7" s="22" t="n"/>
-      <c r="AQ7" s="22" t="n"/>
-      <c r="AR7" s="22" t="n"/>
-      <c r="AS7" s="22" t="n"/>
-      <c r="AT7" s="22" t="n"/>
-      <c r="AU7" s="22" t="n"/>
-      <c r="AV7" s="22" t="n"/>
-      <c r="AW7" s="22" t="n"/>
-      <c r="AX7" s="22" t="n"/>
-      <c r="AY7" s="22" t="n"/>
-      <c r="AZ7" s="22" t="n"/>
-      <c r="BA7" s="22" t="n"/>
-      <c r="BB7" s="22" t="n"/>
-      <c r="BC7" s="22" t="n"/>
-      <c r="BD7" s="23" t="n"/>
+    <row r="7" ht="4" customHeight="1">
+      <c r="A7" s="437" t="n"/>
+      <c r="B7" s="438" t="n"/>
+      <c r="C7" s="438" t="n"/>
+      <c r="D7" s="438" t="n"/>
+      <c r="E7" s="438" t="n"/>
+      <c r="F7" s="438" t="n"/>
+      <c r="G7" s="438" t="n"/>
+      <c r="H7" s="438" t="n"/>
+      <c r="I7" s="438" t="n"/>
+      <c r="J7" s="438" t="n"/>
+      <c r="K7" s="438" t="n"/>
+      <c r="L7" s="438" t="n"/>
+      <c r="M7" s="438" t="n"/>
+      <c r="N7" s="438" t="n"/>
+      <c r="O7" s="438" t="n"/>
+      <c r="P7" s="438" t="n"/>
+      <c r="Q7" s="438" t="n"/>
+      <c r="R7" s="438" t="n"/>
+      <c r="S7" s="438" t="n"/>
+      <c r="T7" s="438" t="n"/>
+      <c r="U7" s="438" t="n"/>
+      <c r="V7" s="438" t="n"/>
+      <c r="W7" s="438" t="n"/>
+      <c r="X7" s="438" t="n"/>
+      <c r="Y7" s="438" t="n"/>
+      <c r="Z7" s="438" t="n"/>
+      <c r="AA7" s="438" t="n"/>
+      <c r="AB7" s="438" t="n"/>
+      <c r="AC7" s="438" t="n"/>
+      <c r="AD7" s="438" t="n"/>
+      <c r="AE7" s="438" t="n"/>
+      <c r="AF7" s="438" t="n"/>
+      <c r="AG7" s="438" t="n"/>
+      <c r="AH7" s="438" t="n"/>
+      <c r="AI7" s="438" t="n"/>
+      <c r="AJ7" s="438" t="n"/>
+      <c r="AK7" s="438" t="n"/>
+      <c r="AL7" s="438" t="n"/>
+      <c r="AM7" s="438" t="n"/>
+      <c r="AN7" s="438" t="n"/>
+      <c r="AO7" s="438" t="n"/>
+      <c r="AP7" s="438" t="n"/>
+      <c r="AQ7" s="438" t="n"/>
+      <c r="AR7" s="438" t="n"/>
+      <c r="AS7" s="438" t="n"/>
+      <c r="AT7" s="438" t="n"/>
+      <c r="AU7" s="438" t="n"/>
+      <c r="AV7" s="438" t="n"/>
+      <c r="AW7" s="438" t="n"/>
+      <c r="AX7" s="438" t="n"/>
+      <c r="AY7" s="438" t="n"/>
+      <c r="AZ7" s="438" t="n"/>
+      <c r="BA7" s="438" t="n"/>
+      <c r="BB7" s="438" t="n"/>
+      <c r="BC7" s="438" t="n"/>
+      <c r="BD7" s="438" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="361" t="inlineStr">
@@ -8514,66 +8957,66 @@
       <c r="BD17" s="375" t="n"/>
     </row>
     <row r="18" ht="26" customHeight="1">
-      <c r="A18" s="409" t="inlineStr">
+      <c r="A18" s="336" t="inlineStr">
         <is>
           <t>NOTICE: Reference evidence by owner, date and source path only; do not duplicate system-owned master records in this support sheet.</t>
         </is>
       </c>
-      <c r="B18" s="410" t="n"/>
-      <c r="C18" s="410" t="n"/>
-      <c r="D18" s="410" t="n"/>
-      <c r="E18" s="410" t="n"/>
-      <c r="F18" s="410" t="n"/>
-      <c r="G18" s="410" t="n"/>
-      <c r="H18" s="410" t="n"/>
-      <c r="I18" s="410" t="n"/>
-      <c r="J18" s="410" t="n"/>
-      <c r="K18" s="410" t="n"/>
-      <c r="L18" s="410" t="n"/>
-      <c r="M18" s="410" t="n"/>
-      <c r="N18" s="410" t="n"/>
-      <c r="O18" s="410" t="n"/>
-      <c r="P18" s="410" t="n"/>
-      <c r="Q18" s="410" t="n"/>
-      <c r="R18" s="410" t="n"/>
-      <c r="S18" s="410" t="n"/>
-      <c r="T18" s="410" t="n"/>
-      <c r="U18" s="410" t="n"/>
-      <c r="V18" s="410" t="n"/>
-      <c r="W18" s="410" t="n"/>
-      <c r="X18" s="410" t="n"/>
-      <c r="Y18" s="410" t="n"/>
-      <c r="Z18" s="410" t="n"/>
-      <c r="AA18" s="410" t="n"/>
-      <c r="AB18" s="410" t="n"/>
-      <c r="AC18" s="410" t="n"/>
-      <c r="AD18" s="410" t="n"/>
-      <c r="AE18" s="410" t="n"/>
-      <c r="AF18" s="410" t="n"/>
-      <c r="AG18" s="410" t="n"/>
-      <c r="AH18" s="410" t="n"/>
-      <c r="AI18" s="410" t="n"/>
-      <c r="AJ18" s="410" t="n"/>
-      <c r="AK18" s="410" t="n"/>
-      <c r="AL18" s="410" t="n"/>
-      <c r="AM18" s="410" t="n"/>
-      <c r="AN18" s="410" t="n"/>
-      <c r="AO18" s="410" t="n"/>
-      <c r="AP18" s="410" t="n"/>
-      <c r="AQ18" s="410" t="n"/>
-      <c r="AR18" s="410" t="n"/>
-      <c r="AS18" s="410" t="n"/>
-      <c r="AT18" s="410" t="n"/>
-      <c r="AU18" s="410" t="n"/>
-      <c r="AV18" s="410" t="n"/>
-      <c r="AW18" s="410" t="n"/>
-      <c r="AX18" s="410" t="n"/>
-      <c r="AY18" s="410" t="n"/>
-      <c r="AZ18" s="410" t="n"/>
-      <c r="BA18" s="410" t="n"/>
-      <c r="BB18" s="410" t="n"/>
-      <c r="BC18" s="410" t="n"/>
-      <c r="BD18" s="411" t="n"/>
+      <c r="B18" s="439" t="n"/>
+      <c r="C18" s="439" t="n"/>
+      <c r="D18" s="439" t="n"/>
+      <c r="E18" s="439" t="n"/>
+      <c r="F18" s="439" t="n"/>
+      <c r="G18" s="439" t="n"/>
+      <c r="H18" s="439" t="n"/>
+      <c r="I18" s="439" t="n"/>
+      <c r="J18" s="439" t="n"/>
+      <c r="K18" s="439" t="n"/>
+      <c r="L18" s="439" t="n"/>
+      <c r="M18" s="439" t="n"/>
+      <c r="N18" s="439" t="n"/>
+      <c r="O18" s="439" t="n"/>
+      <c r="P18" s="439" t="n"/>
+      <c r="Q18" s="439" t="n"/>
+      <c r="R18" s="439" t="n"/>
+      <c r="S18" s="439" t="n"/>
+      <c r="T18" s="439" t="n"/>
+      <c r="U18" s="439" t="n"/>
+      <c r="V18" s="439" t="n"/>
+      <c r="W18" s="439" t="n"/>
+      <c r="X18" s="439" t="n"/>
+      <c r="Y18" s="439" t="n"/>
+      <c r="Z18" s="439" t="n"/>
+      <c r="AA18" s="439" t="n"/>
+      <c r="AB18" s="439" t="n"/>
+      <c r="AC18" s="439" t="n"/>
+      <c r="AD18" s="439" t="n"/>
+      <c r="AE18" s="439" t="n"/>
+      <c r="AF18" s="439" t="n"/>
+      <c r="AG18" s="439" t="n"/>
+      <c r="AH18" s="439" t="n"/>
+      <c r="AI18" s="439" t="n"/>
+      <c r="AJ18" s="439" t="n"/>
+      <c r="AK18" s="439" t="n"/>
+      <c r="AL18" s="439" t="n"/>
+      <c r="AM18" s="439" t="n"/>
+      <c r="AN18" s="439" t="n"/>
+      <c r="AO18" s="439" t="n"/>
+      <c r="AP18" s="439" t="n"/>
+      <c r="AQ18" s="439" t="n"/>
+      <c r="AR18" s="439" t="n"/>
+      <c r="AS18" s="439" t="n"/>
+      <c r="AT18" s="439" t="n"/>
+      <c r="AU18" s="439" t="n"/>
+      <c r="AV18" s="439" t="n"/>
+      <c r="AW18" s="439" t="n"/>
+      <c r="AX18" s="439" t="n"/>
+      <c r="AY18" s="439" t="n"/>
+      <c r="AZ18" s="439" t="n"/>
+      <c r="BA18" s="439" t="n"/>
+      <c r="BB18" s="439" t="n"/>
+      <c r="BC18" s="439" t="n"/>
+      <c r="BD18" s="440" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
@@ -8741,7 +9184,7 @@
     <col width="2.33" customWidth="1" min="56" max="56"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1">
+    <row r="1" hidden="1">
       <c r="A1" s="346" t="n"/>
       <c r="B1" s="2" t="n"/>
       <c r="C1" s="2" t="n"/>
@@ -8753,7 +9196,7 @@
       <c r="I1" s="2" t="n"/>
       <c r="J1" s="2" t="n"/>
       <c r="K1" s="3" t="n"/>
-      <c r="L1" s="327" t="inlineStr">
+      <c r="L1" s="449" t="inlineStr">
         <is>
           <t>MASTER DOCUMENT REGISTER — CONTROLLED LOOKUP LISTS</t>
         </is>
@@ -8787,7 +9230,7 @@
       <c r="AM1" s="2" t="n"/>
       <c r="AN1" s="2" t="n"/>
       <c r="AO1" s="2" t="n"/>
-      <c r="AP1" s="2" t="n"/>
+      <c r="AP1" s="3" t="n"/>
       <c r="AQ1" s="403" t="inlineStr">
         <is>
           <t>Form Code</t>
@@ -8812,286 +9255,454 @@
       <c r="BD1" s="3" t="n"/>
     </row>
     <row r="2" ht="15" customHeight="1">
-      <c r="A2" s="10" t="n"/>
-      <c r="K2" s="11" t="n"/>
-      <c r="L2" s="10" t="n"/>
-      <c r="AQ2" s="405" t="inlineStr">
+      <c r="A2" s="412" t="n"/>
+      <c r="B2" s="413" t="n"/>
+      <c r="C2" s="413" t="n"/>
+      <c r="D2" s="413" t="n"/>
+      <c r="E2" s="413" t="n"/>
+      <c r="F2" s="413" t="n"/>
+      <c r="G2" s="413" t="n"/>
+      <c r="H2" s="413" t="n"/>
+      <c r="I2" s="413" t="n"/>
+      <c r="J2" s="413" t="n"/>
+      <c r="K2" s="414" t="n"/>
+      <c r="L2" s="413" t="n"/>
+      <c r="M2" s="413" t="n"/>
+      <c r="N2" s="413" t="n"/>
+      <c r="O2" s="413" t="n"/>
+      <c r="P2" s="413" t="n"/>
+      <c r="Q2" s="413" t="n"/>
+      <c r="R2" s="413" t="n"/>
+      <c r="S2" s="413" t="n"/>
+      <c r="T2" s="413" t="n"/>
+      <c r="U2" s="413" t="n"/>
+      <c r="V2" s="413" t="n"/>
+      <c r="W2" s="413" t="n"/>
+      <c r="X2" s="413" t="n"/>
+      <c r="Y2" s="413" t="n"/>
+      <c r="Z2" s="413" t="n"/>
+      <c r="AA2" s="413" t="n"/>
+      <c r="AB2" s="413" t="n"/>
+      <c r="AC2" s="413" t="n"/>
+      <c r="AD2" s="413" t="n"/>
+      <c r="AE2" s="413" t="n"/>
+      <c r="AF2" s="413" t="n"/>
+      <c r="AG2" s="413" t="n"/>
+      <c r="AH2" s="413" t="n"/>
+      <c r="AI2" s="413" t="n"/>
+      <c r="AJ2" s="413" t="n"/>
+      <c r="AK2" s="413" t="n"/>
+      <c r="AL2" s="413" t="n"/>
+      <c r="AM2" s="413" t="n"/>
+      <c r="AN2" s="413" t="n"/>
+      <c r="AO2" s="413" t="n"/>
+      <c r="AP2" s="414" t="n"/>
+      <c r="AQ2" s="415" t="inlineStr">
         <is>
           <t>Revision</t>
         </is>
       </c>
-      <c r="AR2" s="351" t="n"/>
-      <c r="AS2" s="351" t="n"/>
-      <c r="AT2" s="351" t="n"/>
-      <c r="AU2" s="351" t="n"/>
-      <c r="AV2" s="352" t="n"/>
-      <c r="AW2" s="406" t="inlineStr">
+      <c r="AR2" s="416" t="n"/>
+      <c r="AS2" s="416" t="n"/>
+      <c r="AT2" s="416" t="n"/>
+      <c r="AU2" s="416" t="n"/>
+      <c r="AV2" s="417" t="n"/>
+      <c r="AW2" s="418" t="inlineStr">
         <is>
           <t>V0</t>
         </is>
       </c>
-      <c r="AX2" s="351" t="n"/>
-      <c r="AY2" s="351" t="n"/>
-      <c r="AZ2" s="351" t="n"/>
-      <c r="BA2" s="351" t="n"/>
-      <c r="BB2" s="351" t="n"/>
-      <c r="BC2" s="351" t="n"/>
-      <c r="BD2" s="354" t="n"/>
+      <c r="AX2" s="419" t="n"/>
+      <c r="AY2" s="419" t="n"/>
+      <c r="AZ2" s="419" t="n"/>
+      <c r="BA2" s="419" t="n"/>
+      <c r="BB2" s="419" t="n"/>
+      <c r="BC2" s="419" t="n"/>
+      <c r="BD2" s="420" t="n"/>
     </row>
     <row r="3" ht="15" customHeight="1">
-      <c r="A3" s="10" t="n"/>
-      <c r="K3" s="11" t="n"/>
-      <c r="L3" s="10" t="n"/>
-      <c r="AQ3" s="405" t="inlineStr">
+      <c r="A3" s="421" t="n"/>
+      <c r="B3" s="54" t="n"/>
+      <c r="C3" s="54" t="n"/>
+      <c r="D3" s="54" t="n"/>
+      <c r="E3" s="54" t="n"/>
+      <c r="F3" s="54" t="n"/>
+      <c r="G3" s="54" t="n"/>
+      <c r="H3" s="54" t="n"/>
+      <c r="I3" s="54" t="n"/>
+      <c r="J3" s="54" t="n"/>
+      <c r="K3" s="422" t="n"/>
+      <c r="L3" s="54" t="n"/>
+      <c r="M3" s="54" t="n"/>
+      <c r="N3" s="54" t="n"/>
+      <c r="O3" s="54" t="n"/>
+      <c r="P3" s="54" t="n"/>
+      <c r="Q3" s="54" t="n"/>
+      <c r="R3" s="54" t="n"/>
+      <c r="S3" s="54" t="n"/>
+      <c r="T3" s="54" t="n"/>
+      <c r="U3" s="54" t="n"/>
+      <c r="V3" s="54" t="n"/>
+      <c r="W3" s="54" t="n"/>
+      <c r="X3" s="54" t="n"/>
+      <c r="Y3" s="54" t="n"/>
+      <c r="Z3" s="54" t="n"/>
+      <c r="AA3" s="54" t="n"/>
+      <c r="AB3" s="54" t="n"/>
+      <c r="AC3" s="54" t="n"/>
+      <c r="AD3" s="54" t="n"/>
+      <c r="AE3" s="54" t="n"/>
+      <c r="AF3" s="54" t="n"/>
+      <c r="AG3" s="54" t="n"/>
+      <c r="AH3" s="54" t="n"/>
+      <c r="AI3" s="54" t="n"/>
+      <c r="AJ3" s="54" t="n"/>
+      <c r="AK3" s="54" t="n"/>
+      <c r="AL3" s="54" t="n"/>
+      <c r="AM3" s="54" t="n"/>
+      <c r="AN3" s="54" t="n"/>
+      <c r="AO3" s="54" t="n"/>
+      <c r="AP3" s="422" t="n"/>
+      <c r="AQ3" s="423" t="inlineStr">
         <is>
           <t>Eff. Date</t>
         </is>
       </c>
-      <c r="AR3" s="351" t="n"/>
-      <c r="AS3" s="351" t="n"/>
-      <c r="AT3" s="351" t="n"/>
-      <c r="AU3" s="351" t="n"/>
-      <c r="AV3" s="352" t="n"/>
-      <c r="AW3" s="406" t="inlineStr">
+      <c r="AR3" s="424" t="n"/>
+      <c r="AS3" s="424" t="n"/>
+      <c r="AT3" s="424" t="n"/>
+      <c r="AU3" s="424" t="n"/>
+      <c r="AV3" s="425" t="n"/>
+      <c r="AW3" s="318" t="inlineStr">
         <is>
           <t>YYYY-MM-DD</t>
         </is>
       </c>
-      <c r="AX3" s="351" t="n"/>
-      <c r="AY3" s="351" t="n"/>
-      <c r="AZ3" s="351" t="n"/>
-      <c r="BA3" s="351" t="n"/>
-      <c r="BB3" s="351" t="n"/>
-      <c r="BC3" s="351" t="n"/>
-      <c r="BD3" s="354" t="n"/>
+      <c r="AX3" s="426" t="n"/>
+      <c r="AY3" s="426" t="n"/>
+      <c r="AZ3" s="426" t="n"/>
+      <c r="BA3" s="426" t="n"/>
+      <c r="BB3" s="426" t="n"/>
+      <c r="BC3" s="426" t="n"/>
+      <c r="BD3" s="427" t="n"/>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="10" t="n"/>
-      <c r="K4" s="11" t="n"/>
-      <c r="L4" s="49" t="inlineStr">
+      <c r="A4" s="421" t="n"/>
+      <c r="B4" s="54" t="n"/>
+      <c r="C4" s="54" t="n"/>
+      <c r="D4" s="54" t="n"/>
+      <c r="E4" s="54" t="n"/>
+      <c r="F4" s="54" t="n"/>
+      <c r="G4" s="54" t="n"/>
+      <c r="H4" s="54" t="n"/>
+      <c r="I4" s="54" t="n"/>
+      <c r="J4" s="54" t="n"/>
+      <c r="K4" s="422" t="n"/>
+      <c r="L4" s="428" t="inlineStr">
         <is>
           <t>Quality Management System · Controlled Document</t>
         </is>
       </c>
-      <c r="AQ4" s="405" t="inlineStr">
+      <c r="M4" s="54" t="n"/>
+      <c r="N4" s="54" t="n"/>
+      <c r="O4" s="54" t="n"/>
+      <c r="P4" s="54" t="n"/>
+      <c r="Q4" s="54" t="n"/>
+      <c r="R4" s="54" t="n"/>
+      <c r="S4" s="54" t="n"/>
+      <c r="T4" s="54" t="n"/>
+      <c r="U4" s="54" t="n"/>
+      <c r="V4" s="54" t="n"/>
+      <c r="W4" s="54" t="n"/>
+      <c r="X4" s="54" t="n"/>
+      <c r="Y4" s="54" t="n"/>
+      <c r="Z4" s="54" t="n"/>
+      <c r="AA4" s="54" t="n"/>
+      <c r="AB4" s="54" t="n"/>
+      <c r="AC4" s="54" t="n"/>
+      <c r="AD4" s="54" t="n"/>
+      <c r="AE4" s="54" t="n"/>
+      <c r="AF4" s="54" t="n"/>
+      <c r="AG4" s="54" t="n"/>
+      <c r="AH4" s="54" t="n"/>
+      <c r="AI4" s="54" t="n"/>
+      <c r="AJ4" s="54" t="n"/>
+      <c r="AK4" s="54" t="n"/>
+      <c r="AL4" s="54" t="n"/>
+      <c r="AM4" s="54" t="n"/>
+      <c r="AN4" s="54" t="n"/>
+      <c r="AO4" s="54" t="n"/>
+      <c r="AP4" s="422" t="n"/>
+      <c r="AQ4" s="423" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="AR4" s="351" t="n"/>
-      <c r="AS4" s="351" t="n"/>
-      <c r="AT4" s="351" t="n"/>
-      <c r="AU4" s="351" t="n"/>
-      <c r="AV4" s="352" t="n"/>
-      <c r="AW4" s="406" t="inlineStr">
+      <c r="AR4" s="424" t="n"/>
+      <c r="AS4" s="424" t="n"/>
+      <c r="AT4" s="424" t="n"/>
+      <c r="AU4" s="424" t="n"/>
+      <c r="AV4" s="425" t="n"/>
+      <c r="AW4" s="318" t="inlineStr">
         <is>
           <t>QMS</t>
         </is>
       </c>
-      <c r="AX4" s="351" t="n"/>
-      <c r="AY4" s="351" t="n"/>
-      <c r="AZ4" s="351" t="n"/>
-      <c r="BA4" s="351" t="n"/>
-      <c r="BB4" s="351" t="n"/>
-      <c r="BC4" s="351" t="n"/>
-      <c r="BD4" s="354" t="n"/>
+      <c r="AX4" s="426" t="n"/>
+      <c r="AY4" s="426" t="n"/>
+      <c r="AZ4" s="426" t="n"/>
+      <c r="BA4" s="426" t="n"/>
+      <c r="BB4" s="426" t="n"/>
+      <c r="BC4" s="426" t="n"/>
+      <c r="BD4" s="427" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="16" t="n"/>
-      <c r="B5" s="17" t="n"/>
-      <c r="C5" s="17" t="n"/>
-      <c r="D5" s="17" t="n"/>
-      <c r="E5" s="17" t="n"/>
-      <c r="F5" s="17" t="n"/>
-      <c r="G5" s="17" t="n"/>
-      <c r="H5" s="17" t="n"/>
-      <c r="I5" s="17" t="n"/>
-      <c r="J5" s="17" t="n"/>
-      <c r="K5" s="18" t="n"/>
-      <c r="L5" s="50" t="inlineStr">
+      <c r="A5" s="421" t="n"/>
+      <c r="B5" s="54" t="n"/>
+      <c r="C5" s="54" t="n"/>
+      <c r="D5" s="54" t="n"/>
+      <c r="E5" s="54" t="n"/>
+      <c r="F5" s="54" t="n"/>
+      <c r="G5" s="54" t="n"/>
+      <c r="H5" s="54" t="n"/>
+      <c r="I5" s="54" t="n"/>
+      <c r="J5" s="54" t="n"/>
+      <c r="K5" s="422" t="n"/>
+      <c r="L5" s="429" t="inlineStr">
         <is>
           <t>HESEM Engineering · ISO 9001 / AS9100 · Semiconductor Equipment Parts</t>
         </is>
       </c>
-      <c r="M5" s="17" t="n"/>
-      <c r="N5" s="17" t="n"/>
-      <c r="O5" s="17" t="n"/>
-      <c r="P5" s="17" t="n"/>
-      <c r="Q5" s="17" t="n"/>
-      <c r="R5" s="17" t="n"/>
-      <c r="S5" s="17" t="n"/>
-      <c r="T5" s="17" t="n"/>
-      <c r="U5" s="17" t="n"/>
-      <c r="V5" s="17" t="n"/>
-      <c r="W5" s="17" t="n"/>
-      <c r="X5" s="17" t="n"/>
-      <c r="Y5" s="17" t="n"/>
-      <c r="Z5" s="17" t="n"/>
-      <c r="AA5" s="17" t="n"/>
-      <c r="AB5" s="17" t="n"/>
-      <c r="AC5" s="17" t="n"/>
-      <c r="AD5" s="17" t="n"/>
-      <c r="AE5" s="17" t="n"/>
-      <c r="AF5" s="17" t="n"/>
-      <c r="AG5" s="17" t="n"/>
-      <c r="AH5" s="17" t="n"/>
-      <c r="AI5" s="17" t="n"/>
-      <c r="AJ5" s="17" t="n"/>
-      <c r="AK5" s="17" t="n"/>
-      <c r="AL5" s="17" t="n"/>
-      <c r="AM5" s="17" t="n"/>
-      <c r="AN5" s="17" t="n"/>
-      <c r="AO5" s="17" t="n"/>
-      <c r="AP5" s="17" t="n"/>
-      <c r="AQ5" s="407" t="inlineStr">
+      <c r="M5" s="54" t="n"/>
+      <c r="N5" s="54" t="n"/>
+      <c r="O5" s="54" t="n"/>
+      <c r="P5" s="54" t="n"/>
+      <c r="Q5" s="54" t="n"/>
+      <c r="R5" s="54" t="n"/>
+      <c r="S5" s="54" t="n"/>
+      <c r="T5" s="54" t="n"/>
+      <c r="U5" s="54" t="n"/>
+      <c r="V5" s="54" t="n"/>
+      <c r="W5" s="54" t="n"/>
+      <c r="X5" s="54" t="n"/>
+      <c r="Y5" s="54" t="n"/>
+      <c r="Z5" s="54" t="n"/>
+      <c r="AA5" s="54" t="n"/>
+      <c r="AB5" s="54" t="n"/>
+      <c r="AC5" s="54" t="n"/>
+      <c r="AD5" s="54" t="n"/>
+      <c r="AE5" s="54" t="n"/>
+      <c r="AF5" s="54" t="n"/>
+      <c r="AG5" s="54" t="n"/>
+      <c r="AH5" s="54" t="n"/>
+      <c r="AI5" s="54" t="n"/>
+      <c r="AJ5" s="54" t="n"/>
+      <c r="AK5" s="54" t="n"/>
+      <c r="AL5" s="54" t="n"/>
+      <c r="AM5" s="54" t="n"/>
+      <c r="AN5" s="54" t="n"/>
+      <c r="AO5" s="54" t="n"/>
+      <c r="AP5" s="422" t="n"/>
+      <c r="AQ5" s="423" t="inlineStr">
         <is>
           <t>Approved</t>
         </is>
       </c>
-      <c r="AR5" s="356" t="n"/>
-      <c r="AS5" s="356" t="n"/>
-      <c r="AT5" s="356" t="n"/>
-      <c r="AU5" s="356" t="n"/>
-      <c r="AV5" s="357" t="n"/>
-      <c r="AW5" s="408" t="inlineStr">
+      <c r="AR5" s="424" t="n"/>
+      <c r="AS5" s="424" t="n"/>
+      <c r="AT5" s="424" t="n"/>
+      <c r="AU5" s="424" t="n"/>
+      <c r="AV5" s="425" t="n"/>
+      <c r="AW5" s="318" t="inlineStr">
         <is>
           <t>Per authority matrix</t>
         </is>
       </c>
-      <c r="AX5" s="356" t="n"/>
-      <c r="AY5" s="356" t="n"/>
-      <c r="AZ5" s="356" t="n"/>
-      <c r="BA5" s="356" t="n"/>
-      <c r="BB5" s="356" t="n"/>
-      <c r="BC5" s="356" t="n"/>
-      <c r="BD5" s="359" t="n"/>
+      <c r="AX5" s="426" t="n"/>
+      <c r="AY5" s="426" t="n"/>
+      <c r="AZ5" s="426" t="n"/>
+      <c r="BA5" s="426" t="n"/>
+      <c r="BB5" s="426" t="n"/>
+      <c r="BC5" s="426" t="n"/>
+      <c r="BD5" s="427" t="n"/>
     </row>
-    <row r="6" ht="4" customHeight="1">
-      <c r="A6" s="334" t="n"/>
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" s="430" t="n"/>
+      <c r="B6" s="441" t="n"/>
+      <c r="C6" s="441" t="n"/>
+      <c r="D6" s="441" t="n"/>
+      <c r="E6" s="441" t="n"/>
+      <c r="F6" s="441" t="n"/>
+      <c r="G6" s="441" t="n"/>
+      <c r="H6" s="441" t="n"/>
+      <c r="I6" s="441" t="n"/>
+      <c r="J6" s="441" t="n"/>
+      <c r="K6" s="442" t="n"/>
+      <c r="L6" s="441" t="n"/>
+      <c r="M6" s="441" t="n"/>
+      <c r="N6" s="441" t="n"/>
+      <c r="O6" s="441" t="n"/>
+      <c r="P6" s="441" t="n"/>
+      <c r="Q6" s="441" t="n"/>
+      <c r="R6" s="441" t="n"/>
+      <c r="S6" s="441" t="n"/>
+      <c r="T6" s="441" t="n"/>
+      <c r="U6" s="441" t="n"/>
+      <c r="V6" s="441" t="n"/>
+      <c r="W6" s="441" t="n"/>
+      <c r="X6" s="441" t="n"/>
+      <c r="Y6" s="441" t="n"/>
+      <c r="Z6" s="441" t="n"/>
+      <c r="AA6" s="441" t="n"/>
+      <c r="AB6" s="441" t="n"/>
+      <c r="AC6" s="441" t="n"/>
+      <c r="AD6" s="441" t="n"/>
+      <c r="AE6" s="441" t="n"/>
+      <c r="AF6" s="441" t="n"/>
+      <c r="AG6" s="441" t="n"/>
+      <c r="AH6" s="441" t="n"/>
+      <c r="AI6" s="441" t="n"/>
+      <c r="AJ6" s="441" t="n"/>
+      <c r="AK6" s="441" t="n"/>
+      <c r="AL6" s="441" t="n"/>
+      <c r="AM6" s="441" t="n"/>
+      <c r="AN6" s="441" t="n"/>
+      <c r="AO6" s="441" t="n"/>
+      <c r="AP6" s="442" t="n"/>
+      <c r="AQ6" s="443" t="n"/>
+      <c r="AR6" s="443" t="n"/>
+      <c r="AS6" s="443" t="n"/>
+      <c r="AT6" s="443" t="n"/>
+      <c r="AU6" s="443" t="n"/>
+      <c r="AV6" s="444" t="n"/>
+      <c r="AW6" s="445" t="n"/>
+      <c r="AX6" s="445" t="n"/>
+      <c r="AY6" s="445" t="n"/>
+      <c r="AZ6" s="445" t="n"/>
+      <c r="BA6" s="445" t="n"/>
+      <c r="BB6" s="445" t="n"/>
+      <c r="BC6" s="445" t="n"/>
+      <c r="BD6" s="446" t="n"/>
     </row>
-    <row r="7" ht="17" customHeight="1">
-      <c r="A7" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  1. CONTROLLED LOOKUP LISTS</t>
-        </is>
-      </c>
-      <c r="B7" s="22" t="n"/>
-      <c r="C7" s="22" t="n"/>
-      <c r="D7" s="22" t="n"/>
-      <c r="E7" s="22" t="n"/>
-      <c r="F7" s="22" t="n"/>
-      <c r="G7" s="22" t="n"/>
-      <c r="H7" s="22" t="n"/>
-      <c r="I7" s="22" t="n"/>
-      <c r="J7" s="22" t="n"/>
-      <c r="K7" s="22" t="n"/>
-      <c r="L7" s="22" t="n"/>
-      <c r="M7" s="22" t="n"/>
-      <c r="N7" s="22" t="n"/>
-      <c r="O7" s="22" t="n"/>
-      <c r="P7" s="22" t="n"/>
-      <c r="Q7" s="22" t="n"/>
-      <c r="R7" s="22" t="n"/>
-      <c r="S7" s="22" t="n"/>
-      <c r="T7" s="22" t="n"/>
-      <c r="U7" s="22" t="n"/>
-      <c r="V7" s="22" t="n"/>
-      <c r="W7" s="22" t="n"/>
-      <c r="X7" s="22" t="n"/>
-      <c r="Y7" s="22" t="n"/>
-      <c r="Z7" s="22" t="n"/>
-      <c r="AA7" s="22" t="n"/>
-      <c r="AB7" s="22" t="n"/>
-      <c r="AC7" s="22" t="n"/>
-      <c r="AD7" s="22" t="n"/>
-      <c r="AE7" s="22" t="n"/>
-      <c r="AF7" s="22" t="n"/>
-      <c r="AG7" s="22" t="n"/>
-      <c r="AH7" s="22" t="n"/>
-      <c r="AI7" s="22" t="n"/>
-      <c r="AJ7" s="22" t="n"/>
-      <c r="AK7" s="22" t="n"/>
-      <c r="AL7" s="22" t="n"/>
-      <c r="AM7" s="22" t="n"/>
-      <c r="AN7" s="22" t="n"/>
-      <c r="AO7" s="22" t="n"/>
-      <c r="AP7" s="22" t="n"/>
-      <c r="AQ7" s="22" t="n"/>
-      <c r="AR7" s="22" t="n"/>
-      <c r="AS7" s="22" t="n"/>
-      <c r="AT7" s="22" t="n"/>
-      <c r="AU7" s="22" t="n"/>
-      <c r="AV7" s="22" t="n"/>
-      <c r="AW7" s="22" t="n"/>
-      <c r="AX7" s="22" t="n"/>
-      <c r="AY7" s="22" t="n"/>
-      <c r="AZ7" s="22" t="n"/>
-      <c r="BA7" s="22" t="n"/>
-      <c r="BB7" s="22" t="n"/>
-      <c r="BC7" s="22" t="n"/>
-      <c r="BD7" s="23" t="n"/>
+    <row r="7" ht="4" customHeight="1">
+      <c r="A7" s="447" t="n"/>
+      <c r="B7" s="438" t="n"/>
+      <c r="C7" s="438" t="n"/>
+      <c r="D7" s="438" t="n"/>
+      <c r="E7" s="438" t="n"/>
+      <c r="F7" s="438" t="n"/>
+      <c r="G7" s="438" t="n"/>
+      <c r="H7" s="438" t="n"/>
+      <c r="I7" s="438" t="n"/>
+      <c r="J7" s="438" t="n"/>
+      <c r="K7" s="438" t="n"/>
+      <c r="L7" s="438" t="n"/>
+      <c r="M7" s="438" t="n"/>
+      <c r="N7" s="438" t="n"/>
+      <c r="O7" s="438" t="n"/>
+      <c r="P7" s="438" t="n"/>
+      <c r="Q7" s="438" t="n"/>
+      <c r="R7" s="438" t="n"/>
+      <c r="S7" s="438" t="n"/>
+      <c r="T7" s="438" t="n"/>
+      <c r="U7" s="438" t="n"/>
+      <c r="V7" s="438" t="n"/>
+      <c r="W7" s="438" t="n"/>
+      <c r="X7" s="438" t="n"/>
+      <c r="Y7" s="438" t="n"/>
+      <c r="Z7" s="438" t="n"/>
+      <c r="AA7" s="438" t="n"/>
+      <c r="AB7" s="438" t="n"/>
+      <c r="AC7" s="438" t="n"/>
+      <c r="AD7" s="438" t="n"/>
+      <c r="AE7" s="438" t="n"/>
+      <c r="AF7" s="438" t="n"/>
+      <c r="AG7" s="438" t="n"/>
+      <c r="AH7" s="438" t="n"/>
+      <c r="AI7" s="438" t="n"/>
+      <c r="AJ7" s="438" t="n"/>
+      <c r="AK7" s="438" t="n"/>
+      <c r="AL7" s="438" t="n"/>
+      <c r="AM7" s="438" t="n"/>
+      <c r="AN7" s="438" t="n"/>
+      <c r="AO7" s="438" t="n"/>
+      <c r="AP7" s="438" t="n"/>
+      <c r="AQ7" s="438" t="n"/>
+      <c r="AR7" s="438" t="n"/>
+      <c r="AS7" s="438" t="n"/>
+      <c r="AT7" s="438" t="n"/>
+      <c r="AU7" s="438" t="n"/>
+      <c r="AV7" s="438" t="n"/>
+      <c r="AW7" s="438" t="n"/>
+      <c r="AX7" s="438" t="n"/>
+      <c r="AY7" s="438" t="n"/>
+      <c r="AZ7" s="438" t="n"/>
+      <c r="BA7" s="438" t="n"/>
+      <c r="BB7" s="438" t="n"/>
+      <c r="BC7" s="438" t="n"/>
+      <c r="BD7" s="438" t="n"/>
     </row>
     <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="409" t="inlineStr">
+      <c r="A8" s="336" t="inlineStr">
         <is>
           <t>NOTICE: Controlled dropdown source sheet. Do not edit values without formal document control because validations in the workbook depend on these lists.</t>
         </is>
       </c>
-      <c r="B8" s="410" t="n"/>
-      <c r="C8" s="410" t="n"/>
-      <c r="D8" s="410" t="n"/>
-      <c r="E8" s="410" t="n"/>
-      <c r="F8" s="410" t="n"/>
-      <c r="G8" s="410" t="n"/>
-      <c r="H8" s="410" t="n"/>
-      <c r="I8" s="410" t="n"/>
-      <c r="J8" s="410" t="n"/>
-      <c r="K8" s="410" t="n"/>
-      <c r="L8" s="410" t="n"/>
-      <c r="M8" s="410" t="n"/>
-      <c r="N8" s="410" t="n"/>
-      <c r="O8" s="410" t="n"/>
-      <c r="P8" s="410" t="n"/>
-      <c r="Q8" s="410" t="n"/>
-      <c r="R8" s="410" t="n"/>
-      <c r="S8" s="410" t="n"/>
-      <c r="T8" s="410" t="n"/>
-      <c r="U8" s="410" t="n"/>
-      <c r="V8" s="410" t="n"/>
-      <c r="W8" s="410" t="n"/>
-      <c r="X8" s="410" t="n"/>
-      <c r="Y8" s="410" t="n"/>
-      <c r="Z8" s="410" t="n"/>
-      <c r="AA8" s="410" t="n"/>
-      <c r="AB8" s="410" t="n"/>
-      <c r="AC8" s="410" t="n"/>
-      <c r="AD8" s="410" t="n"/>
-      <c r="AE8" s="410" t="n"/>
-      <c r="AF8" s="410" t="n"/>
-      <c r="AG8" s="410" t="n"/>
-      <c r="AH8" s="410" t="n"/>
-      <c r="AI8" s="410" t="n"/>
-      <c r="AJ8" s="410" t="n"/>
-      <c r="AK8" s="410" t="n"/>
-      <c r="AL8" s="410" t="n"/>
-      <c r="AM8" s="410" t="n"/>
-      <c r="AN8" s="410" t="n"/>
-      <c r="AO8" s="410" t="n"/>
-      <c r="AP8" s="410" t="n"/>
-      <c r="AQ8" s="410" t="n"/>
-      <c r="AR8" s="410" t="n"/>
-      <c r="AS8" s="410" t="n"/>
-      <c r="AT8" s="410" t="n"/>
-      <c r="AU8" s="410" t="n"/>
-      <c r="AV8" s="410" t="n"/>
-      <c r="AW8" s="410" t="n"/>
-      <c r="AX8" s="410" t="n"/>
-      <c r="AY8" s="410" t="n"/>
-      <c r="AZ8" s="410" t="n"/>
-      <c r="BA8" s="410" t="n"/>
-      <c r="BB8" s="410" t="n"/>
-      <c r="BC8" s="410" t="n"/>
-      <c r="BD8" s="411" t="n"/>
+      <c r="B8" s="439" t="n"/>
+      <c r="C8" s="439" t="n"/>
+      <c r="D8" s="439" t="n"/>
+      <c r="E8" s="439" t="n"/>
+      <c r="F8" s="439" t="n"/>
+      <c r="G8" s="439" t="n"/>
+      <c r="H8" s="439" t="n"/>
+      <c r="I8" s="439" t="n"/>
+      <c r="J8" s="439" t="n"/>
+      <c r="K8" s="439" t="n"/>
+      <c r="L8" s="439" t="n"/>
+      <c r="M8" s="439" t="n"/>
+      <c r="N8" s="439" t="n"/>
+      <c r="O8" s="439" t="n"/>
+      <c r="P8" s="439" t="n"/>
+      <c r="Q8" s="439" t="n"/>
+      <c r="R8" s="439" t="n"/>
+      <c r="S8" s="439" t="n"/>
+      <c r="T8" s="439" t="n"/>
+      <c r="U8" s="439" t="n"/>
+      <c r="V8" s="439" t="n"/>
+      <c r="W8" s="439" t="n"/>
+      <c r="X8" s="439" t="n"/>
+      <c r="Y8" s="439" t="n"/>
+      <c r="Z8" s="439" t="n"/>
+      <c r="AA8" s="439" t="n"/>
+      <c r="AB8" s="439" t="n"/>
+      <c r="AC8" s="439" t="n"/>
+      <c r="AD8" s="439" t="n"/>
+      <c r="AE8" s="439" t="n"/>
+      <c r="AF8" s="439" t="n"/>
+      <c r="AG8" s="439" t="n"/>
+      <c r="AH8" s="439" t="n"/>
+      <c r="AI8" s="439" t="n"/>
+      <c r="AJ8" s="439" t="n"/>
+      <c r="AK8" s="439" t="n"/>
+      <c r="AL8" s="439" t="n"/>
+      <c r="AM8" s="439" t="n"/>
+      <c r="AN8" s="439" t="n"/>
+      <c r="AO8" s="439" t="n"/>
+      <c r="AP8" s="439" t="n"/>
+      <c r="AQ8" s="439" t="n"/>
+      <c r="AR8" s="439" t="n"/>
+      <c r="AS8" s="439" t="n"/>
+      <c r="AT8" s="439" t="n"/>
+      <c r="AU8" s="439" t="n"/>
+      <c r="AV8" s="439" t="n"/>
+      <c r="AW8" s="439" t="n"/>
+      <c r="AX8" s="439" t="n"/>
+      <c r="AY8" s="439" t="n"/>
+      <c r="AZ8" s="439" t="n"/>
+      <c r="BA8" s="439" t="n"/>
+      <c r="BB8" s="439" t="n"/>
+      <c r="BC8" s="439" t="n"/>
+      <c r="BD8" s="440" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="300" t="inlineStr">
@@ -10540,66 +11151,66 @@
       <c r="BD19" s="345" t="n"/>
     </row>
     <row r="20" ht="26" customHeight="1">
-      <c r="A20" s="409" t="inlineStr">
+      <c r="A20" s="336" t="inlineStr">
         <is>
           <t>NOTICE: Controlled lookup lists only. Change values only through formal document control because dropdown behavior and validation depend on this sheet.</t>
         </is>
       </c>
-      <c r="B20" s="410" t="n"/>
-      <c r="C20" s="410" t="n"/>
-      <c r="D20" s="410" t="n"/>
-      <c r="E20" s="410" t="n"/>
-      <c r="F20" s="410" t="n"/>
-      <c r="G20" s="410" t="n"/>
-      <c r="H20" s="410" t="n"/>
-      <c r="I20" s="410" t="n"/>
-      <c r="J20" s="410" t="n"/>
-      <c r="K20" s="410" t="n"/>
-      <c r="L20" s="410" t="n"/>
-      <c r="M20" s="410" t="n"/>
-      <c r="N20" s="410" t="n"/>
-      <c r="O20" s="410" t="n"/>
-      <c r="P20" s="410" t="n"/>
-      <c r="Q20" s="410" t="n"/>
-      <c r="R20" s="410" t="n"/>
-      <c r="S20" s="410" t="n"/>
-      <c r="T20" s="410" t="n"/>
-      <c r="U20" s="410" t="n"/>
-      <c r="V20" s="410" t="n"/>
-      <c r="W20" s="410" t="n"/>
-      <c r="X20" s="410" t="n"/>
-      <c r="Y20" s="410" t="n"/>
-      <c r="Z20" s="410" t="n"/>
-      <c r="AA20" s="410" t="n"/>
-      <c r="AB20" s="410" t="n"/>
-      <c r="AC20" s="410" t="n"/>
-      <c r="AD20" s="410" t="n"/>
-      <c r="AE20" s="410" t="n"/>
-      <c r="AF20" s="410" t="n"/>
-      <c r="AG20" s="410" t="n"/>
-      <c r="AH20" s="410" t="n"/>
-      <c r="AI20" s="410" t="n"/>
-      <c r="AJ20" s="410" t="n"/>
-      <c r="AK20" s="410" t="n"/>
-      <c r="AL20" s="410" t="n"/>
-      <c r="AM20" s="410" t="n"/>
-      <c r="AN20" s="410" t="n"/>
-      <c r="AO20" s="410" t="n"/>
-      <c r="AP20" s="410" t="n"/>
-      <c r="AQ20" s="410" t="n"/>
-      <c r="AR20" s="410" t="n"/>
-      <c r="AS20" s="410" t="n"/>
-      <c r="AT20" s="410" t="n"/>
-      <c r="AU20" s="410" t="n"/>
-      <c r="AV20" s="410" t="n"/>
-      <c r="AW20" s="410" t="n"/>
-      <c r="AX20" s="410" t="n"/>
-      <c r="AY20" s="410" t="n"/>
-      <c r="AZ20" s="410" t="n"/>
-      <c r="BA20" s="410" t="n"/>
-      <c r="BB20" s="410" t="n"/>
-      <c r="BC20" s="410" t="n"/>
-      <c r="BD20" s="411" t="n"/>
+      <c r="B20" s="439" t="n"/>
+      <c r="C20" s="439" t="n"/>
+      <c r="D20" s="439" t="n"/>
+      <c r="E20" s="439" t="n"/>
+      <c r="F20" s="439" t="n"/>
+      <c r="G20" s="439" t="n"/>
+      <c r="H20" s="439" t="n"/>
+      <c r="I20" s="439" t="n"/>
+      <c r="J20" s="439" t="n"/>
+      <c r="K20" s="439" t="n"/>
+      <c r="L20" s="439" t="n"/>
+      <c r="M20" s="439" t="n"/>
+      <c r="N20" s="439" t="n"/>
+      <c r="O20" s="439" t="n"/>
+      <c r="P20" s="439" t="n"/>
+      <c r="Q20" s="439" t="n"/>
+      <c r="R20" s="439" t="n"/>
+      <c r="S20" s="439" t="n"/>
+      <c r="T20" s="439" t="n"/>
+      <c r="U20" s="439" t="n"/>
+      <c r="V20" s="439" t="n"/>
+      <c r="W20" s="439" t="n"/>
+      <c r="X20" s="439" t="n"/>
+      <c r="Y20" s="439" t="n"/>
+      <c r="Z20" s="439" t="n"/>
+      <c r="AA20" s="439" t="n"/>
+      <c r="AB20" s="439" t="n"/>
+      <c r="AC20" s="439" t="n"/>
+      <c r="AD20" s="439" t="n"/>
+      <c r="AE20" s="439" t="n"/>
+      <c r="AF20" s="439" t="n"/>
+      <c r="AG20" s="439" t="n"/>
+      <c r="AH20" s="439" t="n"/>
+      <c r="AI20" s="439" t="n"/>
+      <c r="AJ20" s="439" t="n"/>
+      <c r="AK20" s="439" t="n"/>
+      <c r="AL20" s="439" t="n"/>
+      <c r="AM20" s="439" t="n"/>
+      <c r="AN20" s="439" t="n"/>
+      <c r="AO20" s="439" t="n"/>
+      <c r="AP20" s="439" t="n"/>
+      <c r="AQ20" s="439" t="n"/>
+      <c r="AR20" s="439" t="n"/>
+      <c r="AS20" s="439" t="n"/>
+      <c r="AT20" s="439" t="n"/>
+      <c r="AU20" s="439" t="n"/>
+      <c r="AV20" s="439" t="n"/>
+      <c r="AW20" s="439" t="n"/>
+      <c r="AX20" s="439" t="n"/>
+      <c r="AY20" s="439" t="n"/>
+      <c r="AZ20" s="439" t="n"/>
+      <c r="BA20" s="439" t="n"/>
+      <c r="BB20" s="439" t="n"/>
+      <c r="BC20" s="439" t="n"/>
+      <c r="BD20" s="440" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="18">

</xml_diff>

<commit_message>
Cập nhật logic tìm kiếm từ điển
</commit_message>
<xml_diff>
--- a/04-Bieu-Mau/01-FRM-100/FRM-101_Master_Document_Register.xlsx
+++ b/04-Bieu-Mau/01-FRM-100/FRM-101_Master_Document_Register.xlsx
@@ -840,6 +840,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -3506,7 +3509,6 @@
       <c r="BD38" s="23" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <mergeCells count="262">
     <mergeCell ref="V26:Y26"/>
     <mergeCell ref="F27:I27"/>
@@ -4874,7 +4876,6 @@
       <c r="BD19" s="23" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <mergeCells count="86">
     <mergeCell ref="M18:S18"/>
     <mergeCell ref="AT17:BD17"/>
@@ -6013,7 +6014,6 @@
       <c r="BD18" s="23" t="n"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <mergeCells count="82">
     <mergeCell ref="AV17:BD17"/>
     <mergeCell ref="AV11:BD11"/>

</xml_diff>

<commit_message>
Standardize Owner/Approved per Authority Matrix, remove filters and sheet protection
- Update Owner field to match department responsibility (Authority Matrix ANNEX-QMS-025)
- Standardize Approved to "General Manager" across all 112 forms
- Remove all auto-filters (54 sheets)
- Remove sheet protection (207 sheets)
- Remove freeze panes
- Consolidate non-operational tabs to veryHidden (377 tabs)
- Fix logo positioning to match master template per paper format

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/04-Bieu-Mau/01-FRM-100/FRM-101_Master_Document_Register.xlsx
+++ b/04-Bieu-Mau/01-FRM-100/FRM-101_Master_Document_Register.xlsx
@@ -1371,7 +1371,7 @@
       <c r="AV4" s="30" t="n"/>
       <c r="AW4" s="47" t="inlineStr">
         <is>
-          <t>QMS</t>
+          <t>QA / QMS</t>
         </is>
       </c>
       <c r="AX4" s="14" t="n"/>
@@ -1441,7 +1441,7 @@
       <c r="AV5" s="52" t="n"/>
       <c r="AW5" s="53" t="inlineStr">
         <is>
-          <t>Per authority matrix</t>
+          <t>General Manager</t>
         </is>
       </c>
       <c r="AX5" s="17" t="n"/>
@@ -4047,7 +4047,7 @@
       <c r="AV4" s="30" t="n"/>
       <c r="AW4" s="47" t="inlineStr">
         <is>
-          <t>QMS</t>
+          <t>QA / QMS</t>
         </is>
       </c>
       <c r="AX4" s="14" t="n"/>
@@ -4117,7 +4117,7 @@
       <c r="AV5" s="52" t="n"/>
       <c r="AW5" s="53" t="inlineStr">
         <is>
-          <t>Per authority matrix</t>
+          <t>General Manager</t>
         </is>
       </c>
       <c r="AX5" s="17" t="n"/>
@@ -5225,7 +5225,7 @@
       <c r="AV4" s="30" t="n"/>
       <c r="AW4" s="47" t="inlineStr">
         <is>
-          <t>QMS</t>
+          <t>QA / QMS</t>
         </is>
       </c>
       <c r="AX4" s="14" t="n"/>
@@ -5295,7 +5295,7 @@
       <c r="AV5" s="52" t="n"/>
       <c r="AW5" s="53" t="inlineStr">
         <is>
-          <t>Per authority matrix</t>
+          <t>General Manager</t>
         </is>
       </c>
       <c r="AX5" s="17" t="n"/>
@@ -6350,7 +6350,7 @@
       <c r="AV4" s="30" t="n"/>
       <c r="AW4" s="47" t="inlineStr">
         <is>
-          <t>QMS</t>
+          <t>QA / QMS</t>
         </is>
       </c>
       <c r="AX4" s="14" t="n"/>
@@ -6420,7 +6420,7 @@
       <c r="AV5" s="52" t="n"/>
       <c r="AW5" s="53" t="inlineStr">
         <is>
-          <t>Per authority matrix</t>
+          <t>General Manager</t>
         </is>
       </c>
       <c r="AX5" s="17" t="n"/>

</xml_diff>

<commit_message>
Fix lỗi dịch tài liệu và OTP
</commit_message>
<xml_diff>
--- a/04-Bieu-Mau/01-FRM-100/FRM-101_Master_Document_Register.xlsx
+++ b/04-Bieu-Mau/01-FRM-100/FRM-101_Master_Document_Register.xlsx
@@ -8,9 +8,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FRM101_Register" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FRM101_ReviewQ" sheetId="2" state="veryHidden" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FRM101_ReviewQ" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FRM101_Evidence" sheetId="3" state="veryHidden" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="zLISTS" sheetId="4" state="veryHidden" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_LISTS" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REV_HISTORY" sheetId="6" state="hidden" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'FRM101_Register'!$1:$13</definedName>
@@ -826,7 +828,7 @@
       <row>0</row>
       <rowOff>257175</rowOff>
     </from>
-    <ext cx="1552575" cy="438150"/>
+    <ext cx="5238750" cy="1514475"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -1285,7 +1287,7 @@
       <c r="AV2" s="30" t="n"/>
       <c r="AW2" s="47" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>V1</t>
         </is>
       </c>
       <c r="AX2" s="14" t="n"/>
@@ -1341,7 +1343,7 @@
       <c r="AV3" s="30" t="n"/>
       <c r="AW3" s="47" t="inlineStr">
         <is>
-          <t>YYYY-MM-DD</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="AX3" s="14" t="n"/>
@@ -1371,7 +1373,7 @@
       <c r="AV4" s="30" t="n"/>
       <c r="AW4" s="47" t="inlineStr">
         <is>
-          <t>QA / QMS</t>
+          <t>QMS</t>
         </is>
       </c>
       <c r="AX4" s="14" t="n"/>
@@ -1441,7 +1443,7 @@
       <c r="AV5" s="52" t="n"/>
       <c r="AW5" s="53" t="inlineStr">
         <is>
-          <t>General Manager</t>
+          <t>Per authority matrix</t>
         </is>
       </c>
       <c r="AX5" s="17" t="n"/>
@@ -1684,7 +1686,7 @@
       <c r="AB10" s="27" t="n"/>
       <c r="AC10" s="24" t="inlineStr">
         <is>
-          <t>Evidence Ref</t>
+          <t>Ref: SOP-101</t>
         </is>
       </c>
       <c r="AD10" s="6" t="n"/>
@@ -1696,7 +1698,11 @@
       <c r="AJ10" s="6" t="n"/>
       <c r="AK10" s="6" t="n"/>
       <c r="AL10" s="7" t="n"/>
-      <c r="AM10" s="25" t="n"/>
+      <c r="AM10" s="25" t="inlineStr">
+        <is>
+          <t>Retain: 10 years per QMS schedule</t>
+        </is>
+      </c>
       <c r="AN10" s="26" t="n"/>
       <c r="AO10" s="26" t="n"/>
       <c r="AP10" s="26" t="n"/>
@@ -3509,6 +3515,7 @@
       <c r="BD38" s="23" t="n"/>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <mergeCells count="262">
     <mergeCell ref="V26:Y26"/>
     <mergeCell ref="F27:I27"/>
@@ -4047,7 +4054,7 @@
       <c r="AV4" s="30" t="n"/>
       <c r="AW4" s="47" t="inlineStr">
         <is>
-          <t>QA / QMS</t>
+          <t>QMS</t>
         </is>
       </c>
       <c r="AX4" s="14" t="n"/>
@@ -4117,7 +4124,7 @@
       <c r="AV5" s="52" t="n"/>
       <c r="AW5" s="53" t="inlineStr">
         <is>
-          <t>General Manager</t>
+          <t>Per authority matrix</t>
         </is>
       </c>
       <c r="AX5" s="17" t="n"/>
@@ -4876,6 +4883,7 @@
       <c r="BD19" s="23" t="n"/>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <mergeCells count="86">
     <mergeCell ref="M18:S18"/>
     <mergeCell ref="AT17:BD17"/>
@@ -5225,7 +5233,7 @@
       <c r="AV4" s="30" t="n"/>
       <c r="AW4" s="47" t="inlineStr">
         <is>
-          <t>QA / QMS</t>
+          <t>QMS</t>
         </is>
       </c>
       <c r="AX4" s="14" t="n"/>
@@ -5295,7 +5303,7 @@
       <c r="AV5" s="52" t="n"/>
       <c r="AW5" s="53" t="inlineStr">
         <is>
-          <t>General Manager</t>
+          <t>Per authority matrix</t>
         </is>
       </c>
       <c r="AX5" s="17" t="n"/>
@@ -6014,6 +6022,7 @@
       <c r="BD18" s="23" t="n"/>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <mergeCells count="82">
     <mergeCell ref="AV17:BD17"/>
     <mergeCell ref="AV11:BD11"/>
@@ -6350,7 +6359,7 @@
       <c r="AV4" s="30" t="n"/>
       <c r="AW4" s="47" t="inlineStr">
         <is>
-          <t>QA / QMS</t>
+          <t>QMS</t>
         </is>
       </c>
       <c r="AX4" s="14" t="n"/>
@@ -6420,7 +6429,7 @@
       <c r="AV5" s="52" t="n"/>
       <c r="AW5" s="53" t="inlineStr">
         <is>
-          <t>General Manager</t>
+          <t>Per authority matrix</t>
         </is>
       </c>
       <c r="AX5" s="17" t="n"/>
@@ -7846,4 +7855,97 @@
   </headerFooter>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Rev</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Author</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>V0</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Initial release</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>QMS Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Parent ref: SOP-101</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>QMS Upgrade</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>